<commit_message>
Integrate VP1 machine and record material-flow HOLD
</commit_message>
<xml_diff>
--- a/c2.1/bom/system_bom.xlsx
+++ b/c2.1/bom/system_bom.xlsx
@@ -4179,12 +4179,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>DRV-SH15R</t>
+          <t>DRV-SH40R</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>KHK SH2-15RH reference</t>
+          <t>KHK SH2-40RH reference</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -4236,12 +4236,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>DRV-SH40L</t>
+          <t>DRV-SP12-B12</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>KHK SH2-40LH reference</t>
+          <t>ANSI35 12T sprocket bore12</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -4251,17 +4251,17 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>S45C hardened</t>
+          <t>Steel</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>COTS_REFERENCE_SECONDARY_BORE_HOLD</t>
+          <t>CHAIN_TOOTH_PROFILE_AND_LOAD_HOLD</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>https://khkgears.net/pdf/sh.pdf</t>
+          <t>Supplier drawing / capacity confirmation required before procurement</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
@@ -4281,7 +4281,7 @@
       </c>
       <c r="K75" t="inlineStr">
         <is>
-          <t>Purchased hardened teeth. 25 face + 10 hub. Do not machine teeth from this OD model. 40T bore modified 18 to20. Opposite-hand mating specified; lower-half key is mirrored before axial flip.</t>
+          <t>9.525 pitch. Roller pocket reference only; exact manufacturer tooth form, width and working load must replace this model.</t>
         </is>
       </c>
     </row>
@@ -4293,12 +4293,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>DRV-SH40R</t>
+          <t>DRV-SP24-B20</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>KHK SH2-40RH reference</t>
+          <t>ANSI35 24T sprocket bore20</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -4308,17 +4308,17 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>S45C hardened</t>
+          <t>Steel</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>COTS_REFERENCE_SECONDARY_BORE_HOLD</t>
+          <t>CHAIN_TOOTH_PROFILE_AND_LOAD_HOLD</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>https://khkgears.net/pdf/sh.pdf</t>
+          <t>Supplier drawing / capacity confirmation required before procurement</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
@@ -4338,7 +4338,7 @@
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>Purchased hardened teeth. 25 face + 10 hub. Do not machine teeth from this OD model. 40T bore modified 18 to20. Opposite-hand mating specified; lower-half key is mirrored before axial flip.</t>
+          <t>9.525 pitch. Roller pocket reference only; exact manufacturer tooth form, width and working load must replace this model.</t>
         </is>
       </c>
     </row>
@@ -4350,12 +4350,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>DRV-SP12-B12</t>
+          <t>DRV-SP24-B25</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>ANSI35 12T sprocket bore12</t>
+          <t>ANSI35 24T sprocket bore25</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -4407,12 +4407,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>DRV-SP24-B12</t>
+          <t>KEY-4-70</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>ANSI35 24T sprocket bore12</t>
+          <t>Parallel key4x4x70</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -4422,17 +4422,17 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Steel</t>
+          <t>C45 ground key stock</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>CHAIN_TOOTH_PROFILE_AND_LOAD_HOLD</t>
+          <t>CUSTOM_DFM_HOLD</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Supplier drawing / capacity confirmation required before procurement</t>
+          <t>PPR-C1 original dimensional design; not an empirical qualification</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
@@ -4452,7 +4452,7 @@
       </c>
       <c r="K78" t="inlineStr">
         <is>
-          <t>9.525 pitch. Roller pocket reference only; exact manufacturer tooth form, width and working load must replace this model.</t>
+          <t>Nominal key blank; stock/female-key fit and deburring to drawing review. No printed keys.</t>
         </is>
       </c>
     </row>
@@ -4464,32 +4464,32 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>DRV-SP24-B20</t>
+          <t>KEY-6-16</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>ANSI35 24T sprocket bore20</t>
+          <t>Parallel key6x6x16</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Steel</t>
+          <t>C45 ground key stock</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>CHAIN_TOOTH_PROFILE_AND_LOAD_HOLD</t>
+          <t>CUSTOM_DFM_HOLD</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Supplier drawing / capacity confirmation required before procurement</t>
+          <t>PPR-C1 original dimensional design; not an empirical qualification</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -4504,12 +4504,12 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>REQUOTE_AFTER_QUANTITY_CHANGE</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>9.525 pitch. Roller pocket reference only; exact manufacturer tooth form, width and working load must replace this model.</t>
+          <t>Nominal key blank; stock/female-key fit and deburring to drawing review. No printed keys. VP1 second jackshaft key cut to 14.8 mm before y388 bearing; fit/strength HOLD.</t>
         </is>
       </c>
     </row>
@@ -4521,12 +4521,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>DRV-SP24-B25</t>
+          <t>KEY-6-70</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>ANSI35 24T sprocket bore25</t>
+          <t>Parallel key6x6x70</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -4536,17 +4536,17 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Steel</t>
+          <t>C45 ground key stock</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>CHAIN_TOOTH_PROFILE_AND_LOAD_HOLD</t>
+          <t>CUSTOM_DFM_HOLD</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Supplier drawing / capacity confirmation required before procurement</t>
+          <t>PPR-C1 original dimensional design; not an empirical qualification</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -4566,34 +4566,34 @@
       </c>
       <c r="K80" t="inlineStr">
         <is>
-          <t>9.525 pitch. Roller pocket reference only; exact manufacturer tooth form, width and working load must replace this model.</t>
+          <t>Nominal key blank; stock/female-key fit and deburring to drawing review. No printed keys.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>legacy_interface:drive</t>
+          <t>legacy_interface:drive+frame_mount</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>KEY-4-16</t>
+          <t>DRV-M1-PL</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Parallel key4x4x16</t>
+          <t>TT60 common motor face plate</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>C45 ground key stock</t>
+          <t>S355 steel</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -4618,29 +4618,29 @@
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>REQUOTE_AFTER_QUANTITY_CHANGE</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>Nominal key blank; stock/female-key fit and deburring to drawing review. No printed keys.</t>
+          <t>Motor axis datum(35,32.5); 4x5.5 THRU onPCD45. Confirm motor engagement depth.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>legacy_interface:drive</t>
+          <t>legacy_interface:electrical</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>KEY-4-70</t>
+          <t>EL-PSU</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Parallel key4x4x70</t>
+          <t>Owned 24V 800W PSU</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -4650,17 +4650,17 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>C45 ground key stock</t>
+          <t>Purchased</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>CUSTOM_DFM_HOLD</t>
+          <t>OWNED_MOUNTING_PATTERN_UNMEASURED</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>PPR-C1 original dimensional design; not an empirical qualification</t>
+          <t>PPR_project_handover_2026-09-20.zip / 08_BOM_COMPONENTS.md</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -4670,34 +4670,34 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t/>
+          <t>0</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>OWNED_NO_NEW_PURCHASE</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
         <is>
-          <t>Nominal key blank; stock/female-key fit and deburring to drawing review. No printed keys.</t>
+          <t>No guessed mounting holes. 120x240x65 user measurement; model contains true body only.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>legacy_interface:drive</t>
+          <t>legacy_interface:extruder</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>KEY-6-16</t>
+          <t>BR-51102</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Parallel key6x6x16</t>
+          <t>51102 bearing boundary</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -4707,17 +4707,17 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>C45 ground key stock</t>
+          <t>Bearing steel</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>CUSTOM_DFM_HOLD</t>
+          <t>DATASHEET_BOUNDARY</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>PPR-C1 original dimensional design; not an empirical qualification</t>
+          <t>https://www.nsk.com/engineering/51102-apn.html</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
@@ -4737,24 +4737,24 @@
       </c>
       <c r="K83" t="inlineStr">
         <is>
-          <t>Nominal key blank; stock/female-key fit and deburring to drawing review. No printed keys.</t>
+          <t>Seal, clearance class and exact suffix must be selected. Bearing envelope is not solid steel in mass estimates.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>legacy_interface:drive</t>
+          <t>legacy_interface:extruder</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>KEY-6-70</t>
+          <t>BR-6202</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Parallel key6x6x70</t>
+          <t>6202 bearing boundary</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -4764,17 +4764,17 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>C45 ground key stock</t>
+          <t>Bearing steel</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>CUSTOM_DFM_HOLD</t>
+          <t>STANDARD_SIZE_VERIFY_MPN</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>PPR-C1 original dimensional design; not an empirical qualification</t>
+          <t>Supplier drawing / capacity confirmation required before procurement</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -4794,44 +4794,44 @@
       </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t>Nominal key blank; stock/female-key fit and deburring to drawing review. No printed keys.</t>
+          <t>Seal, clearance class and exact suffix must be selected. Bearing envelope is not solid steel in mass estimates.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>legacy_interface:drive+frame_mount</t>
+          <t>legacy_interface:extruder</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>DRV-M1-PL</t>
+          <t>DRV-M2</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>TT60 common motor face plate</t>
+          <t>M2 TT GMP60 motor reference</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>S355 steel</t>
+          <t>Purchased</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>CUSTOM_DFM_HOLD</t>
+          <t>DATASHEET_INTERFACE_REFERENCE</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>PPR-C1 original dimensional design; not an empirical qualification</t>
+          <t>https://www.ttmotor.com/uploads/GMP60-609760127.pdf</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
@@ -4851,24 +4851,24 @@
       </c>
       <c r="K85" t="inlineStr">
         <is>
-          <t>Motor axis datum(35,32.5); 4x5.5 THRU onPCD45. Confirm motor engagement depth.</t>
+          <t>4xM5 PCD45, pilot32, shaft12 D10.9; encoder and wire exit not dimensioned in this option.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>legacy_interface:electrical</t>
+          <t>legacy_interface:extruder</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>EL-PSU</t>
+          <t>EX-BARREL</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Owned 24V 800W PSU</t>
+          <t>Barrel16.3ID x30OD x256</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -4878,17 +4878,17 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Purchased</t>
+          <t>SCM440 nitrided RFQ</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>OWNED_MOUNTING_PATTERN_UNMEASURED</t>
+          <t>CUSTOM_DFM_HOLD</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>PPR_project_handover_2026-09-20.zip / 08_BOM_COMPONENTS.md</t>
+          <t>PPR-C1 original dimensional design; not an empirical qualification</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -4898,17 +4898,17 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>0</t>
+          <t/>
         </is>
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>OWNED_NO_NEW_PURCHASE</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t>No guessed mounting holes. 120x240x65 user measurement; model contains true body only.</t>
+          <t>Radial cold clearance0.15. Honing, straightness, hot fit, feed hole and die pressure sealing require supplier approval.</t>
         </is>
       </c>
     </row>
@@ -4920,12 +4920,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>BR-51102</t>
+          <t>EX-CPL</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>51102 bearing boundary</t>
+          <t>12-to15 split coupling32 long</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -4935,17 +4935,17 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Bearing steel</t>
+          <t>Steel</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>DATASHEET_BOUNDARY</t>
+          <t>CLAMP_TORQUE_HOLD</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>https://www.nsk.com/engineering/51102-apn.html</t>
+          <t>PPR-C1 original dimensional design; not an empirical qualification</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
@@ -4965,7 +4965,7 @@
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>Seal, clearance class and exact suffix must be selected. Bearing envelope is not solid steel in mass estimates.</t>
+          <t>D-shaft jaw and clamping proof pending, no axial load transfer intent.</t>
         </is>
       </c>
     </row>
@@ -4977,12 +4977,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>BR-6202</t>
+          <t>EX-DIE</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>6202 bearing boundary</t>
+          <t>Die36OD x20 with2mm exit</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -4992,17 +4992,17 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Bearing steel</t>
+          <t>SCM440 or stainless RFQ</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>STANDARD_SIZE_VERIFY_MPN</t>
+          <t>CUSTOM_DFM_HOLD</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>Supplier drawing / capacity confirmation required before procurement</t>
+          <t>PPR-C1 original dimensional design; not an empirical qualification</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
@@ -5022,7 +5022,7 @@
       </c>
       <c r="K88" t="inlineStr">
         <is>
-          <t>Seal, clearance class and exact suffix must be selected. Bearing envelope is not solid steel in mass estimates.</t>
+          <t>2mm die exit is a drawdown candidate for1.75 filament, not final calibration. Heater bore6x38; pressure attachment not yet detailed.</t>
         </is>
       </c>
     </row>
@@ -5034,32 +5034,32 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>DRV-M2</t>
+          <t>EX-H100</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>M2 TT GMP60 motor reference</t>
+          <t>24V100W band heater30ID x40</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Purchased</t>
+          <t>Purchased custom</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>DATASHEET_INTERFACE_REFERENCE</t>
+          <t>HEATER_QUOTE_AND_DRAWING_HOLD</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>https://www.ttmotor.com/uploads/GMP60-609760127.pdf</t>
+          <t>Supplier drawing / capacity confirmation required before procurement</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
@@ -5079,7 +5079,7 @@
       </c>
       <c r="K89" t="inlineStr">
         <is>
-          <t>4xM5 PCD45, pilot32, shaft12 D10.9; encoder and wire exit not dimensioned in this option.</t>
+          <t>3units100W; power density100/(pi*3cm*4cm)=2.65W/cm2. Lead/clamp bulge not invented.</t>
         </is>
       </c>
     </row>
@@ -5091,12 +5091,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>EX-BARREL</t>
+          <t>EX-H60</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Barrel16.3ID x30OD x256</t>
+          <t>24V60W cartridge6x20</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -5106,17 +5106,17 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>SCM440 nitrided RFQ</t>
+          <t>Purchased custom</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>CUSTOM_DFM_HOLD</t>
+          <t>HEATER_QUOTE_AND_DRAWING_HOLD</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>PPR-C1 original dimensional design; not an empirical qualification</t>
+          <t>Supplier drawing / capacity confirmation required before procurement</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
@@ -5136,7 +5136,7 @@
       </c>
       <c r="K90" t="inlineStr">
         <is>
-          <t>Radial cold clearance0.15. Honing, straightness, hot fit, feed hole and die pressure sealing require supplier approval.</t>
+          <t>Rated60W is requirement, not a verified off-the-shelf product.</t>
         </is>
       </c>
     </row>
@@ -5148,12 +5148,12 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>EX-CPL</t>
+          <t>EX-REAR</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>12-to15 split coupling32 long</t>
+          <t>Extruder rear/thrust shaft15</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -5163,12 +5163,12 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Steel</t>
+          <t>SCM440</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>CLAMP_TORQUE_HOLD</t>
+          <t>CUSTOM_DFM_HOLD</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
@@ -5193,7 +5193,7 @@
       </c>
       <c r="K91" t="inlineStr">
         <is>
-          <t>D-shaft jaw and clamping proof pending, no axial load transfer intent.</t>
+          <t>x213..274 inassembly; collar258..264. No thrust transmitted to M2 bearings; shaft-screw connection detail is manufacturing HOLD.</t>
         </is>
       </c>
     </row>
@@ -5205,12 +5205,12 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>EX-DIE</t>
+          <t>EX-SCREW</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Die36OD x20 with2mm exit</t>
+          <t>16mm x256mm compression screw</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -5220,7 +5220,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>SCM440 or stainless RFQ</t>
+          <t>SCM440 QT/nitriding RFQ</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -5250,7 +5250,7 @@
       </c>
       <c r="K92" t="inlineStr">
         <is>
-          <t>2mm die exit is a drawdown candidate for1.75 filament, not final calibration. Heater bore6x38; pressure attachment not yet detailed.</t>
+          <t>Pitch16, flight2, root10 feed /13 meter, L/D16. CAD flight has square flanks; fillets/tip geometry/finish and nitriding supplier confirmation required.</t>
         </is>
       </c>
     </row>
@@ -5262,32 +5262,32 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>EX-H100</t>
+          <t>EX-THRUST</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>24V100W band heater30ID x40</t>
+          <t>Metal thrust carrier39x60x70</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Purchased custom</t>
+          <t>C45</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>HEATER_QUOTE_AND_DRAWING_HOLD</t>
+          <t>CUSTOM_DFM_HOLD</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>Supplier drawing / capacity confirmation required before procurement</t>
+          <t>PPR-C1 original dimensional design; not an empirical qualification</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
@@ -5307,24 +5307,24 @@
       </c>
       <c r="K93" t="inlineStr">
         <is>
-          <t>3units100W; power density100/(pi*3cm*4cm)=2.65W/cm2. Lead/clamp bulge not invented.</t>
+          <t>6202 and51102 distinct radial/thrust functions. Split lid, positive stops and end access need assembly DFM; digital solid only. Four M6 underside pilots atX10/26,Y10/50; mating stand positions232/248,255/295.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>legacy_interface:extruder</t>
+          <t>legacy_interface:feed</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>EX-H60</t>
+          <t>FEED-BUF</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>24V60W cartridge6x20</t>
+          <t>Buffer190x48 top /50x40 throat /height73</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -5334,17 +5334,17 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Purchased custom</t>
+          <t>PC outer shell plus metal throat</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>HEATER_QUOTE_AND_DRAWING_HOLD</t>
+          <t>CUSTOM_DFM_HOLD</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>Supplier drawing / capacity confirmation required before procurement</t>
+          <t>PPR-C1 original dimensional design; not an empirical qualification</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
@@ -5364,24 +5364,24 @@
       </c>
       <c r="K94" t="inlineStr">
         <is>
-          <t>Rated60W is requirement, not a verified off-the-shelf product.</t>
+          <t>Internal geometric volume calculated; usable75pct separately stated. Top fits between Y251..299, ahead of pin rings. Cold throat offset to barrel feed X289.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>legacy_interface:extruder</t>
+          <t>legacy_interface:feed</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>EX-REAR</t>
+          <t>HOP-LID</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Extruder rear/thrust shaft15</t>
+          <t>Interlocked lid180x140</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -5391,7 +5391,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>SCM440</t>
+          <t>PC with metal strike</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -5421,24 +5421,24 @@
       </c>
       <c r="K95" t="inlineStr">
         <is>
-          <t>x213..274 inassembly; collar258..264. No thrust transmitted to M2 bearings; shaft-screw connection detail is manufacturing HOLD.</t>
+          <t>Hinge/guard lock hardware not chosen. NO open-lid operation.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>legacy_interface:extruder</t>
+          <t>legacy_interface:feed</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>EX-SCREW</t>
+          <t>HOPPER</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>16mm x256mm compression screw</t>
+          <t>35deg batch hopper</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>SCM440 QT/nitriding RFQ</t>
+          <t>PC shell + steel lower liner</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -5478,24 +5478,24 @@
       </c>
       <c r="K96" t="inlineStr">
         <is>
-          <t>Pitch16, flight2, root10 feed /13 meter, L/D16. CAD flight has square flanks; fillets/tip geometry/finish and nitriding supplier confirmation required.</t>
+          <t>Whole hopper exceeds print limit; must split into &lt;=210mm panels before printing. Closed lid and standstill interlock mandatory; angle is not an access safety measure.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>legacy_interface:extruder</t>
+          <t>legacy_interface:frame</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>EX-THRUST</t>
+          <t>FR-2020-320</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Metal thrust carrier39x60x70</t>
+          <t>2020 profile cut320</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -5505,17 +5505,17 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>C45</t>
+          <t>Al extrusion - existing</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>CUSTOM_DFM_HOLD</t>
+          <t>OWNED_SLOT_PATTERN_TO_MEASURE</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>PPR-C1 original dimensional design; not an empirical qualification</t>
+          <t>PPR_project_handover_2026-09-20.zip / 08_BOM_COMPONENTS.md</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
@@ -5525,54 +5525,54 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t/>
+          <t>0</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>OWNED_NO_NEW_PURCHASE</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
         <is>
-          <t>6202 and51102 distinct radial/thrust functions. Split lid, positive stops and end access need assembly DFM; digital solid only. Four M6 underside pilots atX10/26,Y10/50; mating stand positions232/248,255/295.</t>
+          <t>Nominal section only. Confirm slot series before buying brackets; 3 mm saw kerf.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>legacy_interface:feed</t>
+          <t>legacy_interface:frame</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>FEED-BUF</t>
+          <t>FR-2020-360</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Buffer190x48 top /50x40 throat /height73</t>
+          <t>2020 profile cut 360</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>PC outer shell plus metal throat</t>
+          <t>Al extrusion - existing</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>CUSTOM_DFM_HOLD</t>
+          <t>OWNED_SLOT_PATTERN_TO_MEASURE</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>PPR-C1 original dimensional design; not an empirical qualification</t>
+          <t>PPR_project_handover_2026-09-20.zip / 08_BOM_COMPONENTS.md</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
@@ -5582,54 +5582,54 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t/>
+          <t>0</t>
         </is>
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>OWNED_NO_NEW_PURCHASE</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
         <is>
-          <t>Internal geometric volume calculated; usable75pct separately stated. Top fits between Y251..299, ahead of pin rings. Cold throat offset to barrel feed X289.</t>
+          <t>Nominal section only. Confirm slot series before buying brackets; 3 mm saw kerf.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>legacy_interface:feed</t>
+          <t>legacy_interface:frame</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>HOP-LID</t>
+          <t>FR-2020-400</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Interlocked lid180x140</t>
+          <t>2020 profile cut 400</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>PC with metal strike</t>
+          <t>Al extrusion - existing</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>CUSTOM_DFM_HOLD</t>
+          <t>OWNED_SLOT_PATTERN_TO_MEASURE</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>PPR-C1 original dimensional design; not an empirical qualification</t>
+          <t>PPR_project_handover_2026-09-20.zip / 08_BOM_COMPONENTS.md</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
@@ -5639,54 +5639,54 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t/>
+          <t>0</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>OWNED_NO_NEW_PURCHASE</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
         <is>
-          <t>Hinge/guard lock hardware not chosen. NO open-lid operation.</t>
+          <t>Nominal section only. Confirm slot series before buying brackets; 3 mm saw kerf.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>legacy_interface:feed</t>
+          <t>legacy_interface:frame</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>HOPPER</t>
+          <t>FR-2020-590</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>35deg batch hopper</t>
+          <t>2020 profile cut 590</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>PC shell + steel lower liner</t>
+          <t>Al extrusion - existing</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>CUSTOM_DFM_HOLD</t>
+          <t>OWNED_SLOT_PATTERN_TO_MEASURE</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>PPR-C1 original dimensional design; not an empirical qualification</t>
+          <t>PPR_project_handover_2026-09-20.zip / 08_BOM_COMPONENTS.md</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
@@ -5696,17 +5696,17 @@
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t/>
+          <t>0</t>
         </is>
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>OWNED_NO_NEW_PURCHASE</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
         <is>
-          <t>Whole hopper exceeds print limit; must split into &lt;=210mm panels before printing. Closed lid and standstill interlock mandatory; angle is not an access safety measure.</t>
+          <t>Nominal section only. Confirm slot series before buying brackets; 3 mm saw kerf.</t>
         </is>
       </c>
     </row>
@@ -5718,17 +5718,17 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>FR-2020-320</t>
+          <t>FR-2040-320</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>2020 profile cut320</t>
+          <t>2040 profile cut 320</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -5775,17 +5775,17 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>FR-2020-360</t>
+          <t>FR-2040-400</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>2020 profile cut 360</t>
+          <t>2040 profile cut 400</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
@@ -5832,12 +5832,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>FR-2020-400</t>
+          <t>FR-2040-630</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>2020 profile cut 400</t>
+          <t>2040 profile cut 630</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -5889,32 +5889,32 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>FR-2020-590</t>
+          <t>FR-BASE</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>2020 profile cut 590</t>
+          <t>Bottom tray 630x400x3</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Al extrusion - existing</t>
+          <t>Al 5052</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>OWNED_SLOT_PATTERN_TO_MEASURE</t>
+          <t>SHEET_DFM_HOLD</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>PPR_project_handover_2026-09-20.zip / 08_BOM_COMPONENTS.md</t>
+          <t>PPR-C1 original dimensional design; not an empirical qualification</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
@@ -5924,54 +5924,54 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>0</t>
+          <t/>
         </is>
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>OWNED_NO_NEW_PURCHASE</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
         <is>
-          <t>Nominal section only. Confirm slot series before buying brackets; 3 mm saw kerf.</t>
+          <t>Mains and hot zones require separate partitions; shown base is not sealed containment.</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>legacy_interface:frame</t>
+          <t>legacy_interface:frame_mount</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>FR-2040-320</t>
+          <t>DRV-DECK</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>2040 profile cut 320</t>
+          <t>Steel drive deck240x194x5</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Al extrusion - existing</t>
+          <t>S355 steel</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>OWNED_SLOT_PATTERN_TO_MEASURE</t>
+          <t>CUSTOM_DFM_HOLD</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>PPR_project_handover_2026-09-20.zip / 08_BOM_COMPONENTS.md</t>
+          <t>PPR-C1 original dimensional design; not an empirical qualification</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
@@ -5981,54 +5981,54 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>0</t>
+          <t/>
         </is>
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>OWNED_NO_NEW_PURCHASE</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
         <is>
-          <t>Nominal section only. Confirm slot series before buying brackets; 3 mm saw kerf.</t>
+          <t>Deck atZ20..25, supported by existing crossmembers. Added4 feet must be included in frame stiffness review.</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>legacy_interface:frame</t>
+          <t>legacy_interface:frame_mount</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>FR-2040-400</t>
+          <t>DRV-M1-FOOT</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>2040 profile cut 400</t>
+          <t>M1 steel mounting foot70x50x19</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Al extrusion - existing</t>
+          <t>Steel</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>OWNED_SLOT_PATTERN_TO_MEASURE</t>
+          <t>CUSTOM_DFM_HOLD</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>PPR_project_handover_2026-09-20.zip / 08_BOM_COMPONENTS.md</t>
+          <t>PPR-C1 original dimensional design; not an empirical qualification</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
@@ -6038,54 +6038,54 @@
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>0</t>
+          <t/>
         </is>
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>OWNED_NO_NEW_PURCHASE</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
         <is>
-          <t>Nominal section only. Confirm slot series before buying brackets; 3 mm saw kerf.</t>
+          <t>Motor plate corner holes to vertical face. Base bolts to drive deck, not to a printed carrier.</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>legacy_interface:frame</t>
+          <t>legacy_interface:frame_mount</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>FR-2040-630</t>
+          <t>DRV-RISER12</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>2040 profile cut 630</t>
+          <t>Input rear bearing riser34x12x10</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Al extrusion - existing</t>
+          <t>Steel</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>OWNED_SLOT_PATTERN_TO_MEASURE</t>
+          <t>CUSTOM_DFM_HOLD</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>PPR_project_handover_2026-09-20.zip / 08_BOM_COMPONENTS.md</t>
+          <t>PPR-C1 original dimensional design; not an empirical qualification</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
@@ -6095,34 +6095,34 @@
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>0</t>
+          <t/>
         </is>
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>OWNED_NO_NEW_PURCHASE</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
         <is>
-          <t>Nominal section only. Confirm slot series before buying brackets; 3 mm saw kerf.</t>
+          <t>Bearing bolt pattern must be transferred to deck after slots/profile series confirmed.</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>legacy_interface:frame</t>
+          <t>legacy_interface:frame_mount</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>FR-BASE</t>
+          <t>DRV-RISER20</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Bottom tray 630x400x3</t>
+          <t>Output rear bearing shim70x18x2.5</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -6132,12 +6132,12 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Al 5052</t>
+          <t>Steel</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>SHEET_DFM_HOLD</t>
+          <t>CUSTOM_DFM_HOLD</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
@@ -6162,7 +6162,7 @@
       </c>
       <c r="K108" t="inlineStr">
         <is>
-          <t>Mains and hot zones require separate partitions; shown base is not sealed containment.</t>
+          <t>2.50 ground shim, full metal bearing support.</t>
         </is>
       </c>
     </row>
@@ -6174,12 +6174,12 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>DRV-DECK</t>
+          <t>EX-STAND</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Steel drive deck240x194x5</t>
+          <t>Thrust stand / coaxial motor bridge</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -6189,7 +6189,7 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>S355 steel</t>
+          <t>Steel</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
@@ -6219,7 +6219,7 @@
       </c>
       <c r="K109" t="inlineStr">
         <is>
-          <t>Deck atZ20..25, supported by existing crossmembers. Added4 feet must be included in frame stiffness review.</t>
+          <t>M2 and thrust carrier share metal stand on deck; no large right-angle gearbox. Top holes4xM6 to carrier. Weld/bolt/pressure proof remains HOLD.</t>
         </is>
       </c>
     </row>
@@ -6231,22 +6231,22 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>DRV-M1-FOOT</t>
+          <t>S1-ROOF-F</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>M1 steel mounting foot70x50x19</t>
+          <t>Front roof bracket30x95x25</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Steel</t>
+          <t>10mm steel welded/folded</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
@@ -6276,7 +6276,7 @@
       </c>
       <c r="K110" t="inlineStr">
         <is>
-          <t>Motor plate corner holes to vertical face. Base bolts to drive deck, not to a printed carrier.</t>
+          <t>Face atY135 against retainer. M6 top hole to existing profile centreY50. Metal roof load path; bend/weld qualification pending.</t>
         </is>
       </c>
     </row>
@@ -6288,22 +6288,22 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>DRV-RISER12</t>
+          <t>S1-ROOF-R</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Input rear bearing riser34x12x10</t>
+          <t>Rear roof bracket30x48x25</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Steel</t>
+          <t>10mm steel welded/folded</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
@@ -6333,7 +6333,7 @@
       </c>
       <c r="K111" t="inlineStr">
         <is>
-          <t>Bearing bolt pattern must be transferred to deck after slots/profile series confirmed.</t>
+          <t>Face atY352; M6 profile connection atY390. Do not print this bracket.</t>
         </is>
       </c>
     </row>
@@ -6345,17 +6345,17 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>DRV-RISER20</t>
+          <t>S2-LEG-L</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Output rear bearing shim70x18x2.5</t>
+          <t>S2 L column / metal foot</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -6390,7 +6390,7 @@
       </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t>2.50 ground shim, full metal bearing support.</t>
+          <t>Foot bottomZ25; topZ210. Centre mounting holeZ203. L sits on5mm deck, R on2020crossmember. Welded joint and anchors DFM hold.</t>
         </is>
       </c>
     </row>
@@ -6402,17 +6402,17 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>EX-STAND</t>
+          <t>S2-LEG-R</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Thrust stand / coaxial motor bridge</t>
+          <t>S2 R column / metal foot</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -6447,44 +6447,44 @@
       </c>
       <c r="K113" t="inlineStr">
         <is>
-          <t>M2 and thrust carrier share metal stand on deck; no large right-angle gearbox. Top holes4xM6 to carrier. Weld/bolt/pressure proof remains HOLD.</t>
+          <t>Foot bottomZ20; topZ210. Centre mounting holeZ203. L sits on5mm deck, R on2020crossmember. Welded joint and anchors DFM hold.</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>legacy_interface:frame_mount</t>
+          <t>system_requirement</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>S1-ROOF-F</t>
+          <t>AUX-DRIVES</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Front roof bracket30x95x25</t>
+          <t>Puller,spool,traverse actuation</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>10mm steel welded/folded</t>
+          <t>Procurement requirement</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>CUSTOM_DFM_HOLD</t>
+          <t>AUX_ACTUATION_HOLD</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>PPR-C1 original dimensional design; not an empirical qualification</t>
+          <t>Supplier drawing / capacity confirmation required before procurement</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
@@ -6504,44 +6504,44 @@
       </c>
       <c r="K114" t="inlineStr">
         <is>
-          <t>Face atY135 against retainer. M6 top hole to existing profile centreY50. Metal roof load path; bend/weld qualification pending.</t>
+          <t>Separate low-power controls, no large third shredder motor.</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>legacy_interface:frame_mount</t>
+          <t>system_requirement</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>S1-ROOF-R</t>
+          <t>CHAIN-A</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Rear roof bracket30x48x25</t>
+          <t>ANSI35 chain94 pitches</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>10mm steel welded/folded</t>
+          <t>Procurement requirement</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>CUSTOM_DFM_HOLD</t>
+          <t>CHAIN_RATING_HOLD</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>PPR-C1 original dimensional design; not an empirical qualification</t>
+          <t>Supplier drawing / capacity confirmation required before procurement</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
@@ -6561,44 +6561,44 @@
       </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t>Face atY352; M6 profile connection atY390. Do not print this bracket.</t>
+          <t>Pitch length895.35mm. Working load and width to confirm.</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>legacy_interface:frame_mount</t>
+          <t>system_requirement</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>S2-LEG-L</t>
+          <t>CHAIN-B</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>S2 L column / metal foot</t>
+          <t>ANSI35 chain84 pitches</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Steel</t>
+          <t>Procurement requirement</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>CUSTOM_DFM_HOLD</t>
+          <t>CHAIN_RATING_HOLD</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>PPR-C1 original dimensional design; not an empirical qualification</t>
+          <t>Supplier drawing / capacity confirmation required before procurement</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
@@ -6618,44 +6618,44 @@
       </c>
       <c r="K116" t="inlineStr">
         <is>
-          <t>Foot bottomZ25; topZ210. Centre mounting holeZ203. L sits on5mm deck, R on2020crossmember. Welded joint and anchors DFM hold.</t>
+          <t>Pitch length800.10mm. Working load and width to confirm.</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>legacy_interface:frame_mount</t>
+          <t>system_requirement</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>S2-LEG-R</t>
+          <t>CTRL-MEGA</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>S2 R column / metal foot</t>
+          <t>Arduino Mega</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Steel</t>
+          <t>Procurement requirement</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>CUSTOM_DFM_HOLD</t>
+          <t>OWNED</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>PPR-C1 original dimensional design; not an empirical qualification</t>
+          <t>PPR_project_handover_2026-09-20.zip / 08_BOM_COMPONENTS.md</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
@@ -6665,17 +6665,17 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t/>
+          <t>0</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>OWNED_NO_NEW_PURCHASE</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>Foot bottomZ20; topZ210. Centre mounting holeZ203. L sits on5mm deck, R on2020crossmember. Welded joint and anchors DFM hold.</t>
+          <t>Reference power allocator is NOT deployable heater firmware.</t>
         </is>
       </c>
     </row>
@@ -6687,12 +6687,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>AUX-DRIVES</t>
+          <t>DRV-TLIMIT</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Puller,spool,traverse actuation</t>
+          <t>Mechanical torque limiter</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -6707,7 +6707,7 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>AUX_ACTUATION_HOLD</t>
+          <t>TORQUE_LIMITER_HOLD</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
@@ -6732,7 +6732,7 @@
       </c>
       <c r="K118" t="inlineStr">
         <is>
-          <t>Separate low-power controls, no large third shredder motor.</t>
+          <t>Shared M1 input; calibration before blade operation.</t>
         </is>
       </c>
     </row>
@@ -6744,17 +6744,17 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>CHAIN-A</t>
+          <t>EL-BTS</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>ANSI35 chain94 pitches</t>
+          <t>Existing BTS7960 modules</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -6764,12 +6764,12 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>CHAIN_RATING_HOLD</t>
+          <t>OWNED_UNQUALIFIED</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>Supplier drawing / capacity confirmation required before procurement</t>
+          <t>PPR_project_handover_2026-09-20.zip / 08_BOM_COMPONENTS.md</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
@@ -6779,17 +6779,17 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t/>
+          <t>0</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>OWNED_NO_NEW_PURCHASE</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
         <is>
-          <t>Pitch length895.35mm. Working load and width to confirm.</t>
+          <t>Do not assume advertised43A continuous.</t>
         </is>
       </c>
     </row>
@@ -6801,12 +6801,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>CHAIN-B</t>
+          <t>EL-DRV</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>ANSI35 chain84 pitches</t>
+          <t>Pololu2995 M1 driver option</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -6821,12 +6821,12 @@
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>CHAIN_RATING_HOLD</t>
+          <t>OPTION_NOT_PURCHASED</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>Supplier drawing / capacity confirmation required before procurement</t>
+          <t>https://www.pololu.com/product/2995</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
@@ -6846,7 +6846,7 @@
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>Pitch length800.10mm. Working load and width to confirm.</t>
+          <t>Configurable current limit; board21A is not terminal43A. Existing BTS7960 requires qualification.</t>
         </is>
       </c>
     </row>
@@ -6858,17 +6858,17 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>CTRL-MEGA</t>
+          <t>EL-TC</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Arduino Mega</t>
+          <t>Adafruit3263 MAX31856</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -6878,12 +6878,12 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>OWNED</t>
+          <t>PURCHASE_CANDIDATE</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>PPR_project_handover_2026-09-20.zip / 08_BOM_COMPONENTS.md</t>
+          <t>https://www.adafruit.com/product/3263</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
@@ -6893,17 +6893,17 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>0</t>
+          <t/>
         </is>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>OWNED_NO_NEW_PURCHASE</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>Reference power allocator is NOT deployable heater firmware.</t>
+          <t>Four independent temperature inputs; K probes exact mechanical model unresolved.</t>
         </is>
       </c>
     </row>
@@ -6915,12 +6915,12 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>DRV-TLIMIT</t>
+          <t>FASTENERS</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Mechanical torque limiter</t>
+          <t>Brackets, metal supports,keys,shims,retainers</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -6935,7 +6935,7 @@
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>TORQUE_LIMITER_HOLD</t>
+          <t>HARDWARE_SCHEDULE_HOLD</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
@@ -6960,7 +6960,7 @@
       </c>
       <c r="K122" t="inlineStr">
         <is>
-          <t>Shared M1 input; calibration before blade operation.</t>
+          <t>Not an orderable quantity list; full mechanical fastener closure is outstanding.</t>
         </is>
       </c>
     </row>
@@ -6972,17 +6972,17 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>EL-BTS</t>
+          <t>FEED-CHUTE</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Existing BTS7960 modules</t>
+          <t>Metal lined transfer chute</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -6992,12 +6992,12 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>OWNED_UNQUALIFIED</t>
+          <t>TRANSFER_PATH_HOLD</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>PPR_project_handover_2026-09-20.zip / 08_BOM_COMPONENTS.md</t>
+          <t>PPR-C1 original dimensional design; not an empirical qualification</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
@@ -7007,17 +7007,17 @@
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>0</t>
+          <t/>
         </is>
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>OWNED_NO_NEW_PURCHASE</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="K123" t="inlineStr">
         <is>
-          <t>Do not assume advertised43A continuous.</t>
+          <t>Complete swept envelope/bridging check and split-print panels before release.</t>
         </is>
       </c>
     </row>
@@ -7029,12 +7029,12 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>EL-DRV</t>
+          <t>GUARDS</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Pololu2995 M1 driver option</t>
+          <t>Steel cutter containment / chain guards / heat shield</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -7049,12 +7049,12 @@
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>OPTION_NOT_PURCHASED</t>
+          <t>SAFETY_GEOMETRY_HOLD</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>https://www.pololu.com/product/2995</t>
+          <t>PPR-C1 original dimensional design; not an empirical qualification</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
@@ -7074,7 +7074,7 @@
       </c>
       <c r="K124" t="inlineStr">
         <is>
-          <t>Configurable current limit; board21A is not terminal43A. Existing BTS7960 requires qualification.</t>
+          <t>Do not operate the open review assembly. Guard geometry still to be detailed.</t>
         </is>
       </c>
     </row>
@@ -7086,17 +7086,17 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>EL-TC</t>
+          <t>SAFE-BRAKE</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Adafruit3263 MAX31856</t>
+          <t>Bus overvoltage/braking protection</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
@@ -7106,12 +7106,12 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>PURCHASE_CANDIDATE</t>
+          <t>REGEN_DESIGN_HOLD</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>https://www.adafruit.com/product/3263</t>
+          <t>Supplier drawing / capacity confirmation required before procurement</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
@@ -7131,7 +7131,7 @@
       </c>
       <c r="K125" t="inlineStr">
         <is>
-          <t>Four independent temperature inputs; K probes exact mechanical model unresolved.</t>
+          <t>PSU sink ability unknown; no regeneration assumption.</t>
         </is>
       </c>
     </row>
@@ -7143,12 +7143,12 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>FASTENERS</t>
+          <t>SAFE-CONTACT</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Brackets, metal supports,keys,shims,retainers</t>
+          <t>24V coil DC rated contactor</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -7163,7 +7163,7 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>HARDWARE_SCHEDULE_HOLD</t>
+          <t>SAFETY_SELECTION_HOLD</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
@@ -7188,7 +7188,7 @@
       </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>Not an orderable quantity list; full mechanical fastener closure is outstanding.</t>
+          <t>Continuous&gt;=35A DC and fault-current breaking coordinated with fuse.</t>
         </is>
       </c>
     </row>
@@ -7200,12 +7200,12 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>FEED-CHUTE</t>
+          <t>SAFE-FUSE</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Metal lined transfer chute</t>
+          <t>Branch and mains fuses / holders</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -7220,12 +7220,12 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>TRANSFER_PATH_HOLD</t>
+          <t>CIRCUIT_DESIGN_HOLD</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>PPR-C1 original dimensional design; not an empirical qualification</t>
+          <t>Supplier drawing / capacity confirmation required before procurement</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
@@ -7245,7 +7245,7 @@
       </c>
       <c r="K127" t="inlineStr">
         <is>
-          <t>Complete swept envelope/bridging check and split-print panels before release.</t>
+          <t>Select from actual cable ampacity, DC breaking and inrush. No guessed fuse order.</t>
         </is>
       </c>
     </row>
@@ -7257,17 +7257,17 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>GUARDS</t>
+          <t>SAFE-LOCK</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Steel cutter containment / chain guards / heat shield</t>
+          <t>Coded/positive-opening guard lock</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
@@ -7277,12 +7277,12 @@
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>SAFETY_GEOMETRY_HOLD</t>
+          <t>SAFETY_SELECTION_HOLD</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>PPR-C1 original dimensional design; not an empirical qualification</t>
+          <t>Supplier drawing / capacity confirmation required before procurement</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
@@ -7302,7 +7302,7 @@
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t>Do not operate the open review assembly. Guard geometry still to be detailed.</t>
+          <t>Lid and service access, standstill unlock, manual reset.</t>
         </is>
       </c>
     </row>
@@ -7314,12 +7314,12 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>SAFE-BRAKE</t>
+          <t>SAFE-STOP</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Bus overvoltage/braking protection</t>
+          <t>Existing E-stop</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -7334,12 +7334,12 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>REGEN_DESIGN_HOLD</t>
+          <t>OWNED_RATING_VERIFY</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>Supplier drawing / capacity confirmation required before procurement</t>
+          <t>PPR_project_handover_2026-09-20.zip / 08_BOM_COMPONENTS.md</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
@@ -7349,17 +7349,17 @@
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t/>
+          <t>0</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>OWNED_NO_NEW_PURCHASE</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
         <is>
-          <t>PSU sink ability unknown; no regeneration assumption.</t>
+          <t>Independent hard cut with contactor; contact configuration verify.</t>
         </is>
       </c>
     </row>
@@ -7371,12 +7371,12 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>SAFE-CONTACT</t>
+          <t>SAFE-THERM</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>24V coil DC rated contactor</t>
+          <t>Independent thermal cutoff chain</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -7416,24 +7416,24 @@
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>Continuous&gt;=35A DC and fault-current breaking coordinated with fuse.</t>
+          <t>Normally closed manual-reset overtemp plus one-shot protection.</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>system_requirement</t>
+          <t>vp1_stage1_3</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>SAFE-FUSE</t>
+          <t>AUG_BEARINGS</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Branch and mains fuses / holders</t>
+          <t>west split pillow plus east journal cradle for the r3 auger shaft</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -7443,22 +7443,22 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Procurement requirement</t>
+          <t>steel plate 5 mm</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>CIRCUIT_DESIGN_HOLD</t>
+          <t>TRANSFER_UNRATED</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>Supplier drawing / capacity confirmation required before procurement</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>C1_INTERFACE_BASELINE</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -7468,54 +7468,54 @@
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>UNQUOTED_NOT_ZERO</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>Select from actual cable ampacity, DC breaking and inrush. No guessed fuse order.</t>
+          <t>Auger shaft supported at both ends - UNQUOTED</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>system_requirement</t>
+          <t>vp1_stage1_3</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>SAFE-LOCK</t>
+          <t>AUG_SHAFT</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Coded/positive-opening guard lock</t>
+          <t>active auger conveyor: r3 shaft x236..370 at y232/z347.1; RH flight root r3/OD r8, pitch 28.5, four turns x238.5..352.5 with 3 mm swept face; 0.032 mm BRep U-shell gap</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Procurement requirement</t>
+          <t>steel shaft + steel flight</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>SAFETY_SELECTION_HOLD</t>
+          <t>TRANSFER_UNRATED</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>Supplier drawing / capacity confirmation required before procurement</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>C1_INTERFACE_BASELINE</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -7525,29 +7525,29 @@
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>UNQUOTED_NOT_ZERO</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>Lid and service access, standstill unlock, manual reset.</t>
+          <t>Conveys +x at -5.4375 rpm for 58 rpm reference M1 via 15/40 gear and 24/12 chain B plus 8:1 worm/wheel; S1 pan pickup and S2 handoff need connected validation - UNQUOTED</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>system_requirement</t>
+          <t>vp1_stage1_3</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>SAFE-STOP</t>
+          <t>AUG_WHEEL</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Existing E-stop</t>
+          <t>16T worm wheel (REFERENCE geometry, unrated), face x359..365, sector web, teeth cut by discrete hobbing of the worm; keyed Ø6 auger bore</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -7557,54 +7557,54 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Procurement requirement</t>
+          <t>steel (reference)</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>OWNED_RATING_VERIFY</t>
+          <t>REFERENCE_UNRATED</t>
         </is>
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>PPR_project_handover_2026-09-20.zip / 08_BOM_COMPONENTS.md</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>C1_INTERFACE_BASELINE</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>0</t>
+          <t/>
         </is>
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>OWNED_NO_NEW_PURCHASE</t>
+          <t>UNQUOTED_NOT_ZERO</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
         <is>
-          <t>Independent hard cut with contactor; contact configuration verify.</t>
+          <t>Matched 1.8 mm key and keyway transfer torque to AUG_SHAFT; tooth strength and wear unqualified - UNQUOTED</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>system_requirement</t>
+          <t>vp1_stage1_3</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>SAFE-THERM</t>
+          <t>CHUTE_BODY</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Independent thermal cutoff chain</t>
+          <t>welded S1-&gt;S2 transfer chute with sealed pan, active screw-conveyor trough and east fallaway</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -7614,22 +7614,22 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Procurement requirement</t>
+          <t>steel sheet 3 mm + formed trough</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>SAFETY_SELECTION_HOLD</t>
+          <t>TRANSFER_UNRATED</t>
         </is>
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>Supplier drawing / capacity confirmation required before procurement</t>
+          <t>VP1-ADR-002</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>C1_INTERFACE_BASELINE</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -7639,12 +7639,12 @@
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>UNQUOTED_NOT_ZERO</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
         <is>
-          <t>Normally closed manual-reset overtemp plus one-shot protection.</t>
+          <t>BRep geometry and digital flow only; material transport and containment are not physically qualified - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -7656,12 +7656,12 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>CHUTE_BODY</t>
+          <t>CHUTE_TROUGH_FLOOR_E</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>welded S1-&gt;S2 transfer chute (pan + 45deg intake lip + sealed walls + fin-bypass channel)</t>
+          <t>bolted trough ledge section over the S2 mouth</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -7671,12 +7671,12 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>steel sheet 3 mm + 45deg lips</t>
+          <t>steel sheet 3 mm</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>GEOMETRY_PASS_SLOPE_DEFECT_DOCUMENTED</t>
+          <t>GEOMETRY_PASS</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
@@ -7701,7 +7701,7 @@
       </c>
       <c r="K135" t="inlineStr">
         <is>
-          <t>BREP collision-audited; trough floor slope ~1 deg (batch accumulation transport) - UNQUOTED</t>
+          <t>Clearance-cut for the frozen saddle jacket - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -7713,12 +7713,12 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>CHUTE_TROUGH_FLOOR_E</t>
+          <t>CROSS_FEED_BEARINGS</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>bolted trough ledge section over the S2 mouth</t>
+          <t>paired cross-feed and idler journal support with structural rails</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -7728,22 +7728,22 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>steel sheet 3 mm</t>
+          <t>steel plate and journal shells</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>GEOMETRY_PASS</t>
+          <t>TRANSFER_UNRATED</t>
         </is>
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>VP1-ADR-002</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -7758,7 +7758,7 @@
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>Clearance-cut for the frozen saddle jacket - UNQUOTED</t>
+          <t>BRep-supported reference geometry; wear and load unqualified - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -7770,12 +7770,12 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>DRV-CHAIN-A</t>
+          <t>CROSS_FEED_GEAR</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>#35 roller chain cut to 896 mm (94 links; chain A: jackshaft 24T -&gt; S1 shaft A 24T)</t>
+          <t>12T keyed output gear on transverse feed shaft</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -7785,22 +7785,22 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>ANSI35 steel roller chain p=9.525</t>
+          <t>steel reference gear</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>PROCUREMENT_HOLD</t>
+          <t>TRANSFER_UNRATED</t>
         </is>
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>VP1-ADR-002</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>VP1-STAGE1</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -7815,7 +7815,7 @@
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>Cut length from tangent+pitch-arc geometry (drive_geometry.json chain_lengths.A=896.0). UNQUOTED: not 0 - the 100000 KRW soft limit applies to quoted lines only</t>
+          <t>1:1 from PDL through idler; tooth contact and torque rating unqualified - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -7827,12 +7827,12 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>DRV-CHAIN-B</t>
+          <t>CROSS_FEED_IDLER</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>#35 roller chain cut to 801 mm (84 links; chain B: input shaft 24T -&gt; S2 12T)</t>
+          <t>12T integral idler and supported journal between PDL and transverse feed gears</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -7842,22 +7842,22 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>ANSI35 steel roller chain p=9.525</t>
+          <t>steel reference gear and shaft</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>PROCUREMENT_HOLD</t>
+          <t>TRANSFER_UNRATED</t>
         </is>
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>VP1-ADR-002</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>VP1-STAGE1</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -7872,7 +7872,7 @@
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>Cut length from tangent+pitch-arc geometry (chain_lengths.B=801.07). UNQUOTED: not 0</t>
+          <t>Two external meshes preserve rotation sign; journal rating unqualified - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -7884,12 +7884,12 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>EL_CONTACTOR</t>
+          <t>CROSS_FEED_SHAFT</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>safety contactor</t>
+          <t>LH helical screw on y-axis x357/z328 with 9 mm pitch and radius 10 mm flight</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -7899,22 +7899,22 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>24 V coil contactor MPN unselected</t>
+          <t>steel shaft and welded flight</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>SAFETY_HARDWARE_REQUIRED</t>
+          <t>TRANSFER_UNRATED</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -7929,7 +7929,7 @@
       </c>
       <c r="K139" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>Active +Y transfer to y250.7; frozen south cap y251..255 remains and final material passage unproven - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -7941,12 +7941,12 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>EL_CURRENT_LIMITER</t>
+          <t>CROSS_FEED_SHELL</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>heater sequencer / current-limit relay bank</t>
+          <t>U cradle and cap-bore inner-radius 5 mm passive outlet bridge</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -7956,22 +7956,22 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>relay bank MPN unselected</t>
+          <t>formed steel sheet</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>CONTROL_UNIMPLEMENTED_IN_FIRMWARE</t>
+          <t>TRANSFER_UNRATED</t>
         </is>
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -7986,7 +7986,7 @@
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>Staged heater control hardware: firmware logic UNIMPLEMENTED; interlock required so a firmware fault cannot energize two bands - UNQUOTED</t>
+          <t>Shell does not cut frozen S2 cap; material crossing cap bridge unproven - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -7998,12 +7998,12 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>EL_DIN_RAIL</t>
+          <t>DRV-CHAIN-A</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>DIN rail 35 mm top-hat x 210</t>
+          <t>#35 roller chain cut to 896 mm (94 links; chain A: jackshaft 24T -&gt; S1 shaft A 24T)</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -8013,7 +8013,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>steel rail</t>
+          <t>ANSI35 steel roller chain p=9.525</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
@@ -8023,12 +8023,12 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-ADR-002</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-STAGE1</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -8043,7 +8043,7 @@
       </c>
       <c r="K141" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>Cut length from tangent+pitch-arc geometry (drive_geometry.json chain_lengths.A=896.0). UNQUOTED: not 0 - the 100000 KRW soft limit applies to quoted lines only</t>
         </is>
       </c>
     </row>
@@ -8055,12 +8055,12 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>EL_DRIVER_1</t>
+          <t>DRV-CHAIN-B</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>stepper/BLDC driver (M1 branch)</t>
+          <t>#35 roller chain cut to 724 mm (76 links; chain B: jackshaft 24T -&gt; S2 12T, ADR-002 rev B)</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -8070,22 +8070,22 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>24 V driver MPN unselected</t>
+          <t>ANSI35 steel roller chain p=9.525</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>MOTOR_UNSELECTED</t>
+          <t>PROCUREMENT_HOLD</t>
         </is>
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-ADR-002</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-STAGE4</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -8100,7 +8100,7 @@
       </c>
       <c r="K142" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>Cut length from tangent+pitch-arc geometry (chain_lengths.B=723.9). UNQUOTED: not 0</t>
         </is>
       </c>
     </row>
@@ -8112,12 +8112,12 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>EL_DRIVER_2</t>
+          <t>EL_CONTACTOR</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>stepper/BLDC driver (M2 branch)</t>
+          <t>safety contactor</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -8127,12 +8127,12 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>24 V driver MPN unselected</t>
+          <t>24 V coil contactor MPN unselected</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>MOTOR_UNSELECTED</t>
+          <t>SAFETY_HARDWARE_REQUIRED</t>
         </is>
       </c>
       <c r="G143" t="inlineStr">
@@ -8169,12 +8169,12 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>EL_DRIVER_3</t>
+          <t>EL_CURRENT_LIMITER</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>stepper/BLDC driver (winder/puller accessory)</t>
+          <t>heater sequencer / current-limit relay bank</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -8184,22 +8184,22 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>24 V driver MPN unselected</t>
+          <t>relay bank MPN unselected</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>MOTOR_UNSELECTED</t>
+          <t>CONTROL_REFERENCE_UNRATED</t>
         </is>
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-STAGE4</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-STAGE4</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -8214,7 +8214,7 @@
       </c>
       <c r="K144" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>Host-tested firmware excludes simultaneous heater bands and rejects demand above 792 W; independent electrical interlock and component ratings still required - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -8226,12 +8226,12 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>EL_ESTOP_BOX</t>
+          <t>EL_DIN_RAIL</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>dual-channel E-stop / lid / service interlock relay box</t>
+          <t>DIN rail 35 mm top-hat x 210</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -8241,12 +8241,12 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>relay box MPN unselected</t>
+          <t>steel rail</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>SAFETY_HARDWARE_REQUIRED</t>
+          <t>PROCUREMENT_HOLD</t>
         </is>
       </c>
       <c r="G145" t="inlineStr">
@@ -8283,12 +8283,12 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>EL_OVERTEMP_BOX</t>
+          <t>EL_DRIVER_1</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>manual-reset independent overtemperature relay box</t>
+          <t>stepper/BLDC driver (M1 branch)</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -8298,12 +8298,12 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>relay box MPN unselected</t>
+          <t>24 V driver MPN unselected</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>SAFETY_HARDWARE_REQUIRED</t>
+          <t>MOTOR_UNSELECTED</t>
         </is>
       </c>
       <c r="G146" t="inlineStr">
@@ -8340,12 +8340,12 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>EL_WIRE_DUCT</t>
+          <t>EL_DRIVER_2</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>slotted wiring duct x 210</t>
+          <t>stepper/BLDC driver (M2 branch)</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -8355,12 +8355,12 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>PVC duct</t>
+          <t>24 V driver MPN unselected</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>PROCUREMENT_HOLD</t>
+          <t>MOTOR_UNSELECTED</t>
         </is>
       </c>
       <c r="G147" t="inlineStr">
@@ -8397,12 +8397,12 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>GUARD_CHAIN_A</t>
+          <t>EL_DRIVER_3</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>chain A top-run lid plate</t>
+          <t>stepper/BLDC driver (winder/puller accessory)</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -8412,17 +8412,17 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>steel plate 3 mm</t>
+          <t>24 V driver MPN unselected</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>CONTAINMENT_UNRATED</t>
+          <t>MOTOR_UNSELECTED</t>
         </is>
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-STAGE3</t>
         </is>
       </c>
       <c r="H148" t="inlineStr">
@@ -8454,12 +8454,12 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>GUARD_CHAIN_B</t>
+          <t>EL_ESTOP_BOX</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>chain B outer guard plate set (4 segments; jackshaft crossing gap)</t>
+          <t>dual-channel E-stop / lid / service interlock relay box</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -8469,17 +8469,17 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>steel plate 3 mm</t>
+          <t>relay box MPN unselected</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>CONTAINMENT_UNRATED</t>
+          <t>SAFETY_HARDWARE_REQUIRED</t>
         </is>
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-STAGE3</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
@@ -8511,12 +8511,12 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>GUARD_LID_INTERLOCK_SEAT</t>
+          <t>EL_OVERTEMP_BOX</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>hopper-lid interlock switch seat</t>
+          <t>manual-reset independent overtemperature relay box</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -8526,17 +8526,17 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>steel plate 3 mm</t>
+          <t>relay box MPN unselected</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>CONTAINMENT_UNRATED</t>
+          <t>SAFETY_HARDWARE_REQUIRED</t>
         </is>
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-STAGE3</t>
         </is>
       </c>
       <c r="H150" t="inlineStr">
@@ -8568,12 +8568,12 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>GUARD_S2_RING</t>
+          <t>EL_WIRE_DUCT</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>S2 rotor ring guard (annular sector r 90..94 over 20..114 deg)</t>
+          <t>slotted wiring duct x 210</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -8583,17 +8583,17 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>steel plate 3 mm</t>
+          <t>PVC duct</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>CONTAINMENT_UNRATED</t>
+          <t>PROCUREMENT_HOLD</t>
         </is>
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-STAGE3</t>
         </is>
       </c>
       <c r="H151" t="inlineStr">
@@ -8613,7 +8613,7 @@
       </c>
       <c r="K151" t="inlineStr">
         <is>
-          <t>Guard plate thickness unrated; service sweep verified - UNQUOTED</t>
+          <t>UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -8625,12 +8625,12 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>PULL_FRAME</t>
+          <t>GUARD_CHAIN_A</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>puller side plates + base (adjustable nip carrier)</t>
+          <t>chain A top-run lid plate</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
@@ -8640,12 +8640,12 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>steel plate 5 mm + 3 mm</t>
+          <t>steel plate 3 mm</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>NIP_RATING_HOLD</t>
+          <t>CONTAINMENT_UNRATED</t>
         </is>
       </c>
       <c r="G152" t="inlineStr">
@@ -8670,7 +8670,7 @@
       </c>
       <c r="K152" t="inlineStr">
         <is>
-          <t>Nip 2.5..5.5 mm with positive stop - UNQUOTED</t>
+          <t>UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -8682,12 +8682,12 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>PULL_MOTOR_REF</t>
+          <t>GUARD_CHAIN_B</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>puller gearmotor reference (not selected)</t>
+          <t>chain B outer guard plate set (continuous; ADR-002 rev B re-route)</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
@@ -8697,12 +8697,12 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>24 V gearmotor MPN unselected</t>
+          <t>steel plate 3 mm</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>MOTOR_UNSELECTED</t>
+          <t>CONTAINMENT_UNRATED</t>
         </is>
       </c>
       <c r="G153" t="inlineStr">
@@ -8727,7 +8727,7 @@
       </c>
       <c r="K153" t="inlineStr">
         <is>
-          <t>UNQUOTED; known motor floors exceed the 100000 KRW soft limit - not 0</t>
+          <t>UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -8739,12 +8739,12 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>PULL_NIP_STOP</t>
+          <t>GUARD_LID_INTERLOCK_SEAT</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>nip positive-stop block (2.5 mm minimum)</t>
+          <t>hopper-lid interlock switch seat</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -8754,12 +8754,12 @@
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>steel</t>
+          <t>steel plate 3 mm</t>
         </is>
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>NIP_RATING_HOLD</t>
+          <t>CONTAINMENT_UNRATED</t>
         </is>
       </c>
       <c r="G154" t="inlineStr">
@@ -8796,12 +8796,12 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>PULL_ROLLER_ADJ</t>
+          <t>GUARD_S2_RING</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>puller adjustable roller dia 20 x 22 + screw carriage</t>
+          <t>S2 rotor ring guard (annular sector r 90..94 over 20..114 deg)</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -8811,12 +8811,12 @@
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>steel; M5 screw</t>
+          <t>steel plate 3 mm</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>NIP_RATING_HOLD</t>
+          <t>CONTAINMENT_UNRATED</t>
         </is>
       </c>
       <c r="G155" t="inlineStr">
@@ -8841,7 +8841,7 @@
       </c>
       <c r="K155" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>Guard plate thickness unrated; service sweep verified - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -8853,12 +8853,12 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>PULL_ROLLER_FIXED</t>
+          <t>PDL_BEARINGS</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>puller drive roller dia 20 x 22</t>
+          <t>two split pillow posts carrying the worm shaft at x353..365, y204..210/352..358</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -8868,22 +8868,22 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>steel; knurl or rubber per TPU grip</t>
+          <t>steel plate 5 mm</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>NIP_RATING_HOLD</t>
+          <t>TRANSFER_UNRATED</t>
         </is>
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -8898,7 +8898,7 @@
       </c>
       <c r="K156" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>Mounted on the support-plate bosses - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -8910,12 +8910,12 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>WIND_FLANGE_L</t>
+          <t>PDL_CHAIN</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>spool flange dia 200</t>
+          <t>#35 roller chain, 35 links incl. offset link; S2 12T second band to PDL_SPROCKET at x362, 1:1</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -8925,22 +8925,22 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>steel plate 6 mm</t>
+          <t>ANSI35 steel roller chain p=9.525</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>WINDER_UNRATED</t>
+          <t>TRANSFER_UNRATED</t>
         </is>
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -8955,7 +8955,7 @@
       </c>
       <c r="K157" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>Nominal333.375 mm versus geometric332.734 mm; 0.641 mm length surplus. Offset-link strength and tension adjustment unqualified; no quote - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -8967,12 +8967,12 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>WIND_FLANGE_R</t>
+          <t>PDL_FEED_GEAR</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>spool flange dia 200</t>
+          <t>12T keyed spur on worm shaft feeding orthogonal screw train</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -8982,22 +8982,22 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>steel plate 6 mm</t>
+          <t>steel reference gear</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>WINDER_UNRATED</t>
+          <t>TRANSFER_UNRATED</t>
         </is>
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -9012,7 +9012,7 @@
       </c>
       <c r="K158" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>Tooth strength and keyed fit unqualified - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -9024,12 +9024,12 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>WIND_MOTOR_REF</t>
+          <t>PDL_SHAFT</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>spool gearmotor reference (not selected)</t>
+          <t>trough worm shaft dia 10 x 188 (r5, y204..392, x362, z374.5), dia 12 keyed chain shoulder y376..392</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -9039,22 +9039,22 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>24 V gearmotor MPN unselected</t>
+          <t>steel rod C45 candidate</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>MOTOR_UNSELECTED</t>
+          <t>TRANSFER_UNRATED</t>
         </is>
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -9069,7 +9069,7 @@
       </c>
       <c r="K159" t="inlineStr">
         <is>
-          <t>UNQUOTED; known motor floors exceed the 100000 KRW soft limit - not 0</t>
+          <t>Carries the RH 2-start worm; keyed 12T sprocket takes 1:1 PDL_CHAIN drive from the S2 12T sprocket - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -9081,12 +9081,12 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>WIND_SPOOL_DRUM</t>
+          <t>PDL_SPROCKET</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>spool drum dia 70 x 58</t>
+          <t>worm-shaft drive sprocket 12T bore 12 mm with keyed hub on shaft shoulder</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
@@ -9096,22 +9096,22 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>steel tube or printed polymer</t>
+          <t>ANSI35 steel sprocket</t>
         </is>
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>WINDER_UNRATED</t>
+          <t>TRANSFER_UNRATED</t>
         </is>
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -9126,7 +9126,7 @@
       </c>
       <c r="K160" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>Bore r6 on y376..392 shaft shoulder r6 with 1.8 mm key in matched slot; torque fit and chain rating UNRATED - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -9138,12 +9138,12 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>WIND_SPOOL_SHAFT</t>
+          <t>PDL_WORM</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>spool shaft dia 16 x 95</t>
+          <t>RH 2-start worm (REFERENCE geometry, unrated): root r6/pitch r6.75/OD r7.5, lead angle 23.3 deg, length 20 (y220..240), keyed Ø10 shaft bore</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -9153,22 +9153,22 @@
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>C45 candidate</t>
+          <t>steel (reference)</t>
         </is>
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>WINDER_UNRATED</t>
+          <t>REFERENCE_UNRATED</t>
         </is>
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
@@ -9183,7 +9183,7 @@
       </c>
       <c r="K161" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>Matched 1.8 mm key and keyway transfer torque from PDL_SHAFT; tooth mesh and loads remain unrated - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -9195,12 +9195,12 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>WIND_TENSIONER</t>
+          <t>PULL_FRAME</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>slip tensioner post + wrap arm</t>
+          <t>puller side plates + base + fixed-roller bearing seats + carriage guide slots</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -9210,22 +9210,22 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>steel</t>
+          <t>steel plate 5 mm + 3 mm</t>
         </is>
       </c>
       <c r="F162" t="inlineStr">
         <is>
-          <t>WINDER_UNRATED</t>
+          <t>NIP_RATING_HOLD</t>
         </is>
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-STAGE4</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-STAGE4</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -9240,7 +9240,7 @@
       </c>
       <c r="K162" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>Positive stop 1.5 mm and adjustable open nip to 3.0 mm; spring carriage grips nominal 1.75 mm filament - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -9252,12 +9252,12 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>WIND_TRAVERSE_RIDER</t>
+          <t>PULL_MOTOR_REF</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>traverse rider block + guide eyelet</t>
+          <t>puller gearmotor reference (not selected)</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
@@ -9267,12 +9267,12 @@
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>steel + printed guide</t>
+          <t>24 V gearmotor MPN unselected</t>
         </is>
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>WINDER_UNRATED</t>
+          <t>MOTOR_UNSELECTED</t>
         </is>
       </c>
       <c r="G163" t="inlineStr">
@@ -9297,7 +9297,7 @@
       </c>
       <c r="K163" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>UNQUOTED; known motor floors exceed the 100000 KRW soft limit - not 0</t>
         </is>
       </c>
     </row>
@@ -9309,50 +9309,677 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
+          <t>PULL_NIP_STOP</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>nip positive-stop cam block (1.5 mm minimum, 3.0 mm open)</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>steel</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>NIP_RATING_HOLD</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>VP1-STAGE2</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>VP1-STAGE3</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>UNQUOTED_NOT_ZERO</t>
+        </is>
+      </c>
+      <c r="K164" t="inlineStr">
+        <is>
+          <t>UNQUOTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>vp1_stage1_3</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>PULL_ROLLER_ADJ</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>puller adjustable roller dia 20 + spring-loaded carriage (guide posts, coil springs, cam stop)</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>steel; M5 screw</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>NIP_RATING_HOLD</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>VP1-STAGE2</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>VP1-STAGE3</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>UNQUOTED_NOT_ZERO</t>
+        </is>
+      </c>
+      <c r="K165" t="inlineStr">
+        <is>
+          <t>Spring-loaded carrier grips 1.5-2.0 mm filament (1.75 nominal, design/parameters.json filament_mm); cam stop range 1.5..3.0 mm - UNQUOTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>vp1_stage1_3</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>PULL_ROLLER_FIXED</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>puller drive roller dia 20 x 22</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>steel; knurl or rubber per TPU grip</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>NIP_RATING_HOLD</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>VP1-STAGE2</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>VP1-STAGE3</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>UNQUOTED_NOT_ZERO</t>
+        </is>
+      </c>
+      <c r="K166" t="inlineStr">
+        <is>
+          <t>UNQUOTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>vp1_stage1_3</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>WIND_FLANGE_L</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>spool flange dia 200</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>steel plate 6 mm</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>WINDER_UNRATED</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>VP1-STAGE2</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>VP1-STAGE3</t>
+        </is>
+      </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>UNQUOTED_NOT_ZERO</t>
+        </is>
+      </c>
+      <c r="K167" t="inlineStr">
+        <is>
+          <t>UNQUOTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>vp1_stage1_3</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>WIND_FLANGE_R</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>spool flange dia 200</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>steel plate 6 mm</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>WINDER_UNRATED</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>VP1-STAGE2</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>VP1-STAGE3</t>
+        </is>
+      </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>UNQUOTED_NOT_ZERO</t>
+        </is>
+      </c>
+      <c r="K168" t="inlineStr">
+        <is>
+          <t>UNQUOTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>vp1_stage1_3</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>WIND_MOTOR_REF</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>spool gearmotor reference (not selected)</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>24 V gearmotor MPN unselected</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>MOTOR_UNSELECTED</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>VP1-STAGE2</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>VP1-STAGE3</t>
+        </is>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>UNQUOTED_NOT_ZERO</t>
+        </is>
+      </c>
+      <c r="K169" t="inlineStr">
+        <is>
+          <t>UNQUOTED; known motor floors exceed the 100000 KRW soft limit - not 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>vp1_stage1_3</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>WIND_SPOOL_BEARINGS</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>spool shaft bearing blocks at BOTH shaft ends</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>steel plate 5 mm + bearing seats</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>WINDER_UNRATED</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>VP1-STAGE4</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>VP1-STAGE4</t>
+        </is>
+      </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>UNQUOTED_NOT_ZERO</t>
+        </is>
+      </c>
+      <c r="K170" t="inlineStr">
+        <is>
+          <t>VP1 Stage 4 grip redesign: shaft supported at both ends - UNQUOTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>vp1_stage1_3</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>WIND_SPOOL_DRUM</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>spool drum dia 70 x 58</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>steel tube or printed polymer</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>WINDER_UNRATED</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>VP1-STAGE2</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>VP1-STAGE3</t>
+        </is>
+      </c>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>UNQUOTED_NOT_ZERO</t>
+        </is>
+      </c>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>UNQUOTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>vp1_stage1_3</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>WIND_SPOOL_SHAFT</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>spool shaft dia 16 x 95</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>C45 candidate</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>WINDER_UNRATED</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>VP1-STAGE2</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>VP1-STAGE3</t>
+        </is>
+      </c>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t>UNQUOTED_NOT_ZERO</t>
+        </is>
+      </c>
+      <c r="K172" t="inlineStr">
+        <is>
+          <t>UNQUOTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>vp1_stage1_3</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>WIND_TENSIONER</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>slip tensioner post + wrap arm</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>steel</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>WINDER_UNRATED</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>VP1-STAGE2</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>VP1-STAGE3</t>
+        </is>
+      </c>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J173" t="inlineStr">
+        <is>
+          <t>UNQUOTED_NOT_ZERO</t>
+        </is>
+      </c>
+      <c r="K173" t="inlineStr">
+        <is>
+          <t>UNQUOTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>vp1_stage1_3</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>WIND_TRAVERSE_RIDER</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>traverse rider block + guide eyelet</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>steel + printed guide</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>WINDER_UNRATED</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>VP1-STAGE2</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>VP1-STAGE3</t>
+        </is>
+      </c>
+      <c r="I174" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J174" t="inlineStr">
+        <is>
+          <t>UNQUOTED_NOT_ZERO</t>
+        </is>
+      </c>
+      <c r="K174" t="inlineStr">
+        <is>
+          <t>UNQUOTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>vp1_stage1_3</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
           <t>WIND_TRAVERSE_SCREW</t>
         </is>
       </c>
-      <c r="C164" t="inlineStr">
+      <c r="C175" t="inlineStr">
         <is>
           <t>traverse lead screw dia 8 x 80</t>
         </is>
       </c>
-      <c r="D164" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E164" t="inlineStr">
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
         <is>
           <t>steel rod</t>
         </is>
       </c>
-      <c r="F164" t="inlineStr">
+      <c r="F175" t="inlineStr">
         <is>
           <t>WINDER_UNRATED</t>
         </is>
       </c>
-      <c r="G164" t="inlineStr">
+      <c r="G175" t="inlineStr">
         <is>
           <t>VP1-STAGE2</t>
         </is>
       </c>
-      <c r="H164" t="inlineStr">
+      <c r="H175" t="inlineStr">
         <is>
           <t>VP1-STAGE3</t>
         </is>
       </c>
-      <c r="I164" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J164" t="inlineStr">
+      <c r="I175" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J175" t="inlineStr">
         <is>
           <t>UNQUOTED_NOT_ZERO</t>
         </is>
       </c>
-      <c r="K164" t="inlineStr">
+      <c r="K175" t="inlineStr">
         <is>
           <t>UNQUOTED</t>
         </is>

</xml_diff>

<commit_message>
Record VP1 powered-transfer geometry and localized flow HOLD
</commit_message>
<xml_diff>
--- a/c2.1/bom/system_bom.xlsx
+++ b/c2.1/bom/system_bom.xlsx
@@ -7889,7 +7889,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>LH helical screw on y-axis x357/z328 with 9 mm pitch and radius 10 mm flight</t>
+          <t>RH helical screw on y-axis x357/z328 with 9 mm pitch and radius 10 mm flight</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -9480,37 +9480,37 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>WIND_FLANGE_L</t>
+          <t>S1_BELT</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>spool flange dia 200</t>
+          <t>two side-loop treads over x80..219; y163.5..223.2 and 240.8..323.5</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>steel plate 6 mm</t>
+          <t>polymer belt with steel-supported drums</t>
         </is>
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>WINDER_UNRATED</t>
+          <t>TRANSFER_UNRATED</t>
         </is>
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -9525,7 +9525,7 @@
       </c>
       <c r="K167" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>Friction and tension unrated; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -9537,12 +9537,12 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>WIND_FLANGE_R</t>
+          <t>S1_BELT_BEARINGS</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>spool flange dia 200</t>
+          <t>four belt shaft support rings in the side rails</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
@@ -9552,22 +9552,22 @@
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>steel plate 6 mm</t>
+          <t>steel bearing seats</t>
         </is>
       </c>
       <c r="F168" t="inlineStr">
         <is>
-          <t>WINDER_UNRATED</t>
+          <t>TRANSFER_UNRATED</t>
         </is>
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
@@ -9582,7 +9582,7 @@
       </c>
       <c r="K168" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>Bearing selection and loads unqualified; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -9594,12 +9594,12 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>WIND_MOTOR_REF</t>
+          <t>S1_BELT_CHAIN</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>spool gearmotor reference (not selected)</t>
+          <t>#35 chain from S1B 24T to west belt 12T</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
@@ -9609,22 +9609,22 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>24 V gearmotor MPN unselected</t>
+          <t>ANSI35 steel chain</t>
         </is>
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>MOTOR_UNSELECTED</t>
+          <t>TRANSFER_UNRATED</t>
         </is>
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
@@ -9639,7 +9639,7 @@
       </c>
       <c r="K169" t="inlineStr">
         <is>
-          <t>UNQUOTED; known motor floors exceed the 100000 KRW soft limit - not 0</t>
+          <t>Tension and strength unrated; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -9651,12 +9651,12 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>WIND_SPOOL_BEARINGS</t>
+          <t>S1_BELT_DRIVE</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>spool shaft bearing blocks at BOTH shaft ends</t>
+          <t>common waisted drive drum at x80; separate r3.8 side and r2.3 central tread seats</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -9666,22 +9666,22 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>steel plate 5 mm + bearing seats</t>
+          <t>steel shaft and drums</t>
         </is>
       </c>
       <c r="F170" t="inlineStr">
         <is>
-          <t>WINDER_UNRATED</t>
+          <t>TRANSFER_UNRATED</t>
         </is>
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t>VP1-STAGE4</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>VP1-STAGE4</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
@@ -9696,7 +9696,7 @@
       </c>
       <c r="K170" t="inlineStr">
         <is>
-          <t>VP1 Stage 4 grip redesign: shaft supported at both ends - UNQUOTED</t>
+          <t>S1B chain-driven; torque and bearing load unrated; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -9708,12 +9708,12 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>WIND_SPOOL_DRUM</t>
+          <t>S1_BELT_FOLLOWER</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>spool drum dia 70 x 58</t>
+          <t>12T sprocket on the west belt driver</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
@@ -9723,22 +9723,22 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>steel tube or printed polymer</t>
+          <t>ANSI35 steel sprocket</t>
         </is>
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t>WINDER_UNRATED</t>
+          <t>TRANSFER_UNRATED</t>
         </is>
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
@@ -9765,12 +9765,12 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>WIND_SPOOL_SHAFT</t>
+          <t>S1_BELT_IDLER</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>spool shaft dia 16 x 95</t>
+          <t>two split side idler drums at x219 leaving the central transfer corridor open</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
@@ -9780,22 +9780,22 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>C45 candidate</t>
+          <t>steel journals and drums</t>
         </is>
       </c>
       <c r="F172" t="inlineStr">
         <is>
-          <t>WINDER_UNRATED</t>
+          <t>TRANSFER_UNRATED</t>
         </is>
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
@@ -9810,7 +9810,7 @@
       </c>
       <c r="K172" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>Two independent journal halves; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -9822,12 +9822,12 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>WIND_TENSIONER</t>
+          <t>S1_SWEEP_BEARINGS</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>slip tensioner post + wrap arm</t>
+          <t>two separated sweep bearing rings in the pan rails</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
@@ -9837,22 +9837,22 @@
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>steel</t>
+          <t>steel bearing seats</t>
         </is>
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>WINDER_UNRATED</t>
+          <t>TRANSFER_UNRATED</t>
         </is>
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
@@ -9879,12 +9879,12 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>WIND_TRAVERSE_RIDER</t>
+          <t>S1_SWEEP_GEAR_DRUM_N</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>traverse rider block + guide eyelet</t>
+          <t>12T gear on the north east belt idler</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
@@ -9894,22 +9894,22 @@
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>steel + printed guide</t>
+          <t>steel gear</t>
         </is>
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>WINDER_UNRATED</t>
+          <t>TRANSFER_UNRATED</t>
         </is>
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
@@ -9936,50 +9936,962 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
+          <t>S1_SWEEP_GEAR_DRUM_S</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>12T gear on the south east belt idler</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>steel gear</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>TRANSFER_UNRATED</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>VP1-STAGE5</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>VP1-STAGE5</t>
+        </is>
+      </c>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J175" t="inlineStr">
+        <is>
+          <t>UNQUOTED_NOT_ZERO</t>
+        </is>
+      </c>
+      <c r="K175" t="inlineStr">
+        <is>
+          <t>UNQUOTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>vp1_stage1_3</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>S1_SWEEP_GEAR_N</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>12T gear on the north sweep shaft</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>steel gear</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>TRANSFER_UNRATED</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>VP1-STAGE5</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>VP1-STAGE5</t>
+        </is>
+      </c>
+      <c r="I176" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J176" t="inlineStr">
+        <is>
+          <t>UNQUOTED_NOT_ZERO</t>
+        </is>
+      </c>
+      <c r="K176" t="inlineStr">
+        <is>
+          <t>UNQUOTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>vp1_stage1_3</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>S1_SWEEP_GEAR_S</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>12T gear on the south sweep shaft</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>steel gear</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>TRANSFER_UNRATED</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>VP1-STAGE5</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>VP1-STAGE5</t>
+        </is>
+      </c>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J177" t="inlineStr">
+        <is>
+          <t>UNQUOTED_NOT_ZERO</t>
+        </is>
+      </c>
+      <c r="K177" t="inlineStr">
+        <is>
+          <t>UNQUOTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>vp1_stage1_3</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>S1_SWEEP_NORTH</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>north transverse screw x226 y236..359 feeding the central lane</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>steel shaft and flight</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>TRANSFER_UNRATED</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>VP1-STAGE5</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>VP1-STAGE5</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>UNQUOTED_NOT_ZERO</t>
+        </is>
+      </c>
+      <c r="K178" t="inlineStr">
+        <is>
+          <t>Contact pickup unproven; UNQUOTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>vp1_stage1_3</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>S1_SWEEP_SOUTH</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>south transverse screw x226 y127..228 feeding the central lane</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>steel shaft and flight</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>TRANSFER_UNRATED</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>VP1-STAGE5</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>VP1-STAGE5</t>
+        </is>
+      </c>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>UNQUOTED_NOT_ZERO</t>
+        </is>
+      </c>
+      <c r="K179" t="inlineStr">
+        <is>
+          <t>Contact pickup unproven; UNQUOTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>vp1_stage1_3</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>S1_TRANSFER_BEARINGS</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>two central idler support rings</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>steel bearing seats</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>TRANSFER_UNRATED</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>VP1-STAGE5</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>VP1-STAGE5</t>
+        </is>
+      </c>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>UNQUOTED_NOT_ZERO</t>
+        </is>
+      </c>
+      <c r="K180" t="inlineStr">
+        <is>
+          <t>UNQUOTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>vp1_stage1_3</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>S1_TRANSFER_BELT</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>central 17 mm tread from x80 to x233.4 inside the two side loops</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>polymer belt</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>TRANSFER_UNRATED</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>VP1-STAGE5</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>VP1-STAGE5</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>UNQUOTED_NOT_ZERO</t>
+        </is>
+      </c>
+      <c r="K181" t="inlineStr">
+        <is>
+          <t>Screw pickup unproven; UNQUOTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>vp1_stage1_3</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>S1_TRANSFER_IDLER</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>central east r2.3 idler at x233.4</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>steel drum</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>TRANSFER_UNRATED</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>VP1-STAGE5</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>VP1-STAGE5</t>
+        </is>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J182" t="inlineStr">
+        <is>
+          <t>UNQUOTED_NOT_ZERO</t>
+        </is>
+      </c>
+      <c r="K182" t="inlineStr">
+        <is>
+          <t>UNQUOTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>vp1_stage1_3</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>WIND_FLANGE_L</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>spool flange dia 200</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>steel plate 6 mm</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>WINDER_UNRATED</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>VP1-STAGE2</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>VP1-STAGE3</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J183" t="inlineStr">
+        <is>
+          <t>UNQUOTED_NOT_ZERO</t>
+        </is>
+      </c>
+      <c r="K183" t="inlineStr">
+        <is>
+          <t>UNQUOTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>vp1_stage1_3</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>WIND_FLANGE_R</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>spool flange dia 200</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>steel plate 6 mm</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>WINDER_UNRATED</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>VP1-STAGE2</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>VP1-STAGE3</t>
+        </is>
+      </c>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J184" t="inlineStr">
+        <is>
+          <t>UNQUOTED_NOT_ZERO</t>
+        </is>
+      </c>
+      <c r="K184" t="inlineStr">
+        <is>
+          <t>UNQUOTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>vp1_stage1_3</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>WIND_MOTOR_REF</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>spool gearmotor reference (not selected)</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>24 V gearmotor MPN unselected</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>MOTOR_UNSELECTED</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>VP1-STAGE2</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>VP1-STAGE3</t>
+        </is>
+      </c>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J185" t="inlineStr">
+        <is>
+          <t>UNQUOTED_NOT_ZERO</t>
+        </is>
+      </c>
+      <c r="K185" t="inlineStr">
+        <is>
+          <t>UNQUOTED; known motor floors exceed the 100000 KRW soft limit - not 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>vp1_stage1_3</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>WIND_SPOOL_BEARINGS</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>spool shaft bearing blocks at BOTH shaft ends</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>steel plate 5 mm + bearing seats</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>WINDER_UNRATED</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>VP1-STAGE4</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>VP1-STAGE4</t>
+        </is>
+      </c>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J186" t="inlineStr">
+        <is>
+          <t>UNQUOTED_NOT_ZERO</t>
+        </is>
+      </c>
+      <c r="K186" t="inlineStr">
+        <is>
+          <t>VP1 Stage 4 grip redesign: shaft supported at both ends - UNQUOTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>vp1_stage1_3</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>WIND_SPOOL_DRUM</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>spool drum dia 70 x 58</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>steel tube or printed polymer</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>WINDER_UNRATED</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>VP1-STAGE2</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>VP1-STAGE3</t>
+        </is>
+      </c>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J187" t="inlineStr">
+        <is>
+          <t>UNQUOTED_NOT_ZERO</t>
+        </is>
+      </c>
+      <c r="K187" t="inlineStr">
+        <is>
+          <t>UNQUOTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>vp1_stage1_3</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>WIND_SPOOL_SHAFT</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>spool shaft dia 16 x 95</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>C45 candidate</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>WINDER_UNRATED</t>
+        </is>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>VP1-STAGE2</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>VP1-STAGE3</t>
+        </is>
+      </c>
+      <c r="I188" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J188" t="inlineStr">
+        <is>
+          <t>UNQUOTED_NOT_ZERO</t>
+        </is>
+      </c>
+      <c r="K188" t="inlineStr">
+        <is>
+          <t>UNQUOTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>vp1_stage1_3</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>WIND_TENSIONER</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>slip tensioner post + wrap arm</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>steel</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>WINDER_UNRATED</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>VP1-STAGE2</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>VP1-STAGE3</t>
+        </is>
+      </c>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J189" t="inlineStr">
+        <is>
+          <t>UNQUOTED_NOT_ZERO</t>
+        </is>
+      </c>
+      <c r="K189" t="inlineStr">
+        <is>
+          <t>UNQUOTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>vp1_stage1_3</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>WIND_TRAVERSE_RIDER</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>traverse rider block + guide eyelet</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>steel + printed guide</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>WINDER_UNRATED</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>VP1-STAGE2</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>VP1-STAGE3</t>
+        </is>
+      </c>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J190" t="inlineStr">
+        <is>
+          <t>UNQUOTED_NOT_ZERO</t>
+        </is>
+      </c>
+      <c r="K190" t="inlineStr">
+        <is>
+          <t>UNQUOTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>vp1_stage1_3</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
           <t>WIND_TRAVERSE_SCREW</t>
         </is>
       </c>
-      <c r="C175" t="inlineStr">
+      <c r="C191" t="inlineStr">
         <is>
           <t>traverse lead screw dia 8 x 80</t>
         </is>
       </c>
-      <c r="D175" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E175" t="inlineStr">
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
         <is>
           <t>steel rod</t>
         </is>
       </c>
-      <c r="F175" t="inlineStr">
+      <c r="F191" t="inlineStr">
         <is>
           <t>WINDER_UNRATED</t>
         </is>
       </c>
-      <c r="G175" t="inlineStr">
+      <c r="G191" t="inlineStr">
         <is>
           <t>VP1-STAGE2</t>
         </is>
       </c>
-      <c r="H175" t="inlineStr">
+      <c r="H191" t="inlineStr">
         <is>
           <t>VP1-STAGE3</t>
         </is>
       </c>
-      <c r="I175" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J175" t="inlineStr">
+      <c r="I191" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J191" t="inlineStr">
         <is>
           <t>UNQUOTED_NOT_ZERO</t>
         </is>
       </c>
-      <c r="K175" t="inlineStr">
+      <c r="K191" t="inlineStr">
         <is>
           <t>UNQUOTED</t>
         </is>

</xml_diff>

<commit_message>
Record VP1 integrated flow failure and restore 500W hard cap
</commit_message>
<xml_diff>
--- a/c2.1/bom/system_bom.xlsx
+++ b/c2.1/bom/system_bom.xlsx
@@ -707,7 +707,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>perforated curved screen reference</t>
+          <t>VP1 gravity-aligned perforated curved screen</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -727,7 +727,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>C2-CAD</t>
+          <t>C2.1-CAD</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -747,7 +747,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Actual perforated C2 generated geometry is integrated; hole diameter does not guarantee maximum particle length</t>
+          <t>Current C2.1 generated screen has 78 straight Ø3 exit paths into buffer; particle capture flow ligament strength mounting and particle length limit remain unverified</t>
         </is>
       </c>
     </row>
@@ -7490,7 +7490,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>active auger conveyor: r3 shaft x236..370 at y232/z347.1; RH flight root r3/OD r8, pitch 28.5, four turns x238.5..352.5 with 3 mm swept face; 0.032 mm BRep U-shell gap</t>
+          <t>active auger conveyor: r3 shaft x236..370 at y232/z347.1; RH flight root r3/OD r8, pitch 28.5, four turns x238.5..352.5 with 3 mm swept face; U-shell bore r9.5, nominal BRep gap 1.085 mm</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -7530,7 +7530,7 @@
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>Conveys +x at -5.4375 rpm for 58 rpm reference M1 via 15/40 gear and 24/12 chain B plus 8:1 worm/wheel; S1 pan pickup and S2 handoff need connected validation - UNQUOTED</t>
+          <t>Conveys +x at -5.4375 rpm for 58 rpm reference M1 via 15/40 gear and 24/12 chain B plus 8:1 worm/wheel; tolerance/runout/heat stack assumed not proven</t>
         </is>
       </c>
     </row>
@@ -7889,7 +7889,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>RH helical screw on y-axis x357/z328 with 9 mm pitch and radius 10 mm flight</t>
+          <t>RH helical screw on y-axis x357/z328 with 9 mm pitch; reduced-radius powered tail to y260.5</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -7929,7 +7929,7 @@
       </c>
       <c r="K139" t="inlineStr">
         <is>
-          <t>Active +Y transfer to y250.7; frozen south cap y251..255 remains and final material passage unproven - UNQUOTED</t>
+          <t>Powered tail overlaps S2 mouth y255 by 5.502 mm; actual fragment handoff unproven - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -7946,7 +7946,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>U cradle and cap-bore inner-radius 5 mm passive outlet bridge</t>
+          <t>U cradle with rotor-relieved outer metal shelf past S2 mouth</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -7986,7 +7986,7 @@
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>Shell does not cut frozen S2 cap; material crossing cap bridge unproven - UNQUOTED</t>
+          <t>Outer shelf y255..258 supports the handoff without entering swept rotor sector; material transfer unproven - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10112,7 +10112,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>north transverse screw x226 y236..359 feeding the central lane</t>
+          <t>north transverse screw x224 y235.5..359 feeding the central lane</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
@@ -10152,7 +10152,7 @@
       </c>
       <c r="K178" t="inlineStr">
         <is>
-          <t>Contact pickup unproven; UNQUOTED</t>
+          <t>Dynamic side-belt pickup under verification; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10169,7 +10169,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>south transverse screw x226 y127..228 feeding the central lane</t>
+          <t>south transverse screw x224 y127..228.5 feeding the central lane</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
@@ -10209,7 +10209,7 @@
       </c>
       <c r="K179" t="inlineStr">
         <is>
-          <t>Contact pickup unproven; UNQUOTED</t>
+          <t>Dynamic side-belt pickup under verification; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10283,7 +10283,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>central 17 mm tread from x80 to x233.4 inside the two side loops</t>
+          <t>central 17 mm tread from x80 to x260 inside the two side loops</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
@@ -10340,7 +10340,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>central east r2.3 idler at x233.4</t>
+          <t>central east r2.3 idler at x260</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">

</xml_diff>

<commit_message>
VP1: integrate material-aware CAD and report connected flow HOLD
</commit_message>
<xml_diff>
--- a/c2.1/bom/system_bom.xlsx
+++ b/c2.1/bom/system_bom.xlsx
@@ -5428,17 +5428,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>legacy_interface:feed</t>
+          <t>legacy_interface:frame</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>HOPPER</t>
+          <t>FR-2020-320</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>35deg batch hopper</t>
+          <t>2020 profile cut320</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -5448,17 +5448,17 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>PC shell + steel lower liner</t>
+          <t>Al extrusion - existing</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>CUSTOM_DFM_HOLD</t>
+          <t>OWNED_SLOT_PATTERN_TO_MEASURE</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>PPR-C1 original dimensional design; not an empirical qualification</t>
+          <t>PPR_project_handover_2026-09-20.zip / 08_BOM_COMPONENTS.md</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
@@ -5468,17 +5468,17 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t/>
+          <t>0</t>
         </is>
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>OWNED_NO_NEW_PURCHASE</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
         <is>
-          <t>Whole hopper exceeds print limit; must split into &lt;=210mm panels before printing. Closed lid and standstill interlock mandatory; angle is not an access safety measure.</t>
+          <t>Nominal section only. Confirm slot series before buying brackets; 3 mm saw kerf.</t>
         </is>
       </c>
     </row>
@@ -5490,17 +5490,17 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>FR-2020-320</t>
+          <t>FR-2020-360</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>2020 profile cut320</t>
+          <t>2020 profile cut 360</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -5547,17 +5547,17 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>FR-2020-360</t>
+          <t>FR-2020-400</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>2020 profile cut 360</t>
+          <t>2020 profile cut 400</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -5604,12 +5604,12 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>FR-2020-400</t>
+          <t>FR-2020-590</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>2020 profile cut 400</t>
+          <t>2020 profile cut 590</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -5661,12 +5661,12 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>FR-2020-590</t>
+          <t>FR-2040-320</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>2020 profile cut 590</t>
+          <t>2040 profile cut 320</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -5718,12 +5718,12 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>FR-2040-320</t>
+          <t>FR-2040-400</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>2040 profile cut 320</t>
+          <t>2040 profile cut 400</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -5775,12 +5775,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>FR-2040-400</t>
+          <t>FR-2040-630</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>2040 profile cut 400</t>
+          <t>2040 profile cut 630</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -5832,32 +5832,32 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>FR-2040-630</t>
+          <t>FR-BASE</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>2040 profile cut 630</t>
+          <t>Bottom tray 630x400x3</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Al extrusion - existing</t>
+          <t>Al 5052</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>OWNED_SLOT_PATTERN_TO_MEASURE</t>
+          <t>SHEET_DFM_HOLD</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>PPR_project_handover_2026-09-20.zip / 08_BOM_COMPONENTS.md</t>
+          <t>PPR-C1 original dimensional design; not an empirical qualification</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
@@ -5867,34 +5867,34 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>0</t>
+          <t/>
         </is>
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>OWNED_NO_NEW_PURCHASE</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
         <is>
-          <t>Nominal section only. Confirm slot series before buying brackets; 3 mm saw kerf.</t>
+          <t>Mains and hot zones require separate partitions; shown base is not sealed containment.</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>legacy_interface:frame</t>
+          <t>legacy_interface:frame_mount</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>FR-BASE</t>
+          <t>DRV-DECK</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Bottom tray 630x400x3</t>
+          <t>Steel drive deck240x194x5</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -5904,12 +5904,12 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Al 5052</t>
+          <t>S355 steel</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>SHEET_DFM_HOLD</t>
+          <t>CUSTOM_DFM_HOLD</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
@@ -5934,7 +5934,7 @@
       </c>
       <c r="K104" t="inlineStr">
         <is>
-          <t>Mains and hot zones require separate partitions; shown base is not sealed containment.</t>
+          <t>Deck atZ20..25, supported by existing crossmembers. Added4 feet must be included in frame stiffness review.</t>
         </is>
       </c>
     </row>
@@ -5946,12 +5946,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>DRV-DECK</t>
+          <t>DRV-M1-FOOT</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Steel drive deck240x194x5</t>
+          <t>M1 steel mounting foot70x50x19</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -5961,7 +5961,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>S355 steel</t>
+          <t>Steel</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -5991,7 +5991,7 @@
       </c>
       <c r="K105" t="inlineStr">
         <is>
-          <t>Deck atZ20..25, supported by existing crossmembers. Added4 feet must be included in frame stiffness review.</t>
+          <t>Motor plate corner holes to vertical face. Base bolts to drive deck, not to a printed carrier.</t>
         </is>
       </c>
     </row>
@@ -6003,12 +6003,12 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>DRV-M1-FOOT</t>
+          <t>DRV-RISER12</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>M1 steel mounting foot70x50x19</t>
+          <t>Input rear bearing riser34x12x10</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -6048,7 +6048,7 @@
       </c>
       <c r="K106" t="inlineStr">
         <is>
-          <t>Motor plate corner holes to vertical face. Base bolts to drive deck, not to a printed carrier.</t>
+          <t>Bearing bolt pattern must be transferred to deck after slots/profile series confirmed.</t>
         </is>
       </c>
     </row>
@@ -6060,12 +6060,12 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>DRV-RISER12</t>
+          <t>DRV-RISER20</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Input rear bearing riser34x12x10</t>
+          <t>Output rear bearing shim70x18x2.5</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -6105,7 +6105,7 @@
       </c>
       <c r="K107" t="inlineStr">
         <is>
-          <t>Bearing bolt pattern must be transferred to deck after slots/profile series confirmed.</t>
+          <t>2.50 ground shim, full metal bearing support.</t>
         </is>
       </c>
     </row>
@@ -6117,12 +6117,12 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>DRV-RISER20</t>
+          <t>EX-STAND</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Output rear bearing shim70x18x2.5</t>
+          <t>Thrust stand / coaxial motor bridge</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -6162,7 +6162,7 @@
       </c>
       <c r="K108" t="inlineStr">
         <is>
-          <t>2.50 ground shim, full metal bearing support.</t>
+          <t>M2 and thrust carrier share metal stand on deck; no large right-angle gearbox. Top holes4xM6 to carrier. Weld/bolt/pressure proof remains HOLD.</t>
         </is>
       </c>
     </row>
@@ -6174,22 +6174,22 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>EX-STAND</t>
+          <t>S1-ROOF-F</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Thrust stand / coaxial motor bridge</t>
+          <t>Front roof bracket30x95x25</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Steel</t>
+          <t>10mm steel welded/folded</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
@@ -6219,7 +6219,7 @@
       </c>
       <c r="K109" t="inlineStr">
         <is>
-          <t>M2 and thrust carrier share metal stand on deck; no large right-angle gearbox. Top holes4xM6 to carrier. Weld/bolt/pressure proof remains HOLD.</t>
+          <t>Face atY135 against retainer. M6 top hole to existing profile centreY50. Metal roof load path; bend/weld qualification pending.</t>
         </is>
       </c>
     </row>
@@ -6231,12 +6231,12 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>S1-ROOF-F</t>
+          <t>S1-ROOF-R</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Front roof bracket30x95x25</t>
+          <t>Rear roof bracket30x48x25</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -6276,7 +6276,7 @@
       </c>
       <c r="K110" t="inlineStr">
         <is>
-          <t>Face atY135 against retainer. M6 top hole to existing profile centreY50. Metal roof load path; bend/weld qualification pending.</t>
+          <t>Face atY352; M6 profile connection atY390. Do not print this bracket.</t>
         </is>
       </c>
     </row>
@@ -6288,12 +6288,12 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>S1-ROOF-R</t>
+          <t>S2-LEG-L</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Rear roof bracket30x48x25</t>
+          <t>S2 L column / metal foot</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -6303,7 +6303,7 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>10mm steel welded/folded</t>
+          <t>Steel</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
@@ -6333,7 +6333,7 @@
       </c>
       <c r="K111" t="inlineStr">
         <is>
-          <t>Face atY352; M6 profile connection atY390. Do not print this bracket.</t>
+          <t>Foot bottomZ25; topZ210. Centre mounting holeZ203. L sits on5mm deck, R on2020crossmember. Welded joint and anchors DFM hold.</t>
         </is>
       </c>
     </row>
@@ -6345,12 +6345,12 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>S2-LEG-L</t>
+          <t>S2-LEG-R</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>S2 L column / metal foot</t>
+          <t>S2 R column / metal foot</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -6390,44 +6390,44 @@
       </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t>Foot bottomZ25; topZ210. Centre mounting holeZ203. L sits on5mm deck, R on2020crossmember. Welded joint and anchors DFM hold.</t>
+          <t>Foot bottomZ20; topZ210. Centre mounting holeZ203. L sits on5mm deck, R on2020crossmember. Welded joint and anchors DFM hold.</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>legacy_interface:frame_mount</t>
+          <t>system_requirement</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>S2-LEG-R</t>
+          <t>AUX-DRIVES</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>S2 R column / metal foot</t>
+          <t>Puller,spool,traverse actuation</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Steel</t>
+          <t>Procurement requirement</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>CUSTOM_DFM_HOLD</t>
+          <t>AUX_ACTUATION_HOLD</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>PPR-C1 original dimensional design; not an empirical qualification</t>
+          <t>Supplier drawing / capacity confirmation required before procurement</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
@@ -6447,7 +6447,7 @@
       </c>
       <c r="K113" t="inlineStr">
         <is>
-          <t>Foot bottomZ20; topZ210. Centre mounting holeZ203. L sits on5mm deck, R on2020crossmember. Welded joint and anchors DFM hold.</t>
+          <t>Separate low-power controls, no large third shredder motor.</t>
         </is>
       </c>
     </row>
@@ -6459,12 +6459,12 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>AUX-DRIVES</t>
+          <t>CHAIN-A</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Puller,spool,traverse actuation</t>
+          <t>ANSI35 chain94 pitches</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -6479,7 +6479,7 @@
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>AUX_ACTUATION_HOLD</t>
+          <t>CHAIN_RATING_HOLD</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
@@ -6504,7 +6504,7 @@
       </c>
       <c r="K114" t="inlineStr">
         <is>
-          <t>Separate low-power controls, no large third shredder motor.</t>
+          <t>Pitch length895.35mm. Working load and width to confirm.</t>
         </is>
       </c>
     </row>
@@ -6516,12 +6516,12 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>CHAIN-A</t>
+          <t>CHAIN-B</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>ANSI35 chain94 pitches</t>
+          <t>ANSI35 chain84 pitches</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -6561,7 +6561,7 @@
       </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t>Pitch length895.35mm. Working load and width to confirm.</t>
+          <t>Pitch length800.10mm. Working load and width to confirm.</t>
         </is>
       </c>
     </row>
@@ -6573,12 +6573,12 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>CHAIN-B</t>
+          <t>CTRL-MEGA</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>ANSI35 chain84 pitches</t>
+          <t>Arduino Mega</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -6593,12 +6593,12 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>CHAIN_RATING_HOLD</t>
+          <t>OWNED</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>Supplier drawing / capacity confirmation required before procurement</t>
+          <t>PPR_project_handover_2026-09-20.zip / 08_BOM_COMPONENTS.md</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
@@ -6608,17 +6608,17 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t/>
+          <t>0</t>
         </is>
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>OWNED_NO_NEW_PURCHASE</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
         <is>
-          <t>Pitch length800.10mm. Working load and width to confirm.</t>
+          <t>Reference power allocator is NOT deployable heater firmware.</t>
         </is>
       </c>
     </row>
@@ -6630,12 +6630,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>CTRL-MEGA</t>
+          <t>DRV-TLIMIT</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Arduino Mega</t>
+          <t>Mechanical torque limiter</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -6650,12 +6650,12 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>OWNED</t>
+          <t>TORQUE_LIMITER_HOLD</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>PPR_project_handover_2026-09-20.zip / 08_BOM_COMPONENTS.md</t>
+          <t>Supplier drawing / capacity confirmation required before procurement</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
@@ -6665,17 +6665,17 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>0</t>
+          <t/>
         </is>
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>OWNED_NO_NEW_PURCHASE</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>Reference power allocator is NOT deployable heater firmware.</t>
+          <t>Shared M1 input; calibration before blade operation.</t>
         </is>
       </c>
     </row>
@@ -6687,17 +6687,17 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>DRV-TLIMIT</t>
+          <t>EL-BTS</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Mechanical torque limiter</t>
+          <t>Existing BTS7960 modules</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -6707,12 +6707,12 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>TORQUE_LIMITER_HOLD</t>
+          <t>OWNED_UNQUALIFIED</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>Supplier drawing / capacity confirmation required before procurement</t>
+          <t>PPR_project_handover_2026-09-20.zip / 08_BOM_COMPONENTS.md</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
@@ -6722,17 +6722,17 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t/>
+          <t>0</t>
         </is>
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>OWNED_NO_NEW_PURCHASE</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
         <is>
-          <t>Shared M1 input; calibration before blade operation.</t>
+          <t>Do not assume advertised43A continuous.</t>
         </is>
       </c>
     </row>
@@ -6744,17 +6744,17 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>EL-BTS</t>
+          <t>EL-DRV</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Existing BTS7960 modules</t>
+          <t>Pololu2995 M1 driver option</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -6764,12 +6764,12 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>OWNED_UNQUALIFIED</t>
+          <t>OPTION_NOT_PURCHASED</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>PPR_project_handover_2026-09-20.zip / 08_BOM_COMPONENTS.md</t>
+          <t>https://www.pololu.com/product/2995</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
@@ -6779,17 +6779,17 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>0</t>
+          <t/>
         </is>
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>OWNED_NO_NEW_PURCHASE</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
         <is>
-          <t>Do not assume advertised43A continuous.</t>
+          <t>Configurable current limit; board21A is not terminal43A. Existing BTS7960 requires qualification.</t>
         </is>
       </c>
     </row>
@@ -6801,17 +6801,17 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>EL-DRV</t>
+          <t>EL-TC</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Pololu2995 M1 driver option</t>
+          <t>Adafruit3263 MAX31856</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
@@ -6821,12 +6821,12 @@
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>OPTION_NOT_PURCHASED</t>
+          <t>PURCHASE_CANDIDATE</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>https://www.pololu.com/product/2995</t>
+          <t>https://www.adafruit.com/product/3263</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
@@ -6846,7 +6846,7 @@
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>Configurable current limit; board21A is not terminal43A. Existing BTS7960 requires qualification.</t>
+          <t>Four independent temperature inputs; K probes exact mechanical model unresolved.</t>
         </is>
       </c>
     </row>
@@ -6858,17 +6858,17 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>EL-TC</t>
+          <t>FASTENERS</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Adafruit3263 MAX31856</t>
+          <t>Brackets, metal supports,keys,shims,retainers</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -6878,12 +6878,12 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>PURCHASE_CANDIDATE</t>
+          <t>HARDWARE_SCHEDULE_HOLD</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>https://www.adafruit.com/product/3263</t>
+          <t>Supplier drawing / capacity confirmation required before procurement</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
@@ -6903,7 +6903,7 @@
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>Four independent temperature inputs; K probes exact mechanical model unresolved.</t>
+          <t>Not an orderable quantity list; full mechanical fastener closure is outstanding.</t>
         </is>
       </c>
     </row>
@@ -6915,12 +6915,12 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>FASTENERS</t>
+          <t>FEED-CHUTE</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Brackets, metal supports,keys,shims,retainers</t>
+          <t>Metal lined transfer chute</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -6935,12 +6935,12 @@
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>HARDWARE_SCHEDULE_HOLD</t>
+          <t>TRANSFER_PATH_HOLD</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>Supplier drawing / capacity confirmation required before procurement</t>
+          <t>PPR-C1 original dimensional design; not an empirical qualification</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
@@ -6960,7 +6960,7 @@
       </c>
       <c r="K122" t="inlineStr">
         <is>
-          <t>Not an orderable quantity list; full mechanical fastener closure is outstanding.</t>
+          <t>Complete swept envelope/bridging check and split-print panels before release.</t>
         </is>
       </c>
     </row>
@@ -6972,12 +6972,12 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>FEED-CHUTE</t>
+          <t>GUARDS</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Metal lined transfer chute</t>
+          <t>Steel cutter containment / chain guards / heat shield</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -6992,7 +6992,7 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>TRANSFER_PATH_HOLD</t>
+          <t>SAFETY_GEOMETRY_HOLD</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
@@ -7017,7 +7017,7 @@
       </c>
       <c r="K123" t="inlineStr">
         <is>
-          <t>Complete swept envelope/bridging check and split-print panels before release.</t>
+          <t>Do not operate the open review assembly. Guard geometry still to be detailed.</t>
         </is>
       </c>
     </row>
@@ -7029,12 +7029,12 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>GUARDS</t>
+          <t>SAFE-BRAKE</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Steel cutter containment / chain guards / heat shield</t>
+          <t>Bus overvoltage/braking protection</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -7049,12 +7049,12 @@
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>SAFETY_GEOMETRY_HOLD</t>
+          <t>REGEN_DESIGN_HOLD</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>PPR-C1 original dimensional design; not an empirical qualification</t>
+          <t>Supplier drawing / capacity confirmation required before procurement</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
@@ -7074,7 +7074,7 @@
       </c>
       <c r="K124" t="inlineStr">
         <is>
-          <t>Do not operate the open review assembly. Guard geometry still to be detailed.</t>
+          <t>PSU sink ability unknown; no regeneration assumption.</t>
         </is>
       </c>
     </row>
@@ -7086,12 +7086,12 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>SAFE-BRAKE</t>
+          <t>SAFE-CONTACT</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Bus overvoltage/braking protection</t>
+          <t>24V coil DC rated contactor</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -7106,7 +7106,7 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>REGEN_DESIGN_HOLD</t>
+          <t>SAFETY_SELECTION_HOLD</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
@@ -7131,7 +7131,7 @@
       </c>
       <c r="K125" t="inlineStr">
         <is>
-          <t>PSU sink ability unknown; no regeneration assumption.</t>
+          <t>Continuous&gt;=35A DC and fault-current breaking coordinated with fuse.</t>
         </is>
       </c>
     </row>
@@ -7143,12 +7143,12 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>SAFE-CONTACT</t>
+          <t>SAFE-FUSE</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>24V coil DC rated contactor</t>
+          <t>Branch and mains fuses / holders</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -7163,7 +7163,7 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>SAFETY_SELECTION_HOLD</t>
+          <t>CIRCUIT_DESIGN_HOLD</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
@@ -7188,7 +7188,7 @@
       </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>Continuous&gt;=35A DC and fault-current breaking coordinated with fuse.</t>
+          <t>Select from actual cable ampacity, DC breaking and inrush. No guessed fuse order.</t>
         </is>
       </c>
     </row>
@@ -7200,17 +7200,17 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>SAFE-FUSE</t>
+          <t>SAFE-LOCK</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Branch and mains fuses / holders</t>
+          <t>Coded/positive-opening guard lock</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
@@ -7220,7 +7220,7 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>CIRCUIT_DESIGN_HOLD</t>
+          <t>SAFETY_SELECTION_HOLD</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
@@ -7245,7 +7245,7 @@
       </c>
       <c r="K127" t="inlineStr">
         <is>
-          <t>Select from actual cable ampacity, DC breaking and inrush. No guessed fuse order.</t>
+          <t>Lid and service access, standstill unlock, manual reset.</t>
         </is>
       </c>
     </row>
@@ -7257,17 +7257,17 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>SAFE-LOCK</t>
+          <t>SAFE-STOP</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Coded/positive-opening guard lock</t>
+          <t>Existing E-stop</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
@@ -7277,12 +7277,12 @@
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>SAFETY_SELECTION_HOLD</t>
+          <t>OWNED_RATING_VERIFY</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>Supplier drawing / capacity confirmation required before procurement</t>
+          <t>PPR_project_handover_2026-09-20.zip / 08_BOM_COMPONENTS.md</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
@@ -7292,17 +7292,17 @@
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t/>
+          <t>0</t>
         </is>
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>OWNED_NO_NEW_PURCHASE</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t>Lid and service access, standstill unlock, manual reset.</t>
+          <t>Independent hard cut with contactor; contact configuration verify.</t>
         </is>
       </c>
     </row>
@@ -7314,12 +7314,12 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>SAFE-STOP</t>
+          <t>SAFE-THERM</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Existing E-stop</t>
+          <t>Independent thermal cutoff chain</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -7334,12 +7334,12 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>OWNED_RATING_VERIFY</t>
+          <t>SAFETY_SELECTION_HOLD</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>PPR_project_handover_2026-09-20.zip / 08_BOM_COMPONENTS.md</t>
+          <t>Supplier drawing / capacity confirmation required before procurement</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
@@ -7349,34 +7349,34 @@
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>0</t>
+          <t/>
         </is>
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>OWNED_NO_NEW_PURCHASE</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
         <is>
-          <t>Independent hard cut with contactor; contact configuration verify.</t>
+          <t>Normally closed manual-reset overtemp plus one-shot protection.</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>system_requirement</t>
+          <t>vp1_stage1_3</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>SAFE-THERM</t>
+          <t>AUG_BEARINGS</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Independent thermal cutoff chain</t>
+          <t>west split pillow plus east journal cradle for the r3 auger shaft</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -7386,22 +7386,22 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Procurement requirement</t>
+          <t>steel plate 5 mm</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>SAFETY_SELECTION_HOLD</t>
+          <t>TRANSFER_UNRATED</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>Supplier drawing / capacity confirmation required before procurement</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>C1_INTERFACE_BASELINE</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -7411,12 +7411,12 @@
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>UNQUOTED_NOT_ZERO</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>Normally closed manual-reset overtemp plus one-shot protection.</t>
+          <t>Auger shaft supported at both ends - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -7428,12 +7428,12 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>AUG_BEARINGS</t>
+          <t>AUG_SHAFT</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>west split pillow plus east journal cradle for the r3 auger shaft</t>
+          <t>active auger conveyor: r3 shaft x236..370 at y232/z347.1; RH flight root r3/OD r8, pitch 28.5, four turns x238.5..352.5 with 3 mm swept face; U-shell bore r9.5, nominal BRep gap 1.085 mm</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -7443,7 +7443,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>steel plate 5 mm</t>
+          <t>steel shaft + steel flight</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -7473,7 +7473,7 @@
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>Auger shaft supported at both ends - UNQUOTED</t>
+          <t>Conveys +x at -5.4375 rpm for 58 rpm reference M1 via 15/40 gear and 24/12 chain B plus 8:1 worm/wheel; tolerance/runout/heat stack assumed not proven</t>
         </is>
       </c>
     </row>
@@ -7485,12 +7485,12 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>AUG_SHAFT</t>
+          <t>AUG_WHEEL</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>active auger conveyor: r3 shaft x236..370 at y232/z347.1; RH flight root r3/OD r8, pitch 28.5, four turns x238.5..352.5 with 3 mm swept face; U-shell bore r9.5, nominal BRep gap 1.085 mm</t>
+          <t>16T worm wheel (REFERENCE geometry, unrated), face x359..365, sector web, teeth cut by discrete hobbing of the worm; keyed Ø6 auger bore</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -7500,12 +7500,12 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>steel shaft + steel flight</t>
+          <t>steel (reference)</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>TRANSFER_UNRATED</t>
+          <t>REFERENCE_UNRATED</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
@@ -7530,7 +7530,7 @@
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>Conveys +x at -5.4375 rpm for 58 rpm reference M1 via 15/40 gear and 24/12 chain B plus 8:1 worm/wheel; tolerance/runout/heat stack assumed not proven</t>
+          <t>Matched 1.8 mm key and keyway transfer torque to AUG_SHAFT; tooth strength and wear unqualified - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -7542,12 +7542,12 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>AUG_WHEEL</t>
+          <t>CHUTE_BODY</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>16T worm wheel (REFERENCE geometry, unrated), face x359..365, sector web, teeth cut by discrete hobbing of the worm; keyed Ø6 auger bore</t>
+          <t>welded S1-&gt;S2 transfer chute with sealed pan, active screw-conveyor trough and east fallaway</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -7557,24 +7557,24 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>steel (reference)</t>
+          <t>steel sheet 3 mm + formed trough</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>REFERENCE_UNRATED</t>
+          <t>TRANSFER_UNRATED</t>
         </is>
       </c>
       <c r="G133" t="inlineStr">
         <is>
+          <t>VP1-ADR-002</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
           <t>VP1-STAGE5</t>
         </is>
       </c>
-      <c r="H133" t="inlineStr">
-        <is>
-          <t>VP1-STAGE5</t>
-        </is>
-      </c>
       <c r="I133" t="inlineStr">
         <is>
           <t/>
@@ -7587,7 +7587,7 @@
       </c>
       <c r="K133" t="inlineStr">
         <is>
-          <t>Matched 1.8 mm key and keyway transfer torque to AUG_SHAFT; tooth strength and wear unqualified - UNQUOTED</t>
+          <t>BRep geometry and digital flow only; material transport and containment are not physically qualified - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -7599,12 +7599,12 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>CHUTE_BODY</t>
+          <t>CHUTE_TROUGH_FLOOR_E</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>welded S1-&gt;S2 transfer chute with sealed pan, active screw-conveyor trough and east fallaway</t>
+          <t>bolted trough ledge section over the S2 mouth</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -7614,12 +7614,12 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>steel sheet 3 mm + formed trough</t>
+          <t>steel sheet 3 mm</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>TRANSFER_UNRATED</t>
+          <t>GEOMETRY_PASS</t>
         </is>
       </c>
       <c r="G134" t="inlineStr">
@@ -7629,7 +7629,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>VP1-STAGE2</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -7644,7 +7644,7 @@
       </c>
       <c r="K134" t="inlineStr">
         <is>
-          <t>BRep geometry and digital flow only; material transport and containment are not physically qualified - UNQUOTED</t>
+          <t>Clearance-cut for the frozen saddle jacket - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -7656,12 +7656,12 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>CHUTE_TROUGH_FLOOR_E</t>
+          <t>CROSS_FEED_BEARINGS</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>bolted trough ledge section over the S2 mouth</t>
+          <t>paired cross-feed and idler journal support with structural rails</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -7671,22 +7671,22 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>steel sheet 3 mm</t>
+          <t>steel plate and journal shells</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>GEOMETRY_PASS</t>
+          <t>TRANSFER_UNRATED</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>VP1-ADR-002</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -7701,7 +7701,7 @@
       </c>
       <c r="K135" t="inlineStr">
         <is>
-          <t>Clearance-cut for the frozen saddle jacket - UNQUOTED</t>
+          <t>BRep-supported reference geometry; wear and load unqualified - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -7713,12 +7713,12 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>CROSS_FEED_BEARINGS</t>
+          <t>CROSS_FEED_GEAR</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>paired cross-feed and idler journal support with structural rails</t>
+          <t>12T keyed output gear on transverse feed shaft</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -7728,7 +7728,7 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>steel plate and journal shells</t>
+          <t>steel reference gear</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
@@ -7758,7 +7758,7 @@
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>BRep-supported reference geometry; wear and load unqualified - UNQUOTED</t>
+          <t>1:1 from PDL through idler; tooth contact and torque rating unqualified - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -7770,12 +7770,12 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>CROSS_FEED_GEAR</t>
+          <t>CROSS_FEED_IDLER</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>12T keyed output gear on transverse feed shaft</t>
+          <t>12T integral idler and supported journal between PDL and transverse feed gears</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -7785,7 +7785,7 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>steel reference gear</t>
+          <t>steel reference gear and shaft</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
@@ -7815,7 +7815,7 @@
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>1:1 from PDL through idler; tooth contact and torque rating unqualified - UNQUOTED</t>
+          <t>Two external meshes preserve rotation sign; journal rating unqualified - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -7827,12 +7827,12 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>CROSS_FEED_IDLER</t>
+          <t>CROSS_FEED_SHAFT</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>12T integral idler and supported journal between PDL and transverse feed gears</t>
+          <t>RH helical screw on y-axis x357/z328 with 9 mm pitch; reduced-radius powered tail to y260.5</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -7842,7 +7842,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>steel reference gear and shaft</t>
+          <t>steel shaft and welded flight</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
@@ -7872,7 +7872,7 @@
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>Two external meshes preserve rotation sign; journal rating unqualified - UNQUOTED</t>
+          <t>Powered tail overlaps S2 mouth y255 by 5.502 mm; actual fragment handoff unproven - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -7884,12 +7884,12 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>CROSS_FEED_SHAFT</t>
+          <t>CROSS_FEED_SHELL</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>RH helical screw on y-axis x357/z328 with 9 mm pitch; reduced-radius powered tail to y260.5</t>
+          <t>U cradle with rotor-relieved outer metal shelf past S2 mouth</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -7899,7 +7899,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>steel shaft and welded flight</t>
+          <t>formed steel sheet</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
@@ -7929,7 +7929,7 @@
       </c>
       <c r="K139" t="inlineStr">
         <is>
-          <t>Powered tail overlaps S2 mouth y255 by 5.502 mm; actual fragment handoff unproven - UNQUOTED</t>
+          <t>Outer shelf y255..258 supports the handoff without entering swept rotor sector; material transfer unproven - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -7941,12 +7941,12 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>CROSS_FEED_SHELL</t>
+          <t>DRV-CHAIN-A</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>U cradle with rotor-relieved outer metal shelf past S2 mouth</t>
+          <t>#35 roller chain cut to 896 mm (94 links; chain A: jackshaft 24T -&gt; S1 shaft A 24T)</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -7956,22 +7956,22 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>formed steel sheet</t>
+          <t>ANSI35 steel roller chain p=9.525</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>TRANSFER_UNRATED</t>
+          <t>PROCUREMENT_HOLD</t>
         </is>
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>VP1-ADR-002</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>VP1-STAGE1</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -7986,7 +7986,7 @@
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>Outer shelf y255..258 supports the handoff without entering swept rotor sector; material transfer unproven - UNQUOTED</t>
+          <t>Cut length from tangent+pitch-arc geometry (drive_geometry.json chain_lengths.A=896.0). UNQUOTED: not 0 - the 100000 KRW soft limit applies to quoted lines only</t>
         </is>
       </c>
     </row>
@@ -7998,12 +7998,12 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>DRV-CHAIN-A</t>
+          <t>DRV-CHAIN-B</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>#35 roller chain cut to 896 mm (94 links; chain A: jackshaft 24T -&gt; S1 shaft A 24T)</t>
+          <t>#35 roller chain cut to 724 mm (76 links; chain B: jackshaft 24T -&gt; S2 12T, ADR-002 rev B)</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -8028,7 +8028,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>VP1-STAGE1</t>
+          <t>VP1-STAGE4</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -8043,7 +8043,7 @@
       </c>
       <c r="K141" t="inlineStr">
         <is>
-          <t>Cut length from tangent+pitch-arc geometry (drive_geometry.json chain_lengths.A=896.0). UNQUOTED: not 0 - the 100000 KRW soft limit applies to quoted lines only</t>
+          <t>Cut length from tangent+pitch-arc geometry (chain_lengths.B=723.9). UNQUOTED: not 0</t>
         </is>
       </c>
     </row>
@@ -8055,12 +8055,12 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>DRV-CHAIN-B</t>
+          <t>EL_CONTACTOR</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>#35 roller chain cut to 724 mm (76 links; chain B: jackshaft 24T -&gt; S2 12T, ADR-002 rev B)</t>
+          <t>safety contactor</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -8070,22 +8070,22 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>ANSI35 steel roller chain p=9.525</t>
+          <t>24 V coil contactor MPN unselected</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>PROCUREMENT_HOLD</t>
+          <t>SAFETY_HARDWARE_REQUIRED</t>
         </is>
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>VP1-ADR-002</t>
+          <t>VP1-STAGE3</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>VP1-STAGE4</t>
+          <t>VP1-STAGE3</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -8100,7 +8100,7 @@
       </c>
       <c r="K142" t="inlineStr">
         <is>
-          <t>Cut length from tangent+pitch-arc geometry (chain_lengths.B=723.9). UNQUOTED: not 0</t>
+          <t>UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -8112,12 +8112,12 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>EL_CONTACTOR</t>
+          <t>EL_CURRENT_LIMITER</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>safety contactor</t>
+          <t>heater sequencer / current-limit relay bank</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -8127,22 +8127,22 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>24 V coil contactor MPN unselected</t>
+          <t>relay bank MPN unselected</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>SAFETY_HARDWARE_REQUIRED</t>
+          <t>CONTROL_REFERENCE_UNRATED</t>
         </is>
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-STAGE4</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-STAGE4</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -8157,7 +8157,7 @@
       </c>
       <c r="K143" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>Host-tested firmware excludes simultaneous heater bands and rejects demand above 792 W; independent electrical interlock and component ratings still required - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -8169,12 +8169,12 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>EL_CURRENT_LIMITER</t>
+          <t>EL_DIN_RAIL</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>heater sequencer / current-limit relay bank</t>
+          <t>DIN rail 35 mm top-hat x 210</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -8184,22 +8184,22 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>relay bank MPN unselected</t>
+          <t>steel rail</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>CONTROL_REFERENCE_UNRATED</t>
+          <t>PROCUREMENT_HOLD</t>
         </is>
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>VP1-STAGE4</t>
+          <t>VP1-STAGE3</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>VP1-STAGE4</t>
+          <t>VP1-STAGE3</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -8214,7 +8214,7 @@
       </c>
       <c r="K144" t="inlineStr">
         <is>
-          <t>Host-tested firmware excludes simultaneous heater bands and rejects demand above 792 W; independent electrical interlock and component ratings still required - UNQUOTED</t>
+          <t>UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -8226,12 +8226,12 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>EL_DIN_RAIL</t>
+          <t>EL_DRIVER_1</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>DIN rail 35 mm top-hat x 210</t>
+          <t>stepper/BLDC driver (M1 branch)</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -8241,12 +8241,12 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>steel rail</t>
+          <t>24 V driver MPN unselected</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>PROCUREMENT_HOLD</t>
+          <t>MOTOR_UNSELECTED</t>
         </is>
       </c>
       <c r="G145" t="inlineStr">
@@ -8283,12 +8283,12 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>EL_DRIVER_1</t>
+          <t>EL_DRIVER_2</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>stepper/BLDC driver (M1 branch)</t>
+          <t>stepper/BLDC driver (M2 branch)</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -8340,12 +8340,12 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>EL_DRIVER_2</t>
+          <t>EL_DRIVER_3</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>stepper/BLDC driver (M2 branch)</t>
+          <t>stepper/BLDC driver (winder/puller accessory)</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -8397,12 +8397,12 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>EL_DRIVER_3</t>
+          <t>EL_ESTOP_BOX</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>stepper/BLDC driver (winder/puller accessory)</t>
+          <t>dual-channel E-stop / lid / service interlock relay box</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -8412,12 +8412,12 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>24 V driver MPN unselected</t>
+          <t>relay box MPN unselected</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>MOTOR_UNSELECTED</t>
+          <t>SAFETY_HARDWARE_REQUIRED</t>
         </is>
       </c>
       <c r="G148" t="inlineStr">
@@ -8454,12 +8454,12 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>EL_ESTOP_BOX</t>
+          <t>EL_OVERTEMP_BOX</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>dual-channel E-stop / lid / service interlock relay box</t>
+          <t>manual-reset independent overtemperature relay box</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -8511,12 +8511,12 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>EL_OVERTEMP_BOX</t>
+          <t>EL_WIRE_DUCT</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>manual-reset independent overtemperature relay box</t>
+          <t>slotted wiring duct x 210</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -8526,12 +8526,12 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>relay box MPN unselected</t>
+          <t>PVC duct</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>SAFETY_HARDWARE_REQUIRED</t>
+          <t>PROCUREMENT_HOLD</t>
         </is>
       </c>
       <c r="G150" t="inlineStr">
@@ -8568,12 +8568,12 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>EL_WIRE_DUCT</t>
+          <t>GUARD_CHAIN_A</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>slotted wiring duct x 210</t>
+          <t>chain A top-run lid plate</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -8583,17 +8583,17 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>PVC duct</t>
+          <t>steel plate 3 mm</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>PROCUREMENT_HOLD</t>
+          <t>CONTAINMENT_UNRATED</t>
         </is>
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-STAGE2</t>
         </is>
       </c>
       <c r="H151" t="inlineStr">
@@ -8625,12 +8625,12 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>GUARD_CHAIN_A</t>
+          <t>GUARD_CHAIN_B</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>chain A top-run lid plate</t>
+          <t>chain B outer guard plate set (continuous; ADR-002 rev B re-route)</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
@@ -8682,12 +8682,12 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>GUARD_CHAIN_B</t>
+          <t>GUARD_LID_INTERLOCK_SEAT</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>chain B outer guard plate set (continuous; ADR-002 rev B re-route)</t>
+          <t>hopper-lid interlock switch seat</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
@@ -8739,12 +8739,12 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>GUARD_LID_INTERLOCK_SEAT</t>
+          <t>GUARD_S2_RING</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>hopper-lid interlock switch seat</t>
+          <t>S2 rotor ring guard (annular sector r 90..94 over 20..114 deg)</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -8784,7 +8784,7 @@
       </c>
       <c r="K154" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>Guard plate thickness unrated; service sweep verified - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -8796,37 +8796,37 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>GUARD_S2_RING</t>
+          <t>HOPPER_FASTENER_M3</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>S2 rotor ring guard (annular sector r 90..94 over 20..114 deg)</t>
+          <t>M3 x 12 through-bolt with low-profile head for PC panel to captive steel seam boss</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>steel plate 3 mm</t>
+          <t>steel metric fastener</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>CONTAINMENT_UNRATED</t>
+          <t>FASTENER_ENVELOPE_HOLD</t>
         </is>
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-HOPPER-SPLIT</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-HOPPER-GEOMETRY</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
@@ -8841,7 +8841,7 @@
       </c>
       <c r="K155" t="inlineStr">
         <is>
-          <t>Guard plate thickness unrated; service sweep verified - UNQUOTED</t>
+          <t>M3 clearance holes and captive bosses are modeled; bolts/heads not modeled or selected. Head bearing/seal outside taper and torque/preload must be qualified before fabrication; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -8853,12 +8853,12 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>PDL_BEARINGS</t>
+          <t>HOPPER_PANEL_L</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>two split pillow posts carrying the worm shaft at x353..365, y204..210/352..358</t>
+          <t>C1 HOPPER.step PC loft cut at world x120, left half with front/rear M3 through-holes</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -8868,22 +8868,22 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>steel plate 5 mm</t>
+          <t>polycarbonate FDM shell nominal 3 mm</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>TRANSFER_UNRATED</t>
+          <t>PRINT_DFM_LINER_HOLD</t>
         </is>
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>VP1-HOPPER-SPLIT</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>VP1-HOPPER-GEOMETRY</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -8898,7 +8898,7 @@
       </c>
       <c r="K156" t="inlineStr">
         <is>
-          <t>Mounted on the support-plate bosses - UNQUOTED</t>
+          <t>Actual CAD bbox 119.258 x 162.2 x 55.497 mm; print orientation/adhesion/infill and assembled joint strength unqualified; historical HOPPER_001 removed from active quantity; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -8910,12 +8910,12 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>PDL_CHAIN</t>
+          <t>HOPPER_PANEL_R</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>#35 roller chain, 35 links incl. offset link; S2 12T second band to PDL_SPROCKET at x362, 1:1</t>
+          <t>C1 HOPPER.step PC loft cut at world x120, right half with front/rear M3 through-holes</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -8925,22 +8925,22 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>ANSI35 steel roller chain p=9.525</t>
+          <t>polycarbonate FDM shell nominal 3 mm</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>TRANSFER_UNRATED</t>
+          <t>PRINT_DFM_LINER_HOLD</t>
         </is>
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>VP1-HOPPER-SPLIT</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>VP1-HOPPER-GEOMETRY</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -8955,7 +8955,7 @@
       </c>
       <c r="K157" t="inlineStr">
         <is>
-          <t>Nominal333.375 mm versus geometric332.734 mm; 0.641 mm length surplus. Offset-link strength and tension adjustment unqualified; no quote - UNQUOTED</t>
+          <t>Actual CAD bbox 117 x 162.2 x 55.497 mm; print orientation/adhesion/infill and assembled joint strength unqualified; historical HOPPER_001 removed from active quantity; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -8967,12 +8967,12 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>PDL_FEED_GEAR</t>
+          <t>HOPPER_SEAM_FRONT</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>12T keyed spur on worm shaft feeding orthogonal screw train</t>
+          <t>40 x 39 x 1.5 mm sloping steel upper front seam strap with four M3 clearance holes and integral captive hex bosses</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -8982,22 +8982,22 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>steel reference gear</t>
+          <t>steel strip and welded captive bosses</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>TRANSFER_UNRATED</t>
+          <t>SEAM_AND_LINER_HOLD</t>
         </is>
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>VP1-HOPPER-SPLIT</t>
         </is>
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>VP1-HOPPER-GEOMETRY</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -9012,7 +9012,7 @@
       </c>
       <c r="K158" t="inlineStr">
         <is>
-          <t>Tooth strength and keyed fit unqualified - UNQUOTED</t>
+          <t>Wall-face support z456..495 across x120 split; not the C1 unmodeled lower steel safety liner; weld and bolt loads unqualified; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -9024,12 +9024,12 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>PDL_SHAFT</t>
+          <t>HOPPER_SEAM_REAR</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>trough worm shaft dia 10 x 188 (r5, y204..392, x362, z374.5), dia 12 keyed chain shoulder y376..392</t>
+          <t>40 x 39 x 1.5 mm sloping steel upper rear seam strap with four M3 clearance holes and integral captive hex bosses</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -9039,22 +9039,22 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>steel rod C45 candidate</t>
+          <t>steel strip and welded captive bosses</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>TRANSFER_UNRATED</t>
+          <t>SEAM_AND_LINER_HOLD</t>
         </is>
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>VP1-HOPPER-SPLIT</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>VP1-HOPPER-GEOMETRY</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -9069,7 +9069,7 @@
       </c>
       <c r="K159" t="inlineStr">
         <is>
-          <t>Carries the RH 2-start worm; keyed 12T sprocket takes 1:1 PDL_CHAIN drive from the S2 12T sprocket - UNQUOTED</t>
+          <t>Wall-face support z456..495 across x120 split; not the C1 unmodeled lower steel safety liner; weld and bolt loads unqualified; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -9081,12 +9081,12 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>PDL_SPROCKET</t>
+          <t>PDL_BEARINGS</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>worm-shaft drive sprocket 12T bore 12 mm with keyed hub on shaft shoulder</t>
+          <t>two split pillow posts carrying the worm shaft at x353..365, y204..210/352..358</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
@@ -9096,7 +9096,7 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>ANSI35 steel sprocket</t>
+          <t>steel plate 5 mm</t>
         </is>
       </c>
       <c r="F160" t="inlineStr">
@@ -9126,7 +9126,7 @@
       </c>
       <c r="K160" t="inlineStr">
         <is>
-          <t>Bore r6 on y376..392 shaft shoulder r6 with 1.8 mm key in matched slot; torque fit and chain rating UNRATED - UNQUOTED</t>
+          <t>Mounted on the support-plate bosses - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -9138,12 +9138,12 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>PDL_WORM</t>
+          <t>PDL_CHAIN</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>RH 2-start worm (REFERENCE geometry, unrated): root r6/pitch r6.75/OD r7.5, lead angle 23.3 deg, length 20 (y220..240), keyed Ø10 shaft bore</t>
+          <t>#35 roller chain, 35 links incl. offset link; S2 12T second band to PDL_SPROCKET at x362, 1:1</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -9153,12 +9153,12 @@
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>steel (reference)</t>
+          <t>ANSI35 steel roller chain p=9.525</t>
         </is>
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>REFERENCE_UNRATED</t>
+          <t>TRANSFER_UNRATED</t>
         </is>
       </c>
       <c r="G161" t="inlineStr">
@@ -9183,7 +9183,7 @@
       </c>
       <c r="K161" t="inlineStr">
         <is>
-          <t>Matched 1.8 mm key and keyway transfer torque from PDL_SHAFT; tooth mesh and loads remain unrated - UNQUOTED</t>
+          <t>Nominal333.375 mm versus geometric332.734 mm; 0.641 mm length surplus. Offset-link strength and tension adjustment unqualified; no quote - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -9195,12 +9195,12 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>PULL_FRAME</t>
+          <t>PDL_FEED_GEAR</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>puller side plates + base + fixed-roller bearing seats + carriage guide slots</t>
+          <t>12T keyed spur on worm shaft feeding orthogonal screw train</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -9210,22 +9210,22 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>steel plate 5 mm + 3 mm</t>
+          <t>steel reference gear</t>
         </is>
       </c>
       <c r="F162" t="inlineStr">
         <is>
-          <t>NIP_RATING_HOLD</t>
+          <t>TRANSFER_UNRATED</t>
         </is>
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>VP1-STAGE4</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>VP1-STAGE4</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -9240,7 +9240,7 @@
       </c>
       <c r="K162" t="inlineStr">
         <is>
-          <t>Positive stop 1.5 mm and adjustable open nip to 3.0 mm; spring carriage grips nominal 1.75 mm filament - UNQUOTED</t>
+          <t>Tooth strength and keyed fit unqualified - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -9252,12 +9252,12 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>PULL_MOTOR_REF</t>
+          <t>PDL_SHAFT</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>puller gearmotor reference (not selected)</t>
+          <t>trough worm shaft dia 10 x 188 (r5, y204..392, x362, z374.5), dia 12 keyed chain shoulder y376..392</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
@@ -9267,22 +9267,22 @@
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>24 V gearmotor MPN unselected</t>
+          <t>steel rod C45 candidate</t>
         </is>
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>MOTOR_UNSELECTED</t>
+          <t>TRANSFER_UNRATED</t>
         </is>
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
@@ -9297,7 +9297,7 @@
       </c>
       <c r="K163" t="inlineStr">
         <is>
-          <t>UNQUOTED; known motor floors exceed the 100000 KRW soft limit - not 0</t>
+          <t>Carries the RH 2-start worm; keyed 12T sprocket takes 1:1 PDL_CHAIN drive from the S2 12T sprocket - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -9309,12 +9309,12 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>PULL_NIP_STOP</t>
+          <t>PDL_SPROCKET</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>nip positive-stop cam block (1.5 mm minimum, 3.0 mm open)</t>
+          <t>worm-shaft drive sprocket 12T bore 12 mm with keyed hub on shaft shoulder</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
@@ -9324,22 +9324,22 @@
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>steel</t>
+          <t>ANSI35 steel sprocket</t>
         </is>
       </c>
       <c r="F164" t="inlineStr">
         <is>
-          <t>NIP_RATING_HOLD</t>
+          <t>TRANSFER_UNRATED</t>
         </is>
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
@@ -9354,7 +9354,7 @@
       </c>
       <c r="K164" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>Bore r6 on y376..392 shaft shoulder r6 with 1.8 mm key in matched slot; torque fit and chain rating UNRATED - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -9366,12 +9366,12 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>PULL_ROLLER_ADJ</t>
+          <t>PDL_WORM</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>puller adjustable roller dia 20 + spring-loaded carriage (guide posts, coil springs, cam stop)</t>
+          <t>RH 2-start worm (REFERENCE geometry, unrated): root r6/pitch r6.75/OD r7.5, lead angle 23.3 deg, length 20 (y220..240), keyed Ø10 shaft bore</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
@@ -9381,22 +9381,22 @@
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>steel; M5 screw</t>
+          <t>steel (reference)</t>
         </is>
       </c>
       <c r="F165" t="inlineStr">
         <is>
-          <t>NIP_RATING_HOLD</t>
+          <t>REFERENCE_UNRATED</t>
         </is>
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
@@ -9411,7 +9411,7 @@
       </c>
       <c r="K165" t="inlineStr">
         <is>
-          <t>Spring-loaded carrier grips 1.5-2.0 mm filament (1.75 nominal, design/parameters.json filament_mm); cam stop range 1.5..3.0 mm - UNQUOTED</t>
+          <t>Matched 1.8 mm key and keyway transfer torque from PDL_SHAFT; tooth mesh and loads remain unrated - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -9423,12 +9423,12 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>PULL_ROLLER_FIXED</t>
+          <t>PULL_FRAME</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>puller drive roller dia 20 x 22</t>
+          <t>puller side plates + base + fixed-roller bearing seats + carriage guide slots</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
@@ -9438,7 +9438,7 @@
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>steel; knurl or rubber per TPU grip</t>
+          <t>steel plate 5 mm + 3 mm</t>
         </is>
       </c>
       <c r="F166" t="inlineStr">
@@ -9448,12 +9448,12 @@
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-STAGE4</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-STAGE4</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
@@ -9468,7 +9468,7 @@
       </c>
       <c r="K166" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>Positive stop 1.5 mm and adjustable open nip to 3.0 mm; spring carriage grips nominal 1.75 mm filament - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -9480,37 +9480,37 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>S1_BELT</t>
+          <t>PULL_MOTOR_REF</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>two side-loop treads over x80..219; y163.5..223.2 and 240.8..323.5</t>
+          <t>puller gearmotor reference (not selected)</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>polymer belt with steel-supported drums</t>
+          <t>24 V gearmotor MPN unselected</t>
         </is>
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>TRANSFER_UNRATED</t>
+          <t>MOTOR_UNSELECTED</t>
         </is>
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>VP1-STAGE2</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>VP1-STAGE3</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -9525,7 +9525,7 @@
       </c>
       <c r="K167" t="inlineStr">
         <is>
-          <t>Friction and tension unrated; UNQUOTED</t>
+          <t>UNQUOTED; known motor floors exceed the 100000 KRW soft limit - not 0</t>
         </is>
       </c>
     </row>
@@ -9537,12 +9537,12 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>S1_BELT_BEARINGS</t>
+          <t>PULL_NIP_STOP</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>four belt shaft support rings in the side rails</t>
+          <t>nip positive-stop cam block (1.5 mm minimum, 3.0 mm open)</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
@@ -9552,22 +9552,22 @@
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>steel bearing seats</t>
+          <t>steel</t>
         </is>
       </c>
       <c r="F168" t="inlineStr">
         <is>
-          <t>TRANSFER_UNRATED</t>
+          <t>NIP_RATING_HOLD</t>
         </is>
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>VP1-STAGE2</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>VP1-STAGE3</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
@@ -9582,7 +9582,7 @@
       </c>
       <c r="K168" t="inlineStr">
         <is>
-          <t>Bearing selection and loads unqualified; UNQUOTED</t>
+          <t>UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -9594,12 +9594,12 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>S1_BELT_CHAIN</t>
+          <t>PULL_ROLLER_ADJ</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>#35 chain from S1B 24T to west belt 12T</t>
+          <t>puller adjustable roller dia 20 + spring-loaded carriage (guide posts, coil springs, cam stop)</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
@@ -9609,22 +9609,22 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>ANSI35 steel chain</t>
+          <t>steel; M5 screw</t>
         </is>
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>TRANSFER_UNRATED</t>
+          <t>NIP_RATING_HOLD</t>
         </is>
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>VP1-STAGE2</t>
         </is>
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>VP1-STAGE3</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
@@ -9639,7 +9639,7 @@
       </c>
       <c r="K169" t="inlineStr">
         <is>
-          <t>Tension and strength unrated; UNQUOTED</t>
+          <t>Spring-loaded carrier grips 1.5-2.0 mm filament (1.75 nominal, design/parameters.json filament_mm); cam stop range 1.5..3.0 mm - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -9651,12 +9651,12 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>S1_BELT_DRIVE</t>
+          <t>PULL_ROLLER_FIXED</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>common waisted drive drum at x80; separate r3.8 side and r2.3 central tread seats</t>
+          <t>puller drive roller dia 20 x 22</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -9666,22 +9666,22 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>steel shaft and drums</t>
+          <t>steel; knurl or rubber per TPU grip</t>
         </is>
       </c>
       <c r="F170" t="inlineStr">
         <is>
-          <t>TRANSFER_UNRATED</t>
+          <t>NIP_RATING_HOLD</t>
         </is>
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>VP1-STAGE2</t>
         </is>
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>VP1-STAGE3</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
@@ -9696,7 +9696,7 @@
       </c>
       <c r="K170" t="inlineStr">
         <is>
-          <t>S1B chain-driven; torque and bearing load unrated; UNQUOTED</t>
+          <t>UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -9708,22 +9708,22 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>S1_BELT_FOLLOWER</t>
+          <t>S1_BELT</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>12T sprocket on the west belt driver</t>
+          <t>two side-loop treads over x80..219; y163.5..223.2 and 240.8..323.5</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>ANSI35 steel sprocket</t>
+          <t>polymer belt with steel-supported drums</t>
         </is>
       </c>
       <c r="F171" t="inlineStr">
@@ -9753,7 +9753,7 @@
       </c>
       <c r="K171" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>Friction and tension unrated; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -9765,12 +9765,12 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>S1_BELT_IDLER</t>
+          <t>S1_BELT_BEARINGS</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>two split side idler drums at x219 leaving the central transfer corridor open</t>
+          <t>four belt shaft support rings in the side rails</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
@@ -9780,7 +9780,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>steel journals and drums</t>
+          <t>steel bearing seats</t>
         </is>
       </c>
       <c r="F172" t="inlineStr">
@@ -9810,7 +9810,7 @@
       </c>
       <c r="K172" t="inlineStr">
         <is>
-          <t>Two independent journal halves; UNQUOTED</t>
+          <t>Bearing selection and loads unqualified; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -9822,12 +9822,12 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>S1_SWEEP_BEARINGS</t>
+          <t>S1_BELT_CHAIN</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>two separated sweep bearing rings in the pan rails</t>
+          <t>#35 chain from S1B 24T to west belt 12T</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
@@ -9837,7 +9837,7 @@
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>steel bearing seats</t>
+          <t>ANSI35 steel chain</t>
         </is>
       </c>
       <c r="F173" t="inlineStr">
@@ -9867,7 +9867,7 @@
       </c>
       <c r="K173" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>Tension and strength unrated; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -9879,12 +9879,12 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>S1_SWEEP_GEAR_DRUM_N</t>
+          <t>S1_BELT_DRIVE</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>12T gear on the north east belt idler</t>
+          <t>common waisted drive drum at x80; separate r3.8 side and r2.3 central tread seats</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
@@ -9894,7 +9894,7 @@
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>steel gear</t>
+          <t>steel shaft and drums</t>
         </is>
       </c>
       <c r="F174" t="inlineStr">
@@ -9924,7 +9924,7 @@
       </c>
       <c r="K174" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>S1B chain-driven; torque and bearing load unrated; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -9936,12 +9936,12 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>S1_SWEEP_GEAR_DRUM_S</t>
+          <t>S1_BELT_FOLLOWER</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>12T gear on the south east belt idler</t>
+          <t>12T sprocket on the west belt driver</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
@@ -9951,7 +9951,7 @@
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>steel gear</t>
+          <t>ANSI35 steel sprocket</t>
         </is>
       </c>
       <c r="F175" t="inlineStr">
@@ -9993,12 +9993,12 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>S1_SWEEP_GEAR_N</t>
+          <t>S1_BELT_IDLER</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>12T gear on the north sweep shaft</t>
+          <t>two split side idler drums at x219 leaving the central transfer corridor open</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -10008,7 +10008,7 @@
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>steel gear</t>
+          <t>steel journals and drums</t>
         </is>
       </c>
       <c r="F176" t="inlineStr">
@@ -10038,7 +10038,7 @@
       </c>
       <c r="K176" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>Two independent journal halves; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10050,12 +10050,12 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>S1_SWEEP_GEAR_S</t>
+          <t>S1_SWEEP_BEARINGS</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>12T gear on the south sweep shaft</t>
+          <t>two separated sweep bearing rings in the pan rails</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
@@ -10065,7 +10065,7 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>steel gear</t>
+          <t>steel bearing seats</t>
         </is>
       </c>
       <c r="F177" t="inlineStr">
@@ -10107,12 +10107,12 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>S1_SWEEP_NORTH</t>
+          <t>S1_SWEEP_GEAR_DRUM_N</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>north transverse screw x224 y235.5..359 feeding the central lane</t>
+          <t>12T gear on the north east belt idler</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
@@ -10122,7 +10122,7 @@
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>steel shaft and flight</t>
+          <t>steel gear</t>
         </is>
       </c>
       <c r="F178" t="inlineStr">
@@ -10152,7 +10152,7 @@
       </c>
       <c r="K178" t="inlineStr">
         <is>
-          <t>Dynamic side-belt pickup under verification; UNQUOTED</t>
+          <t>UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10164,12 +10164,12 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>S1_SWEEP_SOUTH</t>
+          <t>S1_SWEEP_GEAR_DRUM_S</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>south transverse screw x224 y127..228.5 feeding the central lane</t>
+          <t>12T gear on the south east belt idler</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
@@ -10179,7 +10179,7 @@
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>steel shaft and flight</t>
+          <t>steel gear</t>
         </is>
       </c>
       <c r="F179" t="inlineStr">
@@ -10209,7 +10209,7 @@
       </c>
       <c r="K179" t="inlineStr">
         <is>
-          <t>Dynamic side-belt pickup under verification; UNQUOTED</t>
+          <t>UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10221,12 +10221,12 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>S1_TRANSFER_BEARINGS</t>
+          <t>S1_SWEEP_GEAR_N</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>two central idler support rings</t>
+          <t>12T gear on the north sweep shaft</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
@@ -10236,7 +10236,7 @@
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>steel bearing seats</t>
+          <t>steel gear</t>
         </is>
       </c>
       <c r="F180" t="inlineStr">
@@ -10278,12 +10278,12 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>S1_TRANSFER_BELT</t>
+          <t>S1_SWEEP_GEAR_S</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>central 17 mm tread from x80 to x260 inside the two side loops</t>
+          <t>12T gear on the south sweep shaft</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
@@ -10293,7 +10293,7 @@
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>polymer belt</t>
+          <t>steel gear</t>
         </is>
       </c>
       <c r="F181" t="inlineStr">
@@ -10323,7 +10323,7 @@
       </c>
       <c r="K181" t="inlineStr">
         <is>
-          <t>Screw pickup unproven; UNQUOTED</t>
+          <t>UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10335,12 +10335,12 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>S1_TRANSFER_IDLER</t>
+          <t>S1_SWEEP_NORTH</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>central east r2.3 idler at x260</t>
+          <t>north transverse screw x224 y235.5..359 feeding the central lane</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
@@ -10350,7 +10350,7 @@
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>steel drum</t>
+          <t>steel shaft and flight</t>
         </is>
       </c>
       <c r="F182" t="inlineStr">
@@ -10380,7 +10380,7 @@
       </c>
       <c r="K182" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>Dynamic side-belt pickup under verification; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10392,12 +10392,12 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>WIND_FLANGE_L</t>
+          <t>S1_SWEEP_SOUTH</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>spool flange dia 200</t>
+          <t>south transverse screw x224 y127..228.5 feeding the central lane</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
@@ -10407,22 +10407,22 @@
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>steel plate 6 mm</t>
+          <t>steel shaft and flight</t>
         </is>
       </c>
       <c r="F183" t="inlineStr">
         <is>
-          <t>WINDER_UNRATED</t>
+          <t>TRANSFER_UNRATED</t>
         </is>
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
@@ -10437,7 +10437,7 @@
       </c>
       <c r="K183" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>Dynamic side-belt pickup under verification; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10449,12 +10449,12 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>WIND_FLANGE_R</t>
+          <t>S1_TRANSFER_BEARINGS</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>spool flange dia 200</t>
+          <t>two central idler support rings</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
@@ -10464,22 +10464,22 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>steel plate 6 mm</t>
+          <t>steel bearing seats</t>
         </is>
       </c>
       <c r="F184" t="inlineStr">
         <is>
-          <t>WINDER_UNRATED</t>
+          <t>TRANSFER_UNRATED</t>
         </is>
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
@@ -10506,12 +10506,12 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>WIND_MOTOR_REF</t>
+          <t>S1_TRANSFER_BELT</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>spool gearmotor reference (not selected)</t>
+          <t>central 17 mm tread from x80 to x260 inside the two side loops</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
@@ -10521,22 +10521,22 @@
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>24 V gearmotor MPN unselected</t>
+          <t>polymer belt</t>
         </is>
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t>MOTOR_UNSELECTED</t>
+          <t>TRANSFER_UNRATED</t>
         </is>
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
@@ -10551,7 +10551,7 @@
       </c>
       <c r="K185" t="inlineStr">
         <is>
-          <t>UNQUOTED; known motor floors exceed the 100000 KRW soft limit - not 0</t>
+          <t>Screw pickup unproven; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10563,12 +10563,12 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>WIND_SPOOL_BEARINGS</t>
+          <t>S1_TRANSFER_IDLER</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>spool shaft bearing blocks at BOTH shaft ends</t>
+          <t>central east r2.3 idler at x260</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
@@ -10578,22 +10578,22 @@
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>steel plate 5 mm + bearing seats</t>
+          <t>steel drum</t>
         </is>
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t>WINDER_UNRATED</t>
+          <t>TRANSFER_UNRATED</t>
         </is>
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>VP1-STAGE4</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>VP1-STAGE4</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
@@ -10608,7 +10608,7 @@
       </c>
       <c r="K186" t="inlineStr">
         <is>
-          <t>VP1 Stage 4 grip redesign: shaft supported at both ends - UNQUOTED</t>
+          <t>UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10620,12 +10620,12 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>WIND_SPOOL_DRUM</t>
+          <t>WIND_FLANGE_L</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>spool drum dia 70 x 58</t>
+          <t>spool flange dia 200 x 3 mm</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
@@ -10635,12 +10635,12 @@
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>steel tube or printed polymer</t>
+          <t>steel plate 3 mm screening candidate</t>
         </is>
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>WINDER_UNRATED</t>
+          <t>WINDER_STIFFNESS_SCREEN_PASS_HUB_HOLD</t>
         </is>
       </c>
       <c r="G187" t="inlineStr">
@@ -10665,7 +10665,7 @@
       </c>
       <c r="K187" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>20 N assumed rim load; 43.33 MPa/0.194 mm beam screen only; hub bolt balance guard unqualified; unquoted</t>
         </is>
       </c>
     </row>
@@ -10677,12 +10677,12 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>WIND_SPOOL_SHAFT</t>
+          <t>WIND_FLANGE_R</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>spool shaft dia 16 x 95</t>
+          <t>spool flange dia 200 x 3 mm</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
@@ -10692,12 +10692,12 @@
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>C45 candidate</t>
+          <t>steel plate 3 mm screening candidate</t>
         </is>
       </c>
       <c r="F188" t="inlineStr">
         <is>
-          <t>WINDER_UNRATED</t>
+          <t>WINDER_STIFFNESS_SCREEN_PASS_HUB_HOLD</t>
         </is>
       </c>
       <c r="G188" t="inlineStr">
@@ -10722,7 +10722,7 @@
       </c>
       <c r="K188" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>20 N assumed rim load; 43.33 MPa/0.194 mm beam screen only; hub bolt balance guard unqualified; unquoted</t>
         </is>
       </c>
     </row>
@@ -10734,12 +10734,12 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>WIND_TENSIONER</t>
+          <t>WIND_MOTOR_REF</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>slip tensioner post + wrap arm</t>
+          <t>spool gearmotor reference (not selected)</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
@@ -10749,12 +10749,12 @@
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>steel</t>
+          <t>24 V gearmotor MPN unselected</t>
         </is>
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>WINDER_UNRATED</t>
+          <t>MOTOR_UNSELECTED</t>
         </is>
       </c>
       <c r="G189" t="inlineStr">
@@ -10779,7 +10779,7 @@
       </c>
       <c r="K189" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>UNQUOTED; known motor floors exceed the 100000 KRW soft limit - not 0</t>
         </is>
       </c>
     </row>
@@ -10791,12 +10791,12 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>WIND_TRAVERSE_RIDER</t>
+          <t>WIND_SPOOL_BEARINGS</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>traverse rider block + guide eyelet</t>
+          <t>spool shaft bearing blocks at BOTH shaft ends</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
@@ -10806,7 +10806,7 @@
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>steel + printed guide</t>
+          <t>steel plate 5 mm + bearing seats</t>
         </is>
       </c>
       <c r="F190" t="inlineStr">
@@ -10816,12 +10816,12 @@
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-STAGE4</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-STAGE4</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
@@ -10836,7 +10836,7 @@
       </c>
       <c r="K190" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>VP1 Stage 4 grip redesign: shaft supported at both ends - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10848,50 +10848,278 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
+          <t>WIND_SPOOL_DRUM</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>spool drum dia 70 x 58</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>steel tube or printed polymer</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>WINDER_UNRATED</t>
+        </is>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>VP1-STAGE2</t>
+        </is>
+      </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>VP1-STAGE3</t>
+        </is>
+      </c>
+      <c r="I191" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J191" t="inlineStr">
+        <is>
+          <t>UNQUOTED_NOT_ZERO</t>
+        </is>
+      </c>
+      <c r="K191" t="inlineStr">
+        <is>
+          <t>UNQUOTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>vp1_stage1_3</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>WIND_SPOOL_SHAFT</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>spool shaft dia 16 x 95</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>C45 candidate</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>WINDER_UNRATED</t>
+        </is>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>VP1-STAGE2</t>
+        </is>
+      </c>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>VP1-STAGE3</t>
+        </is>
+      </c>
+      <c r="I192" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J192" t="inlineStr">
+        <is>
+          <t>UNQUOTED_NOT_ZERO</t>
+        </is>
+      </c>
+      <c r="K192" t="inlineStr">
+        <is>
+          <t>UNQUOTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>vp1_stage1_3</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>WIND_TENSIONER</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>slip tensioner post + wrap arm</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>steel</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>WINDER_UNRATED</t>
+        </is>
+      </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>VP1-STAGE2</t>
+        </is>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>VP1-STAGE3</t>
+        </is>
+      </c>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J193" t="inlineStr">
+        <is>
+          <t>UNQUOTED_NOT_ZERO</t>
+        </is>
+      </c>
+      <c r="K193" t="inlineStr">
+        <is>
+          <t>UNQUOTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>vp1_stage1_3</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>WIND_TRAVERSE_RIDER</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>traverse rider block + guide eyelet</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>steel + printed guide</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>WINDER_UNRATED</t>
+        </is>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>VP1-STAGE2</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>VP1-STAGE3</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J194" t="inlineStr">
+        <is>
+          <t>UNQUOTED_NOT_ZERO</t>
+        </is>
+      </c>
+      <c r="K194" t="inlineStr">
+        <is>
+          <t>UNQUOTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>vp1_stage1_3</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
           <t>WIND_TRAVERSE_SCREW</t>
         </is>
       </c>
-      <c r="C191" t="inlineStr">
+      <c r="C195" t="inlineStr">
         <is>
           <t>traverse lead screw dia 8 x 80</t>
         </is>
       </c>
-      <c r="D191" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E191" t="inlineStr">
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
         <is>
           <t>steel rod</t>
         </is>
       </c>
-      <c r="F191" t="inlineStr">
+      <c r="F195" t="inlineStr">
         <is>
           <t>WINDER_UNRATED</t>
         </is>
       </c>
-      <c r="G191" t="inlineStr">
+      <c r="G195" t="inlineStr">
         <is>
           <t>VP1-STAGE2</t>
         </is>
       </c>
-      <c r="H191" t="inlineStr">
+      <c r="H195" t="inlineStr">
         <is>
           <t>VP1-STAGE3</t>
         </is>
       </c>
-      <c r="I191" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J191" t="inlineStr">
+      <c r="I195" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J195" t="inlineStr">
         <is>
           <t>UNQUOTED_NOT_ZERO</t>
         </is>
       </c>
-      <c r="K191" t="inlineStr">
+      <c r="K195" t="inlineStr">
         <is>
           <t>UNQUOTED</t>
         </is>

</xml_diff>

<commit_message>
Document VP1 connected-flow HOLD with current CAD and Isaac evidence
</commit_message>
<xml_diff>
--- a/c2.1/bom/system_bom.xlsx
+++ b/c2.1/bom/system_bom.xlsx
@@ -5324,7 +5324,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Buffer190x48 top /50x40 throat /height73</t>
+          <t>Buffer190x48 top /Ø18 octagonal neck15 /height73</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -5364,7 +5364,7 @@
       </c>
       <c r="K94" t="inlineStr">
         <is>
-          <t>Internal geometric volume calculated; usable75pct separately stated. Top fits between Y251..299, ahead of pin rings. Cold throat offset to barrel feed X289.</t>
+          <t>Lower Ø13 clear octagon and Ø18 outer vertical neck centred on the Ø20 barrel feed bore at x299,y275. 15 mm neck precedes barrel handoff; 1 mm nominal radial room is not a manufacturing tolerance. Upper mouth fits Y251..299. Cold shell-to-barrel support, seal and independent metal throat liner remain manufacturing HOLD.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Compare VP1 relocated gravity feed against active transfer path
</commit_message>
<xml_diff>
--- a/c2.1/bom/system_bom.xlsx
+++ b/c2.1/bom/system_bom.xlsx
@@ -5324,7 +5324,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Buffer190x48 top /Ø18 octagonal neck15 /height73</t>
+          <t>Steel screen receiver with inset shoulder</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -5334,7 +5334,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>PC outer shell plus metal throat</t>
+          <t>S355 steel</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -5364,7 +5364,7 @@
       </c>
       <c r="K94" t="inlineStr">
         <is>
-          <t>Lower Ø13 clear octagon and Ø18 outer vertical neck centred on the Ø20 barrel feed bore at x299,y275. 15 mm neck precedes barrel handoff; 1 mm nominal radial room is not a manufacturing tolerance. Upper mouth fits Y251..299. Cold shell-to-barrel support, seal and independent metal throat liner remain manufacturing HOLD.</t>
+          <t>Original 190x48 mouth at z218, outer envelope z145..218; inset at z210 has inner x245..360,y255.5..294.5, covering the nominal S2 screen-bore columns without touching the screen edge at z215.2. Lower Ø13 clear octagonal throat at x299,y275,z145 with Ø18 outer neck z145..160. Weld to separate steel saddle at z145; fasteners, sealing, thermal isolation and fabrication DFM remain HOLD. No material-flow or physical-release claim.</t>
         </is>
       </c>
     </row>
@@ -5376,12 +5376,12 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>HOP-LID</t>
+          <t>FEED-BUF-CLAMP</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Interlocked lid180x140</t>
+          <t>Lower cold-barrel saddle half</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -5391,7 +5391,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>PC with metal strike</t>
+          <t>S355 steel</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -5421,24 +5421,24 @@
       </c>
       <c r="K95" t="inlineStr">
         <is>
-          <t>Hinge/guard lock hardware not chosen. NO open-lid operation.</t>
+          <t>Lower half of FEED-BUF-SADDLE; four M5 holes pair upper ears. Ø30.2 nominal bore on Ø30 barrel has 0.1 mm cold radial clearance, with 0.4 mm seam available for preload; torque and metal-to-barrel seal remain DFM HOLD.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>legacy_interface:frame</t>
+          <t>legacy_interface:feed</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>FR-2020-320</t>
+          <t>FEED-BUF-SADDLE</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>2020 profile cut320</t>
+          <t>Upper cold-barrel saddle and feed sleeve</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -5448,17 +5448,17 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Al extrusion - existing</t>
+          <t>S355 steel</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>OWNED_SLOT_PATTERN_TO_MEASURE</t>
+          <t>CUSTOM_DFM_HOLD</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>PPR_project_handover_2026-09-20.zip / 08_BOM_COMPONENTS.md</t>
+          <t>PPR-C1 original dimensional design; not an empirical qualification</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
@@ -5468,54 +5468,54 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>0</t>
+          <t/>
         </is>
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>OWNED_NO_NEW_PURCHASE</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
         <is>
-          <t>Nominal section only. Confirm slot series before buying brackets; 3 mm saw kerf.</t>
+          <t>Sleeve joins FEED-BUF lower steel face at z145 by qualified weld; upper half of Ø36/Ø30.2 x34 cold-barrel split clamp, 0.4 mm open seam and four M5 through-holes. Bolt preload, weld, seal and thermal fit remain DFM HOLD.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>legacy_interface:frame</t>
+          <t>legacy_interface:feed</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>FR-2020-360</t>
+          <t>HOP-LID</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>2020 profile cut 360</t>
+          <t>Interlocked lid180x140</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Al extrusion - existing</t>
+          <t>PC with metal strike</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>OWNED_SLOT_PATTERN_TO_MEASURE</t>
+          <t>CUSTOM_DFM_HOLD</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>PPR_project_handover_2026-09-20.zip / 08_BOM_COMPONENTS.md</t>
+          <t>PPR-C1 original dimensional design; not an empirical qualification</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
@@ -5525,17 +5525,17 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>0</t>
+          <t/>
         </is>
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>OWNED_NO_NEW_PURCHASE</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
         <is>
-          <t>Nominal section only. Confirm slot series before buying brackets; 3 mm saw kerf.</t>
+          <t>Hinge/guard lock hardware not chosen. NO open-lid operation.</t>
         </is>
       </c>
     </row>
@@ -5547,17 +5547,17 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>FR-2020-400</t>
+          <t>FR-2020-320</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>2020 profile cut 400</t>
+          <t>2020 profile cut320</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -5604,17 +5604,17 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>FR-2020-590</t>
+          <t>FR-2020-360</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>2020 profile cut 590</t>
+          <t>2020 profile cut 360</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -5661,12 +5661,12 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>FR-2040-320</t>
+          <t>FR-2020-400</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>2040 profile cut 320</t>
+          <t>2020 profile cut 400</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -5718,12 +5718,12 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>FR-2040-400</t>
+          <t>FR-2020-590</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>2040 profile cut 400</t>
+          <t>2020 profile cut 590</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -5775,12 +5775,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>FR-2040-630</t>
+          <t>FR-2040-320</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>2040 profile cut 630</t>
+          <t>2040 profile cut 320</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -5832,32 +5832,32 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>FR-BASE</t>
+          <t>FR-2040-400</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Bottom tray 630x400x3</t>
+          <t>2040 profile cut 400</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Al 5052</t>
+          <t>Al extrusion - existing</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>SHEET_DFM_HOLD</t>
+          <t>OWNED_SLOT_PATTERN_TO_MEASURE</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>PPR-C1 original dimensional design; not an empirical qualification</t>
+          <t>PPR_project_handover_2026-09-20.zip / 08_BOM_COMPONENTS.md</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
@@ -5867,54 +5867,54 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t/>
+          <t>0</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>OWNED_NO_NEW_PURCHASE</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
         <is>
-          <t>Mains and hot zones require separate partitions; shown base is not sealed containment.</t>
+          <t>Nominal section only. Confirm slot series before buying brackets; 3 mm saw kerf.</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>legacy_interface:frame_mount</t>
+          <t>legacy_interface:frame</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>DRV-DECK</t>
+          <t>FR-2040-630</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Steel drive deck240x194x5</t>
+          <t>2040 profile cut 630</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>S355 steel</t>
+          <t>Al extrusion - existing</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>CUSTOM_DFM_HOLD</t>
+          <t>OWNED_SLOT_PATTERN_TO_MEASURE</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>PPR-C1 original dimensional design; not an empirical qualification</t>
+          <t>PPR_project_handover_2026-09-20.zip / 08_BOM_COMPONENTS.md</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
@@ -5924,34 +5924,34 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t/>
+          <t>0</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>OWNED_NO_NEW_PURCHASE</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
         <is>
-          <t>Deck atZ20..25, supported by existing crossmembers. Added4 feet must be included in frame stiffness review.</t>
+          <t>Nominal section only. Confirm slot series before buying brackets; 3 mm saw kerf.</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>legacy_interface:frame_mount</t>
+          <t>legacy_interface:frame</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>DRV-M1-FOOT</t>
+          <t>FR-BASE</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>M1 steel mounting foot70x50x19</t>
+          <t>Bottom tray 630x400x3</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -5961,12 +5961,12 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Steel</t>
+          <t>Al 5052</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>CUSTOM_DFM_HOLD</t>
+          <t>SHEET_DFM_HOLD</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
@@ -5991,7 +5991,7 @@
       </c>
       <c r="K105" t="inlineStr">
         <is>
-          <t>Motor plate corner holes to vertical face. Base bolts to drive deck, not to a printed carrier.</t>
+          <t>Mains and hot zones require separate partitions; shown base is not sealed containment.</t>
         </is>
       </c>
     </row>
@@ -6003,12 +6003,12 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>DRV-RISER12</t>
+          <t>DRV-DECK</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Input rear bearing riser34x12x10</t>
+          <t>Steel drive deck240x194x5</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -6018,7 +6018,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Steel</t>
+          <t>S355 steel</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -6048,7 +6048,7 @@
       </c>
       <c r="K106" t="inlineStr">
         <is>
-          <t>Bearing bolt pattern must be transferred to deck after slots/profile series confirmed.</t>
+          <t>Deck atZ20..25, supported by existing crossmembers. Added4 feet must be included in frame stiffness review.</t>
         </is>
       </c>
     </row>
@@ -6060,12 +6060,12 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>DRV-RISER20</t>
+          <t>DRV-M1-FOOT</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Output rear bearing shim70x18x2.5</t>
+          <t>M1 steel mounting foot70x50x19</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -6105,7 +6105,7 @@
       </c>
       <c r="K107" t="inlineStr">
         <is>
-          <t>2.50 ground shim, full metal bearing support.</t>
+          <t>Motor plate corner holes to vertical face. Base bolts to drive deck, not to a printed carrier.</t>
         </is>
       </c>
     </row>
@@ -6117,12 +6117,12 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>EX-STAND</t>
+          <t>DRV-RISER12</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Thrust stand / coaxial motor bridge</t>
+          <t>Input rear bearing riser34x12x10</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -6162,7 +6162,7 @@
       </c>
       <c r="K108" t="inlineStr">
         <is>
-          <t>M2 and thrust carrier share metal stand on deck; no large right-angle gearbox. Top holes4xM6 to carrier. Weld/bolt/pressure proof remains HOLD.</t>
+          <t>Bearing bolt pattern must be transferred to deck after slots/profile series confirmed.</t>
         </is>
       </c>
     </row>
@@ -6174,22 +6174,22 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>S1-ROOF-F</t>
+          <t>DRV-RISER20</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Front roof bracket30x95x25</t>
+          <t>Output rear bearing shim70x18x2.5</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>10mm steel welded/folded</t>
+          <t>Steel</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
@@ -6219,7 +6219,7 @@
       </c>
       <c r="K109" t="inlineStr">
         <is>
-          <t>Face atY135 against retainer. M6 top hole to existing profile centreY50. Metal roof load path; bend/weld qualification pending.</t>
+          <t>2.50 ground shim, full metal bearing support.</t>
         </is>
       </c>
     </row>
@@ -6231,22 +6231,22 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>S1-ROOF-R</t>
+          <t>EX-STAND</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Rear roof bracket30x48x25</t>
+          <t>Thrust stand / coaxial motor bridge</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>10mm steel welded/folded</t>
+          <t>Steel</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
@@ -6276,7 +6276,7 @@
       </c>
       <c r="K110" t="inlineStr">
         <is>
-          <t>Face atY352; M6 profile connection atY390. Do not print this bracket.</t>
+          <t>M2 and thrust carrier share metal stand on deck; no large right-angle gearbox. Top holes4xM6 to carrier. Weld/bolt/pressure proof remains HOLD.</t>
         </is>
       </c>
     </row>
@@ -6288,12 +6288,12 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>S2-LEG-L</t>
+          <t>S1-ROOF-F</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>S2 L column / metal foot</t>
+          <t>Front roof bracket30x95x25</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -6303,7 +6303,7 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Steel</t>
+          <t>10mm steel welded/folded</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
@@ -6333,7 +6333,7 @@
       </c>
       <c r="K111" t="inlineStr">
         <is>
-          <t>Foot bottomZ25; topZ210. Centre mounting holeZ203. L sits on5mm deck, R on2020crossmember. Welded joint and anchors DFM hold.</t>
+          <t>Face atY135 against retainer. M6 top hole to existing profile centreY50. Metal roof load path; bend/weld qualification pending.</t>
         </is>
       </c>
     </row>
@@ -6345,12 +6345,12 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>S2-LEG-R</t>
+          <t>S1-ROOF-R</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>S2 R column / metal foot</t>
+          <t>Rear roof bracket30x48x25</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -6360,7 +6360,7 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Steel</t>
+          <t>10mm steel welded/folded</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
@@ -6390,44 +6390,44 @@
       </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t>Foot bottomZ20; topZ210. Centre mounting holeZ203. L sits on5mm deck, R on2020crossmember. Welded joint and anchors DFM hold.</t>
+          <t>Face atY352; M6 profile connection atY390. Do not print this bracket.</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>system_requirement</t>
+          <t>legacy_interface:frame_mount</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>AUX-DRIVES</t>
+          <t>S2-LEG-L</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Puller,spool,traverse actuation</t>
+          <t>S2 L column / metal foot</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Procurement requirement</t>
+          <t>Steel</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>AUX_ACTUATION_HOLD</t>
+          <t>CUSTOM_DFM_HOLD</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>Supplier drawing / capacity confirmation required before procurement</t>
+          <t>PPR-C1 original dimensional design; not an empirical qualification</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
@@ -6447,44 +6447,44 @@
       </c>
       <c r="K113" t="inlineStr">
         <is>
-          <t>Separate low-power controls, no large third shredder motor.</t>
+          <t>Foot bottomZ25; topZ210. Centre mounting holeZ203. L sits on5mm deck, R on2020crossmember. Welded joint and anchors DFM hold.</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>system_requirement</t>
+          <t>legacy_interface:frame_mount</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>CHAIN-A</t>
+          <t>S2-LEG-R</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>ANSI35 chain94 pitches</t>
+          <t>S2 R column / metal foot</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Procurement requirement</t>
+          <t>Steel</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>CHAIN_RATING_HOLD</t>
+          <t>CUSTOM_DFM_HOLD</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>Supplier drawing / capacity confirmation required before procurement</t>
+          <t>PPR-C1 original dimensional design; not an empirical qualification</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
@@ -6504,7 +6504,7 @@
       </c>
       <c r="K114" t="inlineStr">
         <is>
-          <t>Pitch length895.35mm. Working load and width to confirm.</t>
+          <t>Foot bottomZ20; topZ210. Centre mounting holeZ203. L sits on5mm deck, R on2020crossmember. Welded joint and anchors DFM hold.</t>
         </is>
       </c>
     </row>
@@ -6516,12 +6516,12 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>CHAIN-B</t>
+          <t>AUX-DRIVES</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>ANSI35 chain84 pitches</t>
+          <t>Puller,spool,traverse actuation</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -6536,7 +6536,7 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>CHAIN_RATING_HOLD</t>
+          <t>AUX_ACTUATION_HOLD</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
@@ -6561,7 +6561,7 @@
       </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t>Pitch length800.10mm. Working load and width to confirm.</t>
+          <t>Separate low-power controls, no large third shredder motor.</t>
         </is>
       </c>
     </row>
@@ -6573,12 +6573,12 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>CTRL-MEGA</t>
+          <t>CHAIN-A</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Arduino Mega</t>
+          <t>ANSI35 chain94 pitches</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -6593,12 +6593,12 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>OWNED</t>
+          <t>CHAIN_RATING_HOLD</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>PPR_project_handover_2026-09-20.zip / 08_BOM_COMPONENTS.md</t>
+          <t>Supplier drawing / capacity confirmation required before procurement</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
@@ -6608,17 +6608,17 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>0</t>
+          <t/>
         </is>
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>OWNED_NO_NEW_PURCHASE</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
         <is>
-          <t>Reference power allocator is NOT deployable heater firmware.</t>
+          <t>Pitch length895.35mm. Working load and width to confirm.</t>
         </is>
       </c>
     </row>
@@ -6630,12 +6630,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>DRV-TLIMIT</t>
+          <t>CHAIN-B</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Mechanical torque limiter</t>
+          <t>ANSI35 chain84 pitches</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -6650,7 +6650,7 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>TORQUE_LIMITER_HOLD</t>
+          <t>CHAIN_RATING_HOLD</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
@@ -6675,7 +6675,7 @@
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>Shared M1 input; calibration before blade operation.</t>
+          <t>Pitch length800.10mm. Working load and width to confirm.</t>
         </is>
       </c>
     </row>
@@ -6687,17 +6687,17 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>EL-BTS</t>
+          <t>CTRL-MEGA</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Existing BTS7960 modules</t>
+          <t>Arduino Mega</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -6707,7 +6707,7 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>OWNED_UNQUALIFIED</t>
+          <t>OWNED</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
@@ -6732,7 +6732,7 @@
       </c>
       <c r="K118" t="inlineStr">
         <is>
-          <t>Do not assume advertised43A continuous.</t>
+          <t>Reference power allocator is NOT deployable heater firmware.</t>
         </is>
       </c>
     </row>
@@ -6744,12 +6744,12 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>EL-DRV</t>
+          <t>DRV-TLIMIT</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Pololu2995 M1 driver option</t>
+          <t>Mechanical torque limiter</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -6764,12 +6764,12 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>OPTION_NOT_PURCHASED</t>
+          <t>TORQUE_LIMITER_HOLD</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>https://www.pololu.com/product/2995</t>
+          <t>Supplier drawing / capacity confirmation required before procurement</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
@@ -6789,7 +6789,7 @@
       </c>
       <c r="K119" t="inlineStr">
         <is>
-          <t>Configurable current limit; board21A is not terminal43A. Existing BTS7960 requires qualification.</t>
+          <t>Shared M1 input; calibration before blade operation.</t>
         </is>
       </c>
     </row>
@@ -6801,17 +6801,17 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>EL-TC</t>
+          <t>EL-BTS</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Adafruit3263 MAX31856</t>
+          <t>Existing BTS7960 modules</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
@@ -6821,12 +6821,12 @@
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>PURCHASE_CANDIDATE</t>
+          <t>OWNED_UNQUALIFIED</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>https://www.adafruit.com/product/3263</t>
+          <t>PPR_project_handover_2026-09-20.zip / 08_BOM_COMPONENTS.md</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
@@ -6836,17 +6836,17 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t/>
+          <t>0</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>OWNED_NO_NEW_PURCHASE</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>Four independent temperature inputs; K probes exact mechanical model unresolved.</t>
+          <t>Do not assume advertised43A continuous.</t>
         </is>
       </c>
     </row>
@@ -6858,12 +6858,12 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>FASTENERS</t>
+          <t>EL-DRV</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Brackets, metal supports,keys,shims,retainers</t>
+          <t>Pololu2995 M1 driver option</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -6878,12 +6878,12 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>HARDWARE_SCHEDULE_HOLD</t>
+          <t>OPTION_NOT_PURCHASED</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>Supplier drawing / capacity confirmation required before procurement</t>
+          <t>https://www.pololu.com/product/2995</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
@@ -6903,7 +6903,7 @@
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>Not an orderable quantity list; full mechanical fastener closure is outstanding.</t>
+          <t>Configurable current limit; board21A is not terminal43A. Existing BTS7960 requires qualification.</t>
         </is>
       </c>
     </row>
@@ -6915,17 +6915,17 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>FEED-CHUTE</t>
+          <t>EL-TC</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Metal lined transfer chute</t>
+          <t>Adafruit3263 MAX31856</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
@@ -6935,12 +6935,12 @@
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>TRANSFER_PATH_HOLD</t>
+          <t>PURCHASE_CANDIDATE</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>PPR-C1 original dimensional design; not an empirical qualification</t>
+          <t>https://www.adafruit.com/product/3263</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
@@ -6960,7 +6960,7 @@
       </c>
       <c r="K122" t="inlineStr">
         <is>
-          <t>Complete swept envelope/bridging check and split-print panels before release.</t>
+          <t>Four independent temperature inputs; K probes exact mechanical model unresolved.</t>
         </is>
       </c>
     </row>
@@ -6972,12 +6972,12 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>GUARDS</t>
+          <t>FASTENERS</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Steel cutter containment / chain guards / heat shield</t>
+          <t>Brackets, metal supports,keys,shims,retainers</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -6992,12 +6992,12 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>SAFETY_GEOMETRY_HOLD</t>
+          <t>HARDWARE_SCHEDULE_HOLD</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>PPR-C1 original dimensional design; not an empirical qualification</t>
+          <t>Supplier drawing / capacity confirmation required before procurement</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
@@ -7017,7 +7017,7 @@
       </c>
       <c r="K123" t="inlineStr">
         <is>
-          <t>Do not operate the open review assembly. Guard geometry still to be detailed.</t>
+          <t>Not an orderable quantity list; full mechanical fastener closure is outstanding.</t>
         </is>
       </c>
     </row>
@@ -7029,12 +7029,12 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>SAFE-BRAKE</t>
+          <t>FEED-CHUTE</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Bus overvoltage/braking protection</t>
+          <t>Metal lined transfer chute</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -7049,12 +7049,12 @@
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>REGEN_DESIGN_HOLD</t>
+          <t>TRANSFER_PATH_HOLD</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>Supplier drawing / capacity confirmation required before procurement</t>
+          <t>PPR-C1 original dimensional design; not an empirical qualification</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
@@ -7074,7 +7074,7 @@
       </c>
       <c r="K124" t="inlineStr">
         <is>
-          <t>PSU sink ability unknown; no regeneration assumption.</t>
+          <t>Complete swept envelope/bridging check and split-print panels before release.</t>
         </is>
       </c>
     </row>
@@ -7086,12 +7086,12 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>SAFE-CONTACT</t>
+          <t>GUARDS</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>24V coil DC rated contactor</t>
+          <t>Steel cutter containment / chain guards / heat shield</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -7106,12 +7106,12 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>SAFETY_SELECTION_HOLD</t>
+          <t>SAFETY_GEOMETRY_HOLD</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>Supplier drawing / capacity confirmation required before procurement</t>
+          <t>PPR-C1 original dimensional design; not an empirical qualification</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
@@ -7131,7 +7131,7 @@
       </c>
       <c r="K125" t="inlineStr">
         <is>
-          <t>Continuous&gt;=35A DC and fault-current breaking coordinated with fuse.</t>
+          <t>Do not operate the open review assembly. Guard geometry still to be detailed.</t>
         </is>
       </c>
     </row>
@@ -7143,12 +7143,12 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>SAFE-FUSE</t>
+          <t>SAFE-BRAKE</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Branch and mains fuses / holders</t>
+          <t>Bus overvoltage/braking protection</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -7163,7 +7163,7 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>CIRCUIT_DESIGN_HOLD</t>
+          <t>REGEN_DESIGN_HOLD</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
@@ -7188,7 +7188,7 @@
       </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>Select from actual cable ampacity, DC breaking and inrush. No guessed fuse order.</t>
+          <t>PSU sink ability unknown; no regeneration assumption.</t>
         </is>
       </c>
     </row>
@@ -7200,17 +7200,17 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>SAFE-LOCK</t>
+          <t>SAFE-CONTACT</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Coded/positive-opening guard lock</t>
+          <t>24V coil DC rated contactor</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
@@ -7245,7 +7245,7 @@
       </c>
       <c r="K127" t="inlineStr">
         <is>
-          <t>Lid and service access, standstill unlock, manual reset.</t>
+          <t>Continuous&gt;=35A DC and fault-current breaking coordinated with fuse.</t>
         </is>
       </c>
     </row>
@@ -7257,12 +7257,12 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>SAFE-STOP</t>
+          <t>SAFE-FUSE</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Existing E-stop</t>
+          <t>Branch and mains fuses / holders</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -7277,12 +7277,12 @@
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>OWNED_RATING_VERIFY</t>
+          <t>CIRCUIT_DESIGN_HOLD</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>PPR_project_handover_2026-09-20.zip / 08_BOM_COMPONENTS.md</t>
+          <t>Supplier drawing / capacity confirmation required before procurement</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
@@ -7292,17 +7292,17 @@
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>0</t>
+          <t/>
         </is>
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>OWNED_NO_NEW_PURCHASE</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t>Independent hard cut with contactor; contact configuration verify.</t>
+          <t>Select from actual cable ampacity, DC breaking and inrush. No guessed fuse order.</t>
         </is>
       </c>
     </row>
@@ -7314,17 +7314,17 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>SAFE-THERM</t>
+          <t>SAFE-LOCK</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Independent thermal cutoff chain</t>
+          <t>Coded/positive-opening guard lock</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
@@ -7359,24 +7359,24 @@
       </c>
       <c r="K129" t="inlineStr">
         <is>
-          <t>Normally closed manual-reset overtemp plus one-shot protection.</t>
+          <t>Lid and service access, standstill unlock, manual reset.</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>vp1_stage1_3</t>
+          <t>system_requirement</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>AUG_BEARINGS</t>
+          <t>SAFE-STOP</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>west split pillow plus east journal cradle for the r3 auger shaft</t>
+          <t>Existing E-stop</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -7386,54 +7386,54 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>steel plate 5 mm</t>
+          <t>Procurement requirement</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>TRANSFER_UNRATED</t>
+          <t>OWNED_RATING_VERIFY</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>PPR_project_handover_2026-09-20.zip / 08_BOM_COMPONENTS.md</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>C1_INTERFACE_BASELINE</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t/>
+          <t>0</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>UNQUOTED_NOT_ZERO</t>
+          <t>OWNED_NO_NEW_PURCHASE</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>Auger shaft supported at both ends - UNQUOTED</t>
+          <t>Independent hard cut with contactor; contact configuration verify.</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>vp1_stage1_3</t>
+          <t>system_requirement</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>AUG_SHAFT</t>
+          <t>SAFE-THERM</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>active auger conveyor: r3 shaft x236..370 at y232/z347.1; RH flight root r3/OD r8, pitch 28.5, four turns x238.5..352.5 with 3 mm swept face; U-shell bore r9.5, nominal BRep gap 1.085 mm</t>
+          <t>Independent thermal cutoff chain</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -7443,22 +7443,22 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>steel shaft + steel flight</t>
+          <t>Procurement requirement</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>TRANSFER_UNRATED</t>
+          <t>SAFETY_SELECTION_HOLD</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>Supplier drawing / capacity confirmation required before procurement</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>C1_INTERFACE_BASELINE</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -7468,12 +7468,12 @@
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>UNQUOTED_NOT_ZERO</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>Conveys +x at -5.4375 rpm for 58 rpm reference M1 via 15/40 gear and 24/12 chain B plus 8:1 worm/wheel; tolerance/runout/heat stack assumed not proven</t>
+          <t>Normally closed manual-reset overtemp plus one-shot protection.</t>
         </is>
       </c>
     </row>
@@ -7485,12 +7485,12 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>AUG_WHEEL</t>
+          <t>AUG_BEARINGS</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>16T worm wheel (REFERENCE geometry, unrated), face x359..365, sector web, teeth cut by discrete hobbing of the worm; keyed Ø6 auger bore</t>
+          <t>west split pillow plus east journal cradle for the r3 auger shaft</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -7500,12 +7500,12 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>steel (reference)</t>
+          <t>steel plate 5 mm</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>REFERENCE_UNRATED</t>
+          <t>TRANSFER_UNRATED</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
@@ -7530,7 +7530,7 @@
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>Matched 1.8 mm key and keyway transfer torque to AUG_SHAFT; tooth strength and wear unqualified - UNQUOTED</t>
+          <t>Auger shaft supported at both ends - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -7542,12 +7542,12 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>CHUTE_BODY</t>
+          <t>AUG_SHAFT</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>welded S1-&gt;S2 transfer chute with sealed pan, active screw-conveyor trough and east fallaway</t>
+          <t>active auger conveyor: r3 shaft x236..370 at y232/z347.1; RH flight root r3/OD r8, pitch 28.5, four turns x238.5..352.5 with 3 mm swept face; U-shell bore r9.5, nominal BRep gap 1.085 mm</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -7557,7 +7557,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>steel sheet 3 mm + formed trough</t>
+          <t>steel shaft + steel flight</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
@@ -7567,7 +7567,7 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>VP1-ADR-002</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
@@ -7587,7 +7587,7 @@
       </c>
       <c r="K133" t="inlineStr">
         <is>
-          <t>BRep geometry and digital flow only; material transport and containment are not physically qualified - UNQUOTED</t>
+          <t>Conveys +x at -5.4375 rpm for 58 rpm reference M1 via 15/40 gear and 24/12 chain B plus 8:1 worm/wheel; tolerance/runout/heat stack assumed not proven</t>
         </is>
       </c>
     </row>
@@ -7599,12 +7599,12 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>CHUTE_TROUGH_FLOOR_E</t>
+          <t>AUG_WHEEL</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>bolted trough ledge section over the S2 mouth</t>
+          <t>16T worm wheel (REFERENCE geometry, unrated), face x359..365, sector web, teeth cut by discrete hobbing of the worm; keyed Ø6 auger bore</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -7614,22 +7614,22 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>steel sheet 3 mm</t>
+          <t>steel (reference)</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>GEOMETRY_PASS</t>
+          <t>REFERENCE_UNRATED</t>
         </is>
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>VP1-ADR-002</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -7644,7 +7644,7 @@
       </c>
       <c r="K134" t="inlineStr">
         <is>
-          <t>Clearance-cut for the frozen saddle jacket - UNQUOTED</t>
+          <t>Matched 1.8 mm key and keyway transfer torque to AUG_SHAFT; tooth strength and wear unqualified - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -7656,12 +7656,12 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>CROSS_FEED_BEARINGS</t>
+          <t>CHUTE_BODY</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>paired cross-feed and idler journal support with structural rails</t>
+          <t>welded S1-&gt;S2 transfer chute with sealed pan, active screw-conveyor trough and east fallaway</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -7671,7 +7671,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>steel plate and journal shells</t>
+          <t>steel sheet 3 mm + formed trough</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -7681,14 +7681,14 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
+          <t>VP1-ADR-002</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
           <t>VP1-STAGE5</t>
         </is>
       </c>
-      <c r="H135" t="inlineStr">
-        <is>
-          <t>VP1-STAGE5</t>
-        </is>
-      </c>
       <c r="I135" t="inlineStr">
         <is>
           <t/>
@@ -7701,7 +7701,7 @@
       </c>
       <c r="K135" t="inlineStr">
         <is>
-          <t>BRep-supported reference geometry; wear and load unqualified - UNQUOTED</t>
+          <t>BRep geometry and digital flow only; material transport and containment are not physically qualified - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -7713,12 +7713,12 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>CROSS_FEED_GEAR</t>
+          <t>CHUTE_TROUGH_FLOOR_E</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>12T keyed output gear on transverse feed shaft</t>
+          <t>bolted trough ledge section over the S2 mouth</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -7728,22 +7728,22 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>steel reference gear</t>
+          <t>steel sheet 3 mm</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>TRANSFER_UNRATED</t>
+          <t>GEOMETRY_PASS</t>
         </is>
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>VP1-ADR-002</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>VP1-STAGE2</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -7758,7 +7758,7 @@
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>1:1 from PDL through idler; tooth contact and torque rating unqualified - UNQUOTED</t>
+          <t>Clearance-cut for the frozen saddle jacket - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -7770,12 +7770,12 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>CROSS_FEED_IDLER</t>
+          <t>CROSS_FEED_BEARINGS</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>12T integral idler and supported journal between PDL and transverse feed gears</t>
+          <t>paired cross-feed and idler journal support with structural rails</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -7785,7 +7785,7 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>steel reference gear and shaft</t>
+          <t>steel plate and journal shells</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
@@ -7815,7 +7815,7 @@
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>Two external meshes preserve rotation sign; journal rating unqualified - UNQUOTED</t>
+          <t>BRep-supported reference geometry; wear and load unqualified - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -7827,12 +7827,12 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>CROSS_FEED_SHAFT</t>
+          <t>CROSS_FEED_GEAR</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>RH helical screw on y-axis x357/z328 with 9 mm pitch; reduced-radius powered tail to y260.5</t>
+          <t>12T keyed output gear on transverse feed shaft</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -7842,7 +7842,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>steel shaft and welded flight</t>
+          <t>steel reference gear</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
@@ -7872,7 +7872,7 @@
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>Powered tail overlaps S2 mouth y255 by 5.502 mm; actual fragment handoff unproven - UNQUOTED</t>
+          <t>1:1 from PDL through idler; tooth contact and torque rating unqualified - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -7884,12 +7884,12 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>CROSS_FEED_SHELL</t>
+          <t>CROSS_FEED_IDLER</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>U cradle with rotor-relieved outer metal shelf past S2 mouth</t>
+          <t>12T integral idler and supported journal between PDL and transverse feed gears</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -7899,7 +7899,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>formed steel sheet</t>
+          <t>steel reference gear and shaft</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
@@ -7929,7 +7929,7 @@
       </c>
       <c r="K139" t="inlineStr">
         <is>
-          <t>Outer shelf y255..258 supports the handoff without entering swept rotor sector; material transfer unproven - UNQUOTED</t>
+          <t>Two external meshes preserve rotation sign; journal rating unqualified - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -7941,12 +7941,12 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>DRV-CHAIN-A</t>
+          <t>CROSS_FEED_SHAFT</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>#35 roller chain cut to 896 mm (94 links; chain A: jackshaft 24T -&gt; S1 shaft A 24T)</t>
+          <t>RH helical screw on y-axis x357/z328 with 9 mm pitch; reduced-radius powered tail to y260.5</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -7956,22 +7956,22 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>ANSI35 steel roller chain p=9.525</t>
+          <t>steel shaft and welded flight</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>PROCUREMENT_HOLD</t>
+          <t>TRANSFER_UNRATED</t>
         </is>
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>VP1-ADR-002</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>VP1-STAGE1</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -7986,7 +7986,7 @@
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>Cut length from tangent+pitch-arc geometry (drive_geometry.json chain_lengths.A=896.0). UNQUOTED: not 0 - the 100000 KRW soft limit applies to quoted lines only</t>
+          <t>Powered tail overlaps S2 mouth y255 by 5.502 mm; actual fragment handoff unproven - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -7998,12 +7998,12 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>DRV-CHAIN-B</t>
+          <t>CROSS_FEED_SHELL</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>#35 roller chain cut to 724 mm (76 links; chain B: jackshaft 24T -&gt; S2 12T, ADR-002 rev B)</t>
+          <t>U cradle with rotor-relieved outer metal shelf past S2 mouth</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -8013,22 +8013,22 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>ANSI35 steel roller chain p=9.525</t>
+          <t>formed steel sheet</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>PROCUREMENT_HOLD</t>
+          <t>TRANSFER_UNRATED</t>
         </is>
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>VP1-ADR-002</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>VP1-STAGE4</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -8043,7 +8043,7 @@
       </c>
       <c r="K141" t="inlineStr">
         <is>
-          <t>Cut length from tangent+pitch-arc geometry (chain_lengths.B=723.9). UNQUOTED: not 0</t>
+          <t>Outer shelf y255..258 supports the handoff without entering swept rotor sector; material transfer unproven - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -8055,12 +8055,12 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>EL_CONTACTOR</t>
+          <t>DRV-CHAIN-A</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>safety contactor</t>
+          <t>#35 roller chain cut to 896 mm (94 links; chain A: jackshaft 24T -&gt; S1 shaft A 24T)</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -8070,22 +8070,22 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>24 V coil contactor MPN unselected</t>
+          <t>ANSI35 steel roller chain p=9.525</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>SAFETY_HARDWARE_REQUIRED</t>
+          <t>PROCUREMENT_HOLD</t>
         </is>
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-ADR-002</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-STAGE1</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -8100,7 +8100,7 @@
       </c>
       <c r="K142" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>Cut length from tangent+pitch-arc geometry (drive_geometry.json chain_lengths.A=896.0). UNQUOTED: not 0 - the 100000 KRW soft limit applies to quoted lines only</t>
         </is>
       </c>
     </row>
@@ -8112,12 +8112,12 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>EL_CURRENT_LIMITER</t>
+          <t>DRV-CHAIN-B</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>heater sequencer / current-limit relay bank</t>
+          <t>#35 roller chain cut to 724 mm (76 links; chain B: jackshaft 24T -&gt; S2 12T, ADR-002 rev B)</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -8127,24 +8127,24 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>relay bank MPN unselected</t>
+          <t>ANSI35 steel roller chain p=9.525</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>CONTROL_REFERENCE_UNRATED</t>
+          <t>PROCUREMENT_HOLD</t>
         </is>
       </c>
       <c r="G143" t="inlineStr">
         <is>
+          <t>VP1-ADR-002</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
           <t>VP1-STAGE4</t>
         </is>
       </c>
-      <c r="H143" t="inlineStr">
-        <is>
-          <t>VP1-STAGE4</t>
-        </is>
-      </c>
       <c r="I143" t="inlineStr">
         <is>
           <t/>
@@ -8157,7 +8157,7 @@
       </c>
       <c r="K143" t="inlineStr">
         <is>
-          <t>Host-tested firmware excludes simultaneous heater bands and rejects demand above 792 W; independent electrical interlock and component ratings still required - UNQUOTED</t>
+          <t>Cut length from tangent+pitch-arc geometry (chain_lengths.B=723.9). UNQUOTED: not 0</t>
         </is>
       </c>
     </row>
@@ -8169,12 +8169,12 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>EL_DIN_RAIL</t>
+          <t>EL_CONTACTOR</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>DIN rail 35 mm top-hat x 210</t>
+          <t>safety contactor</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -8184,12 +8184,12 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>steel rail</t>
+          <t>24 V coil contactor MPN unselected</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>PROCUREMENT_HOLD</t>
+          <t>SAFETY_HARDWARE_REQUIRED</t>
         </is>
       </c>
       <c r="G144" t="inlineStr">
@@ -8226,12 +8226,12 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>EL_DRIVER_1</t>
+          <t>EL_CURRENT_LIMITER</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>stepper/BLDC driver (M1 branch)</t>
+          <t>heater sequencer / current-limit relay bank</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -8241,22 +8241,22 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>24 V driver MPN unselected</t>
+          <t>relay bank MPN unselected</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>MOTOR_UNSELECTED</t>
+          <t>CONTROL_REFERENCE_UNRATED</t>
         </is>
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-STAGE4</t>
         </is>
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-STAGE4</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -8271,7 +8271,7 @@
       </c>
       <c r="K145" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>Host-tested firmware excludes simultaneous heater bands and rejects demand above 792 W; independent electrical interlock and component ratings still required - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -8283,12 +8283,12 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>EL_DRIVER_2</t>
+          <t>EL_DIN_RAIL</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>stepper/BLDC driver (M2 branch)</t>
+          <t>DIN rail 35 mm top-hat x 210</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -8298,12 +8298,12 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>24 V driver MPN unselected</t>
+          <t>steel rail</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>MOTOR_UNSELECTED</t>
+          <t>PROCUREMENT_HOLD</t>
         </is>
       </c>
       <c r="G146" t="inlineStr">
@@ -8340,12 +8340,12 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>EL_DRIVER_3</t>
+          <t>EL_DRIVER_1</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>stepper/BLDC driver (winder/puller accessory)</t>
+          <t>stepper/BLDC driver (M1 branch)</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -8397,12 +8397,12 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>EL_ESTOP_BOX</t>
+          <t>EL_DRIVER_2</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>dual-channel E-stop / lid / service interlock relay box</t>
+          <t>stepper/BLDC driver (M2 branch)</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -8412,12 +8412,12 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>relay box MPN unselected</t>
+          <t>24 V driver MPN unselected</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>SAFETY_HARDWARE_REQUIRED</t>
+          <t>MOTOR_UNSELECTED</t>
         </is>
       </c>
       <c r="G148" t="inlineStr">
@@ -8454,12 +8454,12 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>EL_OVERTEMP_BOX</t>
+          <t>EL_DRIVER_3</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>manual-reset independent overtemperature relay box</t>
+          <t>stepper/BLDC driver (winder/puller accessory)</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -8469,12 +8469,12 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>relay box MPN unselected</t>
+          <t>24 V driver MPN unselected</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>SAFETY_HARDWARE_REQUIRED</t>
+          <t>MOTOR_UNSELECTED</t>
         </is>
       </c>
       <c r="G149" t="inlineStr">
@@ -8511,12 +8511,12 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>EL_WIRE_DUCT</t>
+          <t>EL_ESTOP_BOX</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>slotted wiring duct x 210</t>
+          <t>dual-channel E-stop / lid / service interlock relay box</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -8526,12 +8526,12 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>PVC duct</t>
+          <t>relay box MPN unselected</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>PROCUREMENT_HOLD</t>
+          <t>SAFETY_HARDWARE_REQUIRED</t>
         </is>
       </c>
       <c r="G150" t="inlineStr">
@@ -8568,12 +8568,12 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>GUARD_CHAIN_A</t>
+          <t>EL_OVERTEMP_BOX</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>chain A top-run lid plate</t>
+          <t>manual-reset independent overtemperature relay box</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -8583,17 +8583,17 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>steel plate 3 mm</t>
+          <t>relay box MPN unselected</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>CONTAINMENT_UNRATED</t>
+          <t>SAFETY_HARDWARE_REQUIRED</t>
         </is>
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-STAGE3</t>
         </is>
       </c>
       <c r="H151" t="inlineStr">
@@ -8625,12 +8625,12 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>GUARD_CHAIN_B</t>
+          <t>EL_WIRE_DUCT</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>chain B outer guard plate set (continuous; ADR-002 rev B re-route)</t>
+          <t>slotted wiring duct x 210</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
@@ -8640,17 +8640,17 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>steel plate 3 mm</t>
+          <t>PVC duct</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>CONTAINMENT_UNRATED</t>
+          <t>PROCUREMENT_HOLD</t>
         </is>
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-STAGE3</t>
         </is>
       </c>
       <c r="H152" t="inlineStr">
@@ -8682,12 +8682,12 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>GUARD_LID_INTERLOCK_SEAT</t>
+          <t>GUARD_CHAIN_A</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>hopper-lid interlock switch seat</t>
+          <t>chain A top-run lid plate</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
@@ -8739,12 +8739,12 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>GUARD_S2_RING</t>
+          <t>GUARD_CHAIN_B</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>S2 rotor ring guard (annular sector r 90..94 over 20..114 deg)</t>
+          <t>chain B outer guard plate set (continuous; ADR-002 rev B re-route)</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -8784,7 +8784,7 @@
       </c>
       <c r="K154" t="inlineStr">
         <is>
-          <t>Guard plate thickness unrated; service sweep verified - UNQUOTED</t>
+          <t>UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -8796,37 +8796,37 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>HOPPER_FASTENER_M3</t>
+          <t>GUARD_LID_INTERLOCK_SEAT</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>M3 x 12 through-bolt with low-profile head for PC panel to captive steel seam boss</t>
+          <t>hopper-lid interlock switch seat</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>steel metric fastener</t>
+          <t>steel plate 3 mm</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>FASTENER_ENVELOPE_HOLD</t>
+          <t>CONTAINMENT_UNRATED</t>
         </is>
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>VP1-HOPPER-SPLIT</t>
+          <t>VP1-STAGE2</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>VP1-HOPPER-GEOMETRY</t>
+          <t>VP1-STAGE3</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
@@ -8841,7 +8841,7 @@
       </c>
       <c r="K155" t="inlineStr">
         <is>
-          <t>M3 clearance holes and captive bosses are modeled; bolts/heads not modeled or selected. Head bearing/seal outside taper and torque/preload must be qualified before fabrication; UNQUOTED</t>
+          <t>UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -8853,12 +8853,12 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>HOPPER_PANEL_L</t>
+          <t>GUARD_S2_RING</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>C1 HOPPER.step PC loft cut at world x120, left half with front/rear M3 through-holes</t>
+          <t>S2 rotor ring guard (annular sector r 90..94 over 20..114 deg)</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -8868,22 +8868,22 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>polycarbonate FDM shell nominal 3 mm</t>
+          <t>steel plate 3 mm</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>PRINT_DFM_LINER_HOLD</t>
+          <t>CONTAINMENT_UNRATED</t>
         </is>
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>VP1-HOPPER-SPLIT</t>
+          <t>VP1-STAGE2</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>VP1-HOPPER-GEOMETRY</t>
+          <t>VP1-STAGE3</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -8898,7 +8898,7 @@
       </c>
       <c r="K156" t="inlineStr">
         <is>
-          <t>Actual CAD bbox 119.258 x 162.2 x 55.497 mm; print orientation/adhesion/infill and assembled joint strength unqualified; historical HOPPER_001 removed from active quantity; UNQUOTED</t>
+          <t>Guard plate thickness unrated; service sweep verified - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -8910,27 +8910,27 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>HOPPER_PANEL_R</t>
+          <t>HOPPER_FASTENER_M3</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>C1 HOPPER.step PC loft cut at world x120, right half with front/rear M3 through-holes</t>
+          <t>M3 x 12 through-bolt with low-profile head for PC panel to captive steel seam boss</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>polycarbonate FDM shell nominal 3 mm</t>
+          <t>steel metric fastener</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>PRINT_DFM_LINER_HOLD</t>
+          <t>FASTENER_ENVELOPE_HOLD</t>
         </is>
       </c>
       <c r="G157" t="inlineStr">
@@ -8955,7 +8955,7 @@
       </c>
       <c r="K157" t="inlineStr">
         <is>
-          <t>Actual CAD bbox 117 x 162.2 x 55.497 mm; print orientation/adhesion/infill and assembled joint strength unqualified; historical HOPPER_001 removed from active quantity; UNQUOTED</t>
+          <t>M3 clearance holes and captive bosses are modeled; bolts/heads not modeled or selected. Head bearing/seal outside taper and torque/preload must be qualified before fabrication; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -8967,12 +8967,12 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>HOPPER_SEAM_FRONT</t>
+          <t>HOPPER_PANEL_L</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>40 x 39 x 1.5 mm sloping steel upper front seam strap with four M3 clearance holes and integral captive hex bosses</t>
+          <t>C1 HOPPER.step PC loft cut at world x120, left half with front/rear M3 through-holes</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -8982,12 +8982,12 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>steel strip and welded captive bosses</t>
+          <t>polycarbonate FDM shell nominal 3 mm</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>SEAM_AND_LINER_HOLD</t>
+          <t>PRINT_DFM_LINER_HOLD</t>
         </is>
       </c>
       <c r="G158" t="inlineStr">
@@ -9012,7 +9012,7 @@
       </c>
       <c r="K158" t="inlineStr">
         <is>
-          <t>Wall-face support z456..495 across x120 split; not the C1 unmodeled lower steel safety liner; weld and bolt loads unqualified; UNQUOTED</t>
+          <t>Actual CAD bbox 119.258 x 162.2 x 55.497 mm; print orientation/adhesion/infill and assembled joint strength unqualified; historical HOPPER_001 removed from active quantity; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -9024,12 +9024,12 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>HOPPER_SEAM_REAR</t>
+          <t>HOPPER_PANEL_R</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>40 x 39 x 1.5 mm sloping steel upper rear seam strap with four M3 clearance holes and integral captive hex bosses</t>
+          <t>C1 HOPPER.step PC loft cut at world x120, right half with front/rear M3 through-holes</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -9039,12 +9039,12 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>steel strip and welded captive bosses</t>
+          <t>polycarbonate FDM shell nominal 3 mm</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>SEAM_AND_LINER_HOLD</t>
+          <t>PRINT_DFM_LINER_HOLD</t>
         </is>
       </c>
       <c r="G159" t="inlineStr">
@@ -9069,7 +9069,7 @@
       </c>
       <c r="K159" t="inlineStr">
         <is>
-          <t>Wall-face support z456..495 across x120 split; not the C1 unmodeled lower steel safety liner; weld and bolt loads unqualified; UNQUOTED</t>
+          <t>Actual CAD bbox 117 x 162.2 x 55.497 mm; print orientation/adhesion/infill and assembled joint strength unqualified; historical HOPPER_001 removed from active quantity; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -9081,12 +9081,12 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>PDL_BEARINGS</t>
+          <t>HOPPER_SEAM_FRONT</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>two split pillow posts carrying the worm shaft at x353..365, y204..210/352..358</t>
+          <t>40 x 39 x 1.5 mm sloping steel upper front seam strap with four M3 clearance holes and integral captive hex bosses</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
@@ -9096,22 +9096,22 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>steel plate 5 mm</t>
+          <t>steel strip and welded captive bosses</t>
         </is>
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>TRANSFER_UNRATED</t>
+          <t>SEAM_AND_LINER_HOLD</t>
         </is>
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>VP1-HOPPER-SPLIT</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>VP1-HOPPER-GEOMETRY</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -9126,7 +9126,7 @@
       </c>
       <c r="K160" t="inlineStr">
         <is>
-          <t>Mounted on the support-plate bosses - UNQUOTED</t>
+          <t>Wall-face support z456..495 across x120 split; not the C1 unmodeled lower steel safety liner; weld and bolt loads unqualified; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -9138,12 +9138,12 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>PDL_CHAIN</t>
+          <t>HOPPER_SEAM_REAR</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>#35 roller chain, 35 links incl. offset link; S2 12T second band to PDL_SPROCKET at x362, 1:1</t>
+          <t>40 x 39 x 1.5 mm sloping steel upper rear seam strap with four M3 clearance holes and integral captive hex bosses</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -9153,22 +9153,22 @@
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>ANSI35 steel roller chain p=9.525</t>
+          <t>steel strip and welded captive bosses</t>
         </is>
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>TRANSFER_UNRATED</t>
+          <t>SEAM_AND_LINER_HOLD</t>
         </is>
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>VP1-HOPPER-SPLIT</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>VP1-HOPPER-GEOMETRY</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
@@ -9183,7 +9183,7 @@
       </c>
       <c r="K161" t="inlineStr">
         <is>
-          <t>Nominal333.375 mm versus geometric332.734 mm; 0.641 mm length surplus. Offset-link strength and tension adjustment unqualified; no quote - UNQUOTED</t>
+          <t>Wall-face support z456..495 across x120 split; not the C1 unmodeled lower steel safety liner; weld and bolt loads unqualified; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -9195,12 +9195,12 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>PDL_FEED_GEAR</t>
+          <t>PDL_BEARINGS</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>12T keyed spur on worm shaft feeding orthogonal screw train</t>
+          <t>two split pillow posts carrying the worm shaft at x353..365, y204..210/352..358</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -9210,7 +9210,7 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>steel reference gear</t>
+          <t>steel plate 5 mm</t>
         </is>
       </c>
       <c r="F162" t="inlineStr">
@@ -9240,7 +9240,7 @@
       </c>
       <c r="K162" t="inlineStr">
         <is>
-          <t>Tooth strength and keyed fit unqualified - UNQUOTED</t>
+          <t>Mounted on the support-plate bosses - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -9252,12 +9252,12 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>PDL_SHAFT</t>
+          <t>PDL_CHAIN</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>trough worm shaft dia 10 x 188 (r5, y204..392, x362, z374.5), dia 12 keyed chain shoulder y376..392</t>
+          <t>#35 roller chain, 35 links incl. offset link; S2 12T second band to PDL_SPROCKET at x362, 1:1</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
@@ -9267,7 +9267,7 @@
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>steel rod C45 candidate</t>
+          <t>ANSI35 steel roller chain p=9.525</t>
         </is>
       </c>
       <c r="F163" t="inlineStr">
@@ -9297,7 +9297,7 @@
       </c>
       <c r="K163" t="inlineStr">
         <is>
-          <t>Carries the RH 2-start worm; keyed 12T sprocket takes 1:1 PDL_CHAIN drive from the S2 12T sprocket - UNQUOTED</t>
+          <t>Nominal333.375 mm versus geometric332.734 mm; 0.641 mm length surplus. Offset-link strength and tension adjustment unqualified; no quote - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -9309,12 +9309,12 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>PDL_SPROCKET</t>
+          <t>PDL_FEED_GEAR</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>worm-shaft drive sprocket 12T bore 12 mm with keyed hub on shaft shoulder</t>
+          <t>12T keyed spur on worm shaft feeding orthogonal screw train</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
@@ -9324,7 +9324,7 @@
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>ANSI35 steel sprocket</t>
+          <t>steel reference gear</t>
         </is>
       </c>
       <c r="F164" t="inlineStr">
@@ -9354,7 +9354,7 @@
       </c>
       <c r="K164" t="inlineStr">
         <is>
-          <t>Bore r6 on y376..392 shaft shoulder r6 with 1.8 mm key in matched slot; torque fit and chain rating UNRATED - UNQUOTED</t>
+          <t>Tooth strength and keyed fit unqualified - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -9366,12 +9366,12 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>PDL_WORM</t>
+          <t>PDL_SHAFT</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>RH 2-start worm (REFERENCE geometry, unrated): root r6/pitch r6.75/OD r7.5, lead angle 23.3 deg, length 20 (y220..240), keyed Ø10 shaft bore</t>
+          <t>trough worm shaft dia 10 x 188 (r5, y204..392, x362, z374.5), dia 12 keyed chain shoulder y376..392</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
@@ -9381,12 +9381,12 @@
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>steel (reference)</t>
+          <t>steel rod C45 candidate</t>
         </is>
       </c>
       <c r="F165" t="inlineStr">
         <is>
-          <t>REFERENCE_UNRATED</t>
+          <t>TRANSFER_UNRATED</t>
         </is>
       </c>
       <c r="G165" t="inlineStr">
@@ -9411,7 +9411,7 @@
       </c>
       <c r="K165" t="inlineStr">
         <is>
-          <t>Matched 1.8 mm key and keyway transfer torque from PDL_SHAFT; tooth mesh and loads remain unrated - UNQUOTED</t>
+          <t>Carries the RH 2-start worm; keyed 12T sprocket takes 1:1 PDL_CHAIN drive from the S2 12T sprocket - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -9423,12 +9423,12 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>PULL_FRAME</t>
+          <t>PDL_SPROCKET</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>puller side plates + base + fixed-roller bearing seats + carriage guide slots</t>
+          <t>worm-shaft drive sprocket 12T bore 12 mm with keyed hub on shaft shoulder</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
@@ -9438,22 +9438,22 @@
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>steel plate 5 mm + 3 mm</t>
+          <t>ANSI35 steel sprocket</t>
         </is>
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>NIP_RATING_HOLD</t>
+          <t>TRANSFER_UNRATED</t>
         </is>
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>VP1-STAGE4</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>VP1-STAGE4</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
@@ -9468,7 +9468,7 @@
       </c>
       <c r="K166" t="inlineStr">
         <is>
-          <t>Positive stop 1.5 mm and adjustable open nip to 3.0 mm; spring carriage grips nominal 1.75 mm filament - UNQUOTED</t>
+          <t>Bore r6 on y376..392 shaft shoulder r6 with 1.8 mm key in matched slot; torque fit and chain rating UNRATED - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -9480,12 +9480,12 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>PULL_MOTOR_REF</t>
+          <t>PDL_WORM</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>puller gearmotor reference (not selected)</t>
+          <t>RH 2-start worm (REFERENCE geometry, unrated): root r6/pitch r6.75/OD r7.5, lead angle 23.3 deg, length 20 (y220..240), keyed Ø10 shaft bore</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
@@ -9495,22 +9495,22 @@
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>24 V gearmotor MPN unselected</t>
+          <t>steel (reference)</t>
         </is>
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>MOTOR_UNSELECTED</t>
+          <t>REFERENCE_UNRATED</t>
         </is>
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -9525,7 +9525,7 @@
       </c>
       <c r="K167" t="inlineStr">
         <is>
-          <t>UNQUOTED; known motor floors exceed the 100000 KRW soft limit - not 0</t>
+          <t>Matched 1.8 mm key and keyway transfer torque from PDL_SHAFT; tooth mesh and loads remain unrated - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -9537,12 +9537,12 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>PULL_NIP_STOP</t>
+          <t>PULL_FRAME</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>nip positive-stop cam block (1.5 mm minimum, 3.0 mm open)</t>
+          <t>puller side plates + base + fixed-roller bearing seats + carriage guide slots</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
@@ -9552,7 +9552,7 @@
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>steel</t>
+          <t>steel plate 5 mm + 3 mm</t>
         </is>
       </c>
       <c r="F168" t="inlineStr">
@@ -9562,12 +9562,12 @@
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-STAGE4</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-STAGE4</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
@@ -9582,7 +9582,7 @@
       </c>
       <c r="K168" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>Positive stop 1.5 mm and adjustable open nip to 3.0 mm; spring carriage grips nominal 1.75 mm filament - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -9594,12 +9594,12 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>PULL_ROLLER_ADJ</t>
+          <t>PULL_MOTOR_REF</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>puller adjustable roller dia 20 + spring-loaded carriage (guide posts, coil springs, cam stop)</t>
+          <t>puller gearmotor reference (not selected)</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
@@ -9609,12 +9609,12 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>steel; M5 screw</t>
+          <t>24 V gearmotor MPN unselected</t>
         </is>
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>NIP_RATING_HOLD</t>
+          <t>MOTOR_UNSELECTED</t>
         </is>
       </c>
       <c r="G169" t="inlineStr">
@@ -9639,7 +9639,7 @@
       </c>
       <c r="K169" t="inlineStr">
         <is>
-          <t>Spring-loaded carrier grips 1.5-2.0 mm filament (1.75 nominal, design/parameters.json filament_mm); cam stop range 1.5..3.0 mm - UNQUOTED</t>
+          <t>UNQUOTED; known motor floors exceed the 100000 KRW soft limit - not 0</t>
         </is>
       </c>
     </row>
@@ -9651,12 +9651,12 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>PULL_ROLLER_FIXED</t>
+          <t>PULL_NIP_STOP</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>puller drive roller dia 20 x 22</t>
+          <t>nip positive-stop cam block (1.5 mm minimum, 3.0 mm open)</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -9666,7 +9666,7 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>steel; knurl or rubber per TPU grip</t>
+          <t>steel</t>
         </is>
       </c>
       <c r="F170" t="inlineStr">
@@ -9708,37 +9708,37 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>S1_BELT</t>
+          <t>PULL_ROLLER_ADJ</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>two side-loop treads over x80..219; y163.5..223.2 and 240.8..323.5</t>
+          <t>puller adjustable roller dia 20 + spring-loaded carriage (guide posts, coil springs, cam stop)</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>polymer belt with steel-supported drums</t>
+          <t>steel; M5 screw</t>
         </is>
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t>TRANSFER_UNRATED</t>
+          <t>NIP_RATING_HOLD</t>
         </is>
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>VP1-STAGE2</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>VP1-STAGE3</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
@@ -9753,7 +9753,7 @@
       </c>
       <c r="K171" t="inlineStr">
         <is>
-          <t>Friction and tension unrated; UNQUOTED</t>
+          <t>Spring-loaded carrier grips 1.5-2.0 mm filament (1.75 nominal, design/parameters.json filament_mm); cam stop range 1.5..3.0 mm - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -9765,12 +9765,12 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>S1_BELT_BEARINGS</t>
+          <t>PULL_ROLLER_FIXED</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>four belt shaft support rings in the side rails</t>
+          <t>puller drive roller dia 20 x 22</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
@@ -9780,22 +9780,22 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>steel bearing seats</t>
+          <t>steel; knurl or rubber per TPU grip</t>
         </is>
       </c>
       <c r="F172" t="inlineStr">
         <is>
-          <t>TRANSFER_UNRATED</t>
+          <t>NIP_RATING_HOLD</t>
         </is>
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>VP1-STAGE2</t>
         </is>
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>VP1-STAGE3</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
@@ -9810,7 +9810,7 @@
       </c>
       <c r="K172" t="inlineStr">
         <is>
-          <t>Bearing selection and loads unqualified; UNQUOTED</t>
+          <t>UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -9822,22 +9822,22 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>S1_BELT_CHAIN</t>
+          <t>S1_BELT</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>#35 chain from S1B 24T to west belt 12T</t>
+          <t>two side-loop treads over x80..219; y163.5..223.2 and 240.8..323.5</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>ANSI35 steel chain</t>
+          <t>polymer belt with steel-supported drums</t>
         </is>
       </c>
       <c r="F173" t="inlineStr">
@@ -9867,7 +9867,7 @@
       </c>
       <c r="K173" t="inlineStr">
         <is>
-          <t>Tension and strength unrated; UNQUOTED</t>
+          <t>Friction and tension unrated; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -9879,12 +9879,12 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>S1_BELT_DRIVE</t>
+          <t>S1_BELT_BEARINGS</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>common waisted drive drum at x80; separate r3.8 side and r2.3 central tread seats</t>
+          <t>four belt shaft support rings in the side rails</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
@@ -9894,7 +9894,7 @@
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>steel shaft and drums</t>
+          <t>steel bearing seats</t>
         </is>
       </c>
       <c r="F174" t="inlineStr">
@@ -9924,7 +9924,7 @@
       </c>
       <c r="K174" t="inlineStr">
         <is>
-          <t>S1B chain-driven; torque and bearing load unrated; UNQUOTED</t>
+          <t>Bearing selection and loads unqualified; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -9936,12 +9936,12 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>S1_BELT_FOLLOWER</t>
+          <t>S1_BELT_CHAIN</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>12T sprocket on the west belt driver</t>
+          <t>#35 chain from S1B 24T to west belt 12T</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
@@ -9951,7 +9951,7 @@
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>ANSI35 steel sprocket</t>
+          <t>ANSI35 steel chain</t>
         </is>
       </c>
       <c r="F175" t="inlineStr">
@@ -9981,7 +9981,7 @@
       </c>
       <c r="K175" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>Tension and strength unrated; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -9993,12 +9993,12 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>S1_BELT_IDLER</t>
+          <t>S1_BELT_DRIVE</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>two split side idler drums at x219 leaving the central transfer corridor open</t>
+          <t>common waisted drive drum at x80; separate r3.8 side and r2.3 central tread seats</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -10008,7 +10008,7 @@
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>steel journals and drums</t>
+          <t>steel shaft and drums</t>
         </is>
       </c>
       <c r="F176" t="inlineStr">
@@ -10038,7 +10038,7 @@
       </c>
       <c r="K176" t="inlineStr">
         <is>
-          <t>Two independent journal halves; UNQUOTED</t>
+          <t>S1B chain-driven; torque and bearing load unrated; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10050,12 +10050,12 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>S1_SWEEP_BEARINGS</t>
+          <t>S1_BELT_FOLLOWER</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>two separated sweep bearing rings in the pan rails</t>
+          <t>12T sprocket on the west belt driver</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
@@ -10065,7 +10065,7 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>steel bearing seats</t>
+          <t>ANSI35 steel sprocket</t>
         </is>
       </c>
       <c r="F177" t="inlineStr">
@@ -10107,12 +10107,12 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>S1_SWEEP_GEAR_DRUM_N</t>
+          <t>S1_BELT_IDLER</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>12T gear on the north east belt idler</t>
+          <t>two split side idler drums at x219 leaving the central transfer corridor open</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
@@ -10122,7 +10122,7 @@
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>steel gear</t>
+          <t>steel journals and drums</t>
         </is>
       </c>
       <c r="F178" t="inlineStr">
@@ -10152,7 +10152,7 @@
       </c>
       <c r="K178" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>Two independent journal halves; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10164,12 +10164,12 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>S1_SWEEP_GEAR_DRUM_S</t>
+          <t>S1_SWEEP_BEARINGS</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>12T gear on the south east belt idler</t>
+          <t>two separated sweep bearing rings in the pan rails</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
@@ -10179,7 +10179,7 @@
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>steel gear</t>
+          <t>steel bearing seats</t>
         </is>
       </c>
       <c r="F179" t="inlineStr">
@@ -10221,12 +10221,12 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>S1_SWEEP_GEAR_N</t>
+          <t>S1_SWEEP_GEAR_DRUM_N</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>12T gear on the north sweep shaft</t>
+          <t>12T gear on the north east belt idler</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
@@ -10278,12 +10278,12 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>S1_SWEEP_GEAR_S</t>
+          <t>S1_SWEEP_GEAR_DRUM_S</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>12T gear on the south sweep shaft</t>
+          <t>12T gear on the south east belt idler</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
@@ -10335,12 +10335,12 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>S1_SWEEP_NORTH</t>
+          <t>S1_SWEEP_GEAR_N</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>north transverse screw x224 y235.5..359 feeding the central lane</t>
+          <t>12T gear on the north sweep shaft</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
@@ -10350,7 +10350,7 @@
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>steel shaft and flight</t>
+          <t>steel gear</t>
         </is>
       </c>
       <c r="F182" t="inlineStr">
@@ -10380,7 +10380,7 @@
       </c>
       <c r="K182" t="inlineStr">
         <is>
-          <t>Dynamic side-belt pickup under verification; UNQUOTED</t>
+          <t>UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10392,12 +10392,12 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>S1_SWEEP_SOUTH</t>
+          <t>S1_SWEEP_GEAR_S</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>south transverse screw x224 y127..228.5 feeding the central lane</t>
+          <t>12T gear on the south sweep shaft</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
@@ -10407,7 +10407,7 @@
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>steel shaft and flight</t>
+          <t>steel gear</t>
         </is>
       </c>
       <c r="F183" t="inlineStr">
@@ -10437,7 +10437,7 @@
       </c>
       <c r="K183" t="inlineStr">
         <is>
-          <t>Dynamic side-belt pickup under verification; UNQUOTED</t>
+          <t>UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10449,12 +10449,12 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>S1_TRANSFER_BEARINGS</t>
+          <t>S1_SWEEP_NORTH</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>two central idler support rings</t>
+          <t>north transverse screw x224 y235.5..359 feeding the central lane</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
@@ -10464,7 +10464,7 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>steel bearing seats</t>
+          <t>steel shaft and flight</t>
         </is>
       </c>
       <c r="F184" t="inlineStr">
@@ -10494,7 +10494,7 @@
       </c>
       <c r="K184" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>Dynamic side-belt pickup under verification; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10506,12 +10506,12 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>S1_TRANSFER_BELT</t>
+          <t>S1_SWEEP_SOUTH</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>central 17 mm tread from x80 to x260 inside the two side loops</t>
+          <t>south transverse screw x224 y127..228.5 feeding the central lane</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
@@ -10521,7 +10521,7 @@
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>polymer belt</t>
+          <t>steel shaft and flight</t>
         </is>
       </c>
       <c r="F185" t="inlineStr">
@@ -10551,7 +10551,7 @@
       </c>
       <c r="K185" t="inlineStr">
         <is>
-          <t>Screw pickup unproven; UNQUOTED</t>
+          <t>Dynamic side-belt pickup under verification; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10563,12 +10563,12 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>S1_TRANSFER_IDLER</t>
+          <t>S1_TRANSFER_BEARINGS</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>central east r2.3 idler at x260</t>
+          <t>two central idler support rings</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
@@ -10578,7 +10578,7 @@
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>steel drum</t>
+          <t>steel bearing seats</t>
         </is>
       </c>
       <c r="F186" t="inlineStr">
@@ -10620,12 +10620,12 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>WIND_FLANGE_L</t>
+          <t>S1_TRANSFER_BELT</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>spool flange dia 200 x 3 mm</t>
+          <t>central 17 mm tread from x80 to x260 inside the two side loops</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
@@ -10635,22 +10635,22 @@
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>steel plate 3 mm screening candidate</t>
+          <t>polymer belt</t>
         </is>
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>WINDER_STIFFNESS_SCREEN_PASS_HUB_HOLD</t>
+          <t>TRANSFER_UNRATED</t>
         </is>
       </c>
       <c r="G187" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
@@ -10665,7 +10665,7 @@
       </c>
       <c r="K187" t="inlineStr">
         <is>
-          <t>20 N assumed rim load; 43.33 MPa/0.194 mm beam screen only; hub bolt balance guard unqualified; unquoted</t>
+          <t>Screw pickup unproven; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10677,12 +10677,12 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>WIND_FLANGE_R</t>
+          <t>S1_TRANSFER_IDLER</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>spool flange dia 200 x 3 mm</t>
+          <t>central east r2.3 idler at x260</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
@@ -10692,22 +10692,22 @@
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>steel plate 3 mm screening candidate</t>
+          <t>steel drum</t>
         </is>
       </c>
       <c r="F188" t="inlineStr">
         <is>
-          <t>WINDER_STIFFNESS_SCREEN_PASS_HUB_HOLD</t>
+          <t>TRANSFER_UNRATED</t>
         </is>
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
@@ -10722,7 +10722,7 @@
       </c>
       <c r="K188" t="inlineStr">
         <is>
-          <t>20 N assumed rim load; 43.33 MPa/0.194 mm beam screen only; hub bolt balance guard unqualified; unquoted</t>
+          <t>UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10734,12 +10734,12 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>WIND_MOTOR_REF</t>
+          <t>WIND_FLANGE_L</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>spool gearmotor reference (not selected)</t>
+          <t>spool flange dia 200 x 3 mm</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
@@ -10749,12 +10749,12 @@
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>24 V gearmotor MPN unselected</t>
+          <t>steel plate 3 mm screening candidate</t>
         </is>
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>MOTOR_UNSELECTED</t>
+          <t>WINDER_STIFFNESS_SCREEN_PASS_HUB_HOLD</t>
         </is>
       </c>
       <c r="G189" t="inlineStr">
@@ -10779,7 +10779,7 @@
       </c>
       <c r="K189" t="inlineStr">
         <is>
-          <t>UNQUOTED; known motor floors exceed the 100000 KRW soft limit - not 0</t>
+          <t>20 N assumed rim load; 43.33 MPa/0.194 mm beam screen only; hub bolt balance guard unqualified; unquoted</t>
         </is>
       </c>
     </row>
@@ -10791,12 +10791,12 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>WIND_SPOOL_BEARINGS</t>
+          <t>WIND_FLANGE_R</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>spool shaft bearing blocks at BOTH shaft ends</t>
+          <t>spool flange dia 200 x 3 mm</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
@@ -10806,22 +10806,22 @@
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>steel plate 5 mm + bearing seats</t>
+          <t>steel plate 3 mm screening candidate</t>
         </is>
       </c>
       <c r="F190" t="inlineStr">
         <is>
-          <t>WINDER_UNRATED</t>
+          <t>WINDER_STIFFNESS_SCREEN_PASS_HUB_HOLD</t>
         </is>
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>VP1-STAGE4</t>
+          <t>VP1-STAGE2</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>VP1-STAGE4</t>
+          <t>VP1-STAGE3</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
@@ -10836,7 +10836,7 @@
       </c>
       <c r="K190" t="inlineStr">
         <is>
-          <t>VP1 Stage 4 grip redesign: shaft supported at both ends - UNQUOTED</t>
+          <t>20 N assumed rim load; 43.33 MPa/0.194 mm beam screen only; hub bolt balance guard unqualified; unquoted</t>
         </is>
       </c>
     </row>
@@ -10848,12 +10848,12 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>WIND_SPOOL_DRUM</t>
+          <t>WIND_MOTOR_REF</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>spool drum dia 70 x 58</t>
+          <t>spool gearmotor reference (not selected)</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
@@ -10863,12 +10863,12 @@
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>steel tube or printed polymer</t>
+          <t>24 V gearmotor MPN unselected</t>
         </is>
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t>WINDER_UNRATED</t>
+          <t>MOTOR_UNSELECTED</t>
         </is>
       </c>
       <c r="G191" t="inlineStr">
@@ -10893,7 +10893,7 @@
       </c>
       <c r="K191" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>UNQUOTED; known motor floors exceed the 100000 KRW soft limit - not 0</t>
         </is>
       </c>
     </row>
@@ -10905,12 +10905,12 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>WIND_SPOOL_SHAFT</t>
+          <t>WIND_SPOOL_BEARINGS</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>spool shaft dia 16 x 95</t>
+          <t>spool shaft bearing blocks at BOTH shaft ends</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
@@ -10920,7 +10920,7 @@
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>C45 candidate</t>
+          <t>steel plate 5 mm + bearing seats</t>
         </is>
       </c>
       <c r="F192" t="inlineStr">
@@ -10930,12 +10930,12 @@
       </c>
       <c r="G192" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-STAGE4</t>
         </is>
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-STAGE4</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
@@ -10950,7 +10950,7 @@
       </c>
       <c r="K192" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>VP1 Stage 4 grip redesign: shaft supported at both ends - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10962,12 +10962,12 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>WIND_TENSIONER</t>
+          <t>WIND_SPOOL_DRUM</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>slip tensioner post + wrap arm</t>
+          <t>spool drum dia 70 x 58</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
@@ -10977,7 +10977,7 @@
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>steel</t>
+          <t>steel tube or printed polymer</t>
         </is>
       </c>
       <c r="F193" t="inlineStr">
@@ -11019,12 +11019,12 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>WIND_TRAVERSE_RIDER</t>
+          <t>WIND_SPOOL_SHAFT</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>traverse rider block + guide eyelet</t>
+          <t>spool shaft dia 16 x 95</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
@@ -11034,7 +11034,7 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>steel + printed guide</t>
+          <t>C45 candidate</t>
         </is>
       </c>
       <c r="F194" t="inlineStr">
@@ -11076,50 +11076,164 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
+          <t>WIND_TENSIONER</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>slip tensioner post + wrap arm</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>steel</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>WINDER_UNRATED</t>
+        </is>
+      </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>VP1-STAGE2</t>
+        </is>
+      </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>VP1-STAGE3</t>
+        </is>
+      </c>
+      <c r="I195" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J195" t="inlineStr">
+        <is>
+          <t>UNQUOTED_NOT_ZERO</t>
+        </is>
+      </c>
+      <c r="K195" t="inlineStr">
+        <is>
+          <t>UNQUOTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>vp1_stage1_3</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>WIND_TRAVERSE_RIDER</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>traverse rider block + guide eyelet</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>steel + printed guide</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>WINDER_UNRATED</t>
+        </is>
+      </c>
+      <c r="G196" t="inlineStr">
+        <is>
+          <t>VP1-STAGE2</t>
+        </is>
+      </c>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>VP1-STAGE3</t>
+        </is>
+      </c>
+      <c r="I196" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J196" t="inlineStr">
+        <is>
+          <t>UNQUOTED_NOT_ZERO</t>
+        </is>
+      </c>
+      <c r="K196" t="inlineStr">
+        <is>
+          <t>UNQUOTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>vp1_stage1_3</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
           <t>WIND_TRAVERSE_SCREW</t>
         </is>
       </c>
-      <c r="C195" t="inlineStr">
+      <c r="C197" t="inlineStr">
         <is>
           <t>traverse lead screw dia 8 x 80</t>
         </is>
       </c>
-      <c r="D195" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E195" t="inlineStr">
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
         <is>
           <t>steel rod</t>
         </is>
       </c>
-      <c r="F195" t="inlineStr">
+      <c r="F197" t="inlineStr">
         <is>
           <t>WINDER_UNRATED</t>
         </is>
       </c>
-      <c r="G195" t="inlineStr">
+      <c r="G197" t="inlineStr">
         <is>
           <t>VP1-STAGE2</t>
         </is>
       </c>
-      <c r="H195" t="inlineStr">
+      <c r="H197" t="inlineStr">
         <is>
           <t>VP1-STAGE3</t>
         </is>
       </c>
-      <c r="I195" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J195" t="inlineStr">
+      <c r="I197" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J197" t="inlineStr">
         <is>
           <t>UNQUOTED_NOT_ZERO</t>
         </is>
       </c>
-      <c r="K195" t="inlineStr">
+      <c r="K197" t="inlineStr">
         <is>
           <t>UNQUOTED</t>
         </is>

</xml_diff>

<commit_message>
VP1: correct filament feedback model and refresh integrated digital artifacts
</commit_message>
<xml_diff>
--- a/c2.1/bom/system_bom.xlsx
+++ b/c2.1/bom/system_bom.xlsx
@@ -7661,7 +7661,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>welded S1-&gt;S2 transfer chute with sealed pan, active screw-conveyor trough and east fallaway</t>
+          <t>welded S1-&gt;S2 transfer chute with sweep-flight reliefs, central transfer belt and east auger receiver</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -7686,7 +7686,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>VP1-REFERENCE-FEED</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -7701,7 +7701,7 @@
       </c>
       <c r="K135" t="inlineStr">
         <is>
-          <t>BRep geometry and digital flow only; material transport and containment are not physically qualified - UNQUOTED</t>
+          <t>Static BRep clearance only; previous native S1 pickup 10/22 and auger advance 1/22 on older STEP; no new same-particle run; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -7775,7 +7775,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>adjustable cooling duct: rails + sliding baffle (100 mm travel, 50..250 mm ducted length) over COOL-TRAY</t>
+          <t>vented sliding hood on rails with 100 mm travel over COOL-TRAY</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -7785,7 +7785,7 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>steel sheet 3 mm rails + baffle</t>
+          <t>steel sheet 3 mm rails + hood</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
@@ -7815,7 +7815,7 @@
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>COOL-TRAY south wall gains two 78x21 ports and hood top fan gets open aperture; 50..250 mm effective cooling length remains uncalibrated; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -7832,7 +7832,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>third 80 mm fan reference on cooling baffle (9RA0824H1001 class)</t>
+          <t>separate 80x80x38 open-ring third fan envelope on sliding hood</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -7872,7 +7872,7 @@
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>UNRATED 8 W estimate admitted by 500 W allocator; UNQUOTED</t>
+          <t>8 W sensitivity estimate not rated; no PWM assumed; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -8385,7 +8385,7 @@
       </c>
       <c r="K147" t="inlineStr">
         <is>
-          <t>Host-tested firmware excludes simultaneous heater bands and rejects demand above 792 W; independent electrical interlock and component ratings still required - UNQUOTED</t>
+          <t>Host-tested firmware excludes simultaneous heater bands and refuses demands above 500 W modeled cap; independent electrical interlock and component ratings still required - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -8858,7 +8858,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>diameter gauge mounting straps + wall spacers inside COOL-TRAY exit section (x801..807/816..818, bolted to tray walls)</t>
+          <t>diameter gauge mounting straps + wall spacers inside COOL-TRAY exit section (x801..807)</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -9941,7 +9941,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>puller side plates + base + fixed-roller bearing seats + carriage guide slots</t>
+          <t>puller base and side plates with bored Ø8.4 axle seats and east bearing web</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
@@ -9961,12 +9961,12 @@
       </c>
       <c r="G175" t="inlineStr">
         <is>
-          <t>VP1-STAGE4</t>
+          <t>VP1-REFERENCE-FEED</t>
         </is>
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>VP1-STAGE4</t>
+          <t>VP1-REFERENCE-FEED</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
@@ -9981,7 +9981,7 @@
       </c>
       <c r="K175" t="inlineStr">
         <is>
-          <t>Positive stop 1.5 mm and adjustable open nip to 3.0 mm; spring carriage grips nominal 1.75 mm filament - UNQUOTED</t>
+          <t>Ø20 rollers center the filament 11 mm inboard of both roller ends; bearing selection and carriage linear guide still HOLD; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10055,7 +10055,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>nip positive-stop cam block (1.5 mm minimum, 3.0 mm open)</t>
+          <t>underside seat at 1.5 mm roller nip; touches frame/carriage without penetration</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
@@ -10075,12 +10075,12 @@
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-REFERENCE-FEED</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-REFERENCE-FEED</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
@@ -10095,7 +10095,7 @@
       </c>
       <c r="K177" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>Stop attachment and open setting hardware unqualified; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10112,7 +10112,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>puller adjustable roller dia 20 + spring-loaded carriage (guide posts, coil springs, cam stop)</t>
+          <t>puller adjustable roller dia 20 + spring-loaded carriage and guide-post envelopes</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
@@ -10122,7 +10122,7 @@
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>steel; M5 screw</t>
+          <t>steel + springs unselected</t>
         </is>
       </c>
       <c r="F178" t="inlineStr">
@@ -10132,12 +10132,12 @@
       </c>
       <c r="G178" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-REFERENCE-FEED</t>
         </is>
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-REFERENCE-FEED</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
@@ -10152,7 +10152,7 @@
       </c>
       <c r="K178" t="inlineStr">
         <is>
-          <t>Spring-loaded carrier grips 1.5-2.0 mm filament (1.75 nominal, design/parameters.json filament_mm); cam stop range 1.5..3.0 mm - UNQUOTED</t>
+          <t>At modeled minimum gap 1.5 mm the 1.75 mm strand intersects both compliant roller envelopes; actual spring force and guide travel not rated; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10853,7 +10853,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>north transverse screw x224 y235.5..359 feeding the central lane</t>
+          <t>north transverse screw x224 y235.5..359 radius 7.2 flight feeding central lane</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
@@ -10878,7 +10878,7 @@
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>VP1-REFERENCE-FEED</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
@@ -10893,7 +10893,7 @@
       </c>
       <c r="K191" t="inlineStr">
         <is>
-          <t>Dynamic side-belt pickup under verification; UNQUOTED</t>
+          <t>Swept flight reaches previously stranded Ø3 mm envelope near x223/z336.5; actual same-particle pickup untested; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10910,7 +10910,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>south transverse screw x224 y127..228.5 feeding the central lane</t>
+          <t>south transverse screw x224 y127..228.5 radius 7.2 flight feeding central lane</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
@@ -10935,7 +10935,7 @@
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>VP1-REFERENCE-FEED</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
@@ -10950,7 +10950,7 @@
       </c>
       <c r="K192" t="inlineStr">
         <is>
-          <t>Dynamic side-belt pickup under verification; UNQUOTED</t>
+          <t>Floor relief provides swept clearance; flake capture and torque not proven; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -11024,7 +11024,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>central 17 mm tread from x80 to x260 inside the two side loops</t>
+          <t>central 17 mm tread from x80 to x270 inside two side loops</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
@@ -11049,7 +11049,7 @@
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>VP1-REFERENCE-FEED</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
@@ -11064,7 +11064,7 @@
       </c>
       <c r="K194" t="inlineStr">
         <is>
-          <t>Screw pickup unproven; UNQUOTED</t>
+          <t>Extended drum and ramp towards auger inlet; traction and throughflow unproven; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -11081,7 +11081,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>central east r2.3 idler at x260</t>
+          <t>central east r2.05/2.45 idler at x270</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
@@ -11106,7 +11106,7 @@
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>VP1-REFERENCE-FEED</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
@@ -11138,7 +11138,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>SWAP reference-feedstock hopper on FEED-BUF saddle interface (x282..316 y251..299 z145..218); replaces buffer stack for reference runs</t>
+          <t>SWAP hollow side-inlet for reference material on FEED-BUF saddle; not in production assembly</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
@@ -11178,7 +11178,7 @@
       </c>
       <c r="K196" t="inlineStr">
         <is>
-          <t>NOT in production assembly; no interlock credit</t>
+          <t>S2 off; saddle seal/fasteners and flow remain HOLD; no interlock credit; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -11190,12 +11190,12 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>WIND_FLANGE_L</t>
+          <t>WIND_CLUTCH_REF</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>spool flange dia 200 x 3 mm</t>
+          <t>keyed collar + spring envelope + friction washer between driven shaft and loose spool flange</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
@@ -11205,22 +11205,22 @@
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>steel plate 3 mm screening candidate</t>
+          <t>steel collar + friction pad + spring reference</t>
         </is>
       </c>
       <c r="F197" t="inlineStr">
         <is>
-          <t>WINDER_STIFFNESS_SCREEN_PASS_HUB_HOLD</t>
+          <t>TORQUE_LIMIT_UNQUALIFIED</t>
         </is>
       </c>
       <c r="G197" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-REFERENCE-FEED</t>
         </is>
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-REFERENCE-FEED</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
@@ -11235,7 +11235,7 @@
       </c>
       <c r="K197" t="inlineStr">
         <is>
-          <t>20 N assumed rim load; 43.33 MPa/0.194 mm beam screen only; hub bolt balance guard unqualified; unquoted</t>
+          <t>Axial preload/retention and 70 Nmm sensitivity value not physically designed or rated; torque transmission and costs HOLD; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -11247,7 +11247,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>WIND_FLANGE_R</t>
+          <t>WIND_FLANGE_L</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
@@ -11304,12 +11304,12 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>WIND_MOTOR_REF</t>
+          <t>WIND_FLANGE_R</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>spool gearmotor reference (not selected)</t>
+          <t>spool flange dia 200 x 3 mm</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
@@ -11319,12 +11319,12 @@
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>24 V gearmotor MPN unselected</t>
+          <t>steel plate 3 mm screening candidate</t>
         </is>
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t>MOTOR_UNSELECTED</t>
+          <t>WINDER_STIFFNESS_SCREEN_PASS_HUB_HOLD</t>
         </is>
       </c>
       <c r="G199" t="inlineStr">
@@ -11349,7 +11349,7 @@
       </c>
       <c r="K199" t="inlineStr">
         <is>
-          <t>UNQUOTED; known motor floors exceed the 100000 KRW soft limit - not 0</t>
+          <t>20 N assumed rim load; 43.33 MPa/0.194 mm beam screen only; hub bolt balance guard unqualified; unquoted</t>
         </is>
       </c>
     </row>
@@ -11361,12 +11361,12 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>WIND_SPOOL_BEARINGS</t>
+          <t>WIND_MOTOR_REF</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>spool shaft bearing blocks at BOTH shaft ends</t>
+          <t>spool gearmotor reference (not selected)</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
@@ -11376,22 +11376,22 @@
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>steel plate 5 mm + bearing seats</t>
+          <t>24 V gearmotor MPN unselected</t>
         </is>
       </c>
       <c r="F200" t="inlineStr">
         <is>
-          <t>WINDER_UNRATED</t>
+          <t>MOTOR_UNSELECTED</t>
         </is>
       </c>
       <c r="G200" t="inlineStr">
         <is>
-          <t>VP1-STAGE4</t>
+          <t>VP1-STAGE2</t>
         </is>
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>VP1-STAGE4</t>
+          <t>VP1-STAGE3</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
@@ -11406,7 +11406,7 @@
       </c>
       <c r="K200" t="inlineStr">
         <is>
-          <t>VP1 Stage 4 grip redesign: shaft supported at both ends - UNQUOTED</t>
+          <t>UNQUOTED; known motor floors exceed the 100000 KRW soft limit - not 0</t>
         </is>
       </c>
     </row>
@@ -11418,12 +11418,12 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>WIND_SPOOL_DRUM</t>
+          <t>WIND_SPOOL_BEARINGS</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>spool drum dia 70 x 58</t>
+          <t>spool shaft bearing blocks at BOTH shaft ends</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
@@ -11433,7 +11433,7 @@
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>steel tube or printed polymer</t>
+          <t>steel plate 5 mm + bearing seats</t>
         </is>
       </c>
       <c r="F201" t="inlineStr">
@@ -11443,12 +11443,12 @@
       </c>
       <c r="G201" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-STAGE4</t>
         </is>
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-STAGE4</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
@@ -11463,7 +11463,7 @@
       </c>
       <c r="K201" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>VP1 Stage 4 grip redesign: shaft supported at both ends - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -11475,12 +11475,12 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>WIND_SPOOL_SHAFT</t>
+          <t>WIND_SPOOL_DRUM</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>spool shaft dia 16 x 95</t>
+          <t>spool steel drum dia 70 x 58 with loose shaft bore; weld to steel flanges before winding</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
@@ -11490,7 +11490,7 @@
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>C45 candidate</t>
+          <t>steel tube candidate</t>
         </is>
       </c>
       <c r="F202" t="inlineStr">
@@ -11500,12 +11500,12 @@
       </c>
       <c r="G202" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-REFERENCE-FEED</t>
         </is>
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-REFERENCE-FEED</t>
         </is>
       </c>
       <c r="I202" t="inlineStr">
@@ -11520,7 +11520,7 @@
       </c>
       <c r="K202" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>Flange seam and balance unqualified; printed drum would require separate fastener design; friction clutch drives flange rather than loose bore; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -11532,12 +11532,12 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>WIND_TENSIONER</t>
+          <t>WIND_SPOOL_SHAFT</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>slip tensioner post + wrap arm</t>
+          <t>spool shaft dia 16 x 98 with keyed clutch collar seat</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
@@ -11547,7 +11547,7 @@
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>steel</t>
+          <t>C45 candidate</t>
         </is>
       </c>
       <c r="F203" t="inlineStr">
@@ -11577,7 +11577,7 @@
       </c>
       <c r="K203" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>Shaft bearing and key torque rating HOLD; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -11589,12 +11589,12 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>WIND_TRAVERSE_RIDER</t>
+          <t>WIND_TENSIONER</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>traverse rider block + guide eyelet</t>
+          <t>filament path-buffer post + wrap arm</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
@@ -11604,12 +11604,12 @@
       </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t>steel + printed guide</t>
+          <t>steel</t>
         </is>
       </c>
       <c r="F204" t="inlineStr">
         <is>
-          <t>WINDER_UNRATED</t>
+          <t>TENSION_UNRATED</t>
         </is>
       </c>
       <c r="G204" t="inlineStr">
@@ -11634,7 +11634,7 @@
       </c>
       <c r="K204" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>Not a calibrated torque limiter; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -11646,50 +11646,107 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
+          <t>WIND_TRAVERSE_RIDER</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>traverse rider block + guide eyelet</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>steel + printed guide</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>WINDER_UNRATED</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>VP1-STAGE2</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>VP1-STAGE3</t>
+        </is>
+      </c>
+      <c r="I205" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J205" t="inlineStr">
+        <is>
+          <t>UNQUOTED_NOT_ZERO</t>
+        </is>
+      </c>
+      <c r="K205" t="inlineStr">
+        <is>
+          <t>UNQUOTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>vp1_stage1_3</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
           <t>WIND_TRAVERSE_SCREW</t>
         </is>
       </c>
-      <c r="C205" t="inlineStr">
+      <c r="C206" t="inlineStr">
         <is>
           <t>traverse lead screw dia 8 x 80</t>
         </is>
       </c>
-      <c r="D205" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E205" t="inlineStr">
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
         <is>
           <t>steel rod</t>
         </is>
       </c>
-      <c r="F205" t="inlineStr">
+      <c r="F206" t="inlineStr">
         <is>
           <t>WINDER_UNRATED</t>
         </is>
       </c>
-      <c r="G205" t="inlineStr">
+      <c r="G206" t="inlineStr">
         <is>
           <t>VP1-STAGE2</t>
         </is>
       </c>
-      <c r="H205" t="inlineStr">
+      <c r="H206" t="inlineStr">
         <is>
           <t>VP1-STAGE3</t>
         </is>
       </c>
-      <c r="I205" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J205" t="inlineStr">
+      <c r="I206" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J206" t="inlineStr">
         <is>
           <t>UNQUOTED_NOT_ZERO</t>
         </is>
       </c>
-      <c r="K205" t="inlineStr">
+      <c r="K206" t="inlineStr">
         <is>
           <t>UNQUOTED</t>
         </is>

</xml_diff>

<commit_message>
VP1: support downstream load paths and hollow spool
</commit_message>
<xml_diff>
--- a/c2.1/bom/system_bom.xlsx
+++ b/c2.1/bom/system_bom.xlsx
@@ -9936,12 +9936,12 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>PULL_FRAME</t>
+          <t>PULL_COOL_MOUNT</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>puller base and side plates with bored Ø8.4 axle seats and east bearing web</t>
+          <t>rear-frame steel tube rack with tray ledge and puller fastener holes</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
@@ -9951,12 +9951,12 @@
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>steel plate 5 mm + 3 mm</t>
+          <t>steel tube + plate/bar candidate</t>
         </is>
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>NIP_RATING_HOLD</t>
+          <t>NIP_SUPPORT_HOLD</t>
         </is>
       </c>
       <c r="G175" t="inlineStr">
@@ -9981,7 +9981,7 @@
       </c>
       <c r="K175" t="inlineStr">
         <is>
-          <t>Ø20 rollers center the filament 11 mm inboard of both roller ends; bearing selection and carriage linear guide still HOLD; UNQUOTED</t>
+          <t>Contacts rear FR-2040-400_002, COOL-TRAY_001 underside and PULL_FRAME base; bolts, welds, tray connection and load ratings unselected; unquoted NOT zero</t>
         </is>
       </c>
     </row>
@@ -9993,12 +9993,12 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>PULL_MOTOR_REF</t>
+          <t>PULL_FRAME</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>puller gearmotor reference (not selected)</t>
+          <t>puller base and side plates with bored Ø8.4 axle seats and east bearing web</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -10008,22 +10008,22 @@
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>24 V gearmotor MPN unselected</t>
+          <t>steel plate 5 mm + 3 mm</t>
         </is>
       </c>
       <c r="F176" t="inlineStr">
         <is>
-          <t>MOTOR_UNSELECTED</t>
+          <t>NIP_RATING_HOLD</t>
         </is>
       </c>
       <c r="G176" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-REFERENCE-FEED</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-REFERENCE-FEED</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
@@ -10038,7 +10038,7 @@
       </c>
       <c r="K176" t="inlineStr">
         <is>
-          <t>UNQUOTED; known motor floors exceed the 100000 KRW soft limit - not 0</t>
+          <t>Ø20 rollers center the filament 11 mm inboard of both roller ends; bearing selection and carriage linear guide still HOLD; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10050,12 +10050,12 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>PULL_NIP_STOP</t>
+          <t>PULL_MOTOR_REF</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>underside seat at 1.5 mm roller nip; touches frame/carriage without penetration</t>
+          <t>puller gearmotor reference (not selected)</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
@@ -10065,22 +10065,22 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>steel</t>
+          <t>24 V gearmotor MPN unselected</t>
         </is>
       </c>
       <c r="F177" t="inlineStr">
         <is>
-          <t>NIP_RATING_HOLD</t>
+          <t>MOTOR_UNSELECTED</t>
         </is>
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t>VP1-REFERENCE-FEED</t>
+          <t>VP1-STAGE2</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>VP1-REFERENCE-FEED</t>
+          <t>VP1-STAGE3</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
@@ -10095,7 +10095,7 @@
       </c>
       <c r="K177" t="inlineStr">
         <is>
-          <t>Stop attachment and open setting hardware unqualified; UNQUOTED</t>
+          <t>UNQUOTED; known motor floors exceed the 100000 KRW soft limit - not 0</t>
         </is>
       </c>
     </row>
@@ -10107,12 +10107,12 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>PULL_ROLLER_ADJ</t>
+          <t>PULL_NIP_STOP</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>puller adjustable roller dia 20 + spring-loaded carriage and guide-post envelopes</t>
+          <t>underside seat at 1.5 mm roller nip; touches frame/carriage without penetration</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
@@ -10122,7 +10122,7 @@
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>steel + springs unselected</t>
+          <t>steel</t>
         </is>
       </c>
       <c r="F178" t="inlineStr">
@@ -10152,7 +10152,7 @@
       </c>
       <c r="K178" t="inlineStr">
         <is>
-          <t>At modeled minimum gap 1.5 mm the 1.75 mm strand intersects both compliant roller envelopes; actual spring force and guide travel not rated; UNQUOTED</t>
+          <t>Stop attachment and open setting hardware unqualified; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10164,12 +10164,12 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>PULL_ROLLER_FIXED</t>
+          <t>PULL_ROLLER_ADJ</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>puller drive roller dia 20 x 22</t>
+          <t>puller adjustable roller dia 20 + spring-loaded carriage and guide-post envelopes</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
@@ -10179,7 +10179,7 @@
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>steel; knurl or rubber per TPU grip</t>
+          <t>steel + springs unselected</t>
         </is>
       </c>
       <c r="F179" t="inlineStr">
@@ -10189,12 +10189,12 @@
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-REFERENCE-FEED</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-REFERENCE-FEED</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
@@ -10209,7 +10209,7 @@
       </c>
       <c r="K179" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>At modeled minimum gap 1.5 mm the 1.75 mm strand intersects both compliant roller envelopes; actual spring force and guide travel not rated; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10221,37 +10221,37 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>S1_BELT</t>
+          <t>PULL_ROLLER_FIXED</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>two side-loop treads over x80..219; y163.5..223.2 and 240.8..323.5</t>
+          <t>puller drive roller dia 20 x 22</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>polymer belt with steel-supported drums</t>
+          <t>steel; knurl or rubber per TPU grip</t>
         </is>
       </c>
       <c r="F180" t="inlineStr">
         <is>
-          <t>TRANSFER_UNRATED</t>
+          <t>NIP_RATING_HOLD</t>
         </is>
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>VP1-STAGE2</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>VP1-STAGE3</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
@@ -10266,7 +10266,7 @@
       </c>
       <c r="K180" t="inlineStr">
         <is>
-          <t>Friction and tension unrated; UNQUOTED</t>
+          <t>UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10278,22 +10278,22 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>S1_BELT_BEARINGS</t>
+          <t>S1_BELT</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>four belt shaft support rings in the side rails</t>
+          <t>two side-loop treads over x80..219; y163.5..223.2 and 240.8..323.5</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>steel bearing seats</t>
+          <t>polymer belt with steel-supported drums</t>
         </is>
       </c>
       <c r="F181" t="inlineStr">
@@ -10323,7 +10323,7 @@
       </c>
       <c r="K181" t="inlineStr">
         <is>
-          <t>Bearing selection and loads unqualified; UNQUOTED</t>
+          <t>Friction and tension unrated; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10335,12 +10335,12 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>S1_BELT_CHAIN</t>
+          <t>S1_BELT_BEARINGS</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>#35 chain from S1B 24T to west belt 12T</t>
+          <t>four belt shaft support rings in the side rails</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
@@ -10350,7 +10350,7 @@
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>ANSI35 steel chain</t>
+          <t>steel bearing seats</t>
         </is>
       </c>
       <c r="F182" t="inlineStr">
@@ -10380,7 +10380,7 @@
       </c>
       <c r="K182" t="inlineStr">
         <is>
-          <t>Tension and strength unrated; UNQUOTED</t>
+          <t>Bearing selection and loads unqualified; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10392,12 +10392,12 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>S1_BELT_DRIVE</t>
+          <t>S1_BELT_CHAIN</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>common waisted drive drum at x80; separate r3.8 side and r2.3 central tread seats</t>
+          <t>#35 chain from S1B 24T to west belt 12T</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
@@ -10407,7 +10407,7 @@
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>steel shaft and drums</t>
+          <t>ANSI35 steel chain</t>
         </is>
       </c>
       <c r="F183" t="inlineStr">
@@ -10437,7 +10437,7 @@
       </c>
       <c r="K183" t="inlineStr">
         <is>
-          <t>S1B chain-driven; torque and bearing load unrated; UNQUOTED</t>
+          <t>Tension and strength unrated; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10449,12 +10449,12 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>S1_BELT_FOLLOWER</t>
+          <t>S1_BELT_DRIVE</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>12T sprocket on the west belt driver</t>
+          <t>common waisted drive drum at x80; separate r3.8 side and r2.3 central tread seats</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
@@ -10464,7 +10464,7 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>ANSI35 steel sprocket</t>
+          <t>steel shaft and drums</t>
         </is>
       </c>
       <c r="F184" t="inlineStr">
@@ -10494,7 +10494,7 @@
       </c>
       <c r="K184" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>S1B chain-driven; torque and bearing load unrated; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10506,12 +10506,12 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>S1_BELT_IDLER</t>
+          <t>S1_BELT_FOLLOWER</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>two split side idler drums at x219 leaving the central transfer corridor open</t>
+          <t>12T sprocket on the west belt driver</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
@@ -10521,7 +10521,7 @@
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>steel journals and drums</t>
+          <t>ANSI35 steel sprocket</t>
         </is>
       </c>
       <c r="F185" t="inlineStr">
@@ -10551,7 +10551,7 @@
       </c>
       <c r="K185" t="inlineStr">
         <is>
-          <t>Two independent journal halves; UNQUOTED</t>
+          <t>UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10563,12 +10563,12 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>S1_SWEEP_BEARINGS</t>
+          <t>S1_BELT_IDLER</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>two separated sweep bearing rings in the pan rails</t>
+          <t>two split side idler drums at x219 leaving the central transfer corridor open</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
@@ -10578,7 +10578,7 @@
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>steel bearing seats</t>
+          <t>steel journals and drums</t>
         </is>
       </c>
       <c r="F186" t="inlineStr">
@@ -10608,7 +10608,7 @@
       </c>
       <c r="K186" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>Two independent journal halves; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10620,12 +10620,12 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>S1_SWEEP_GEAR_DRUM_N</t>
+          <t>S1_SWEEP_BEARINGS</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>12T gear on the north east belt idler</t>
+          <t>two separated sweep bearing rings in the pan rails</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
@@ -10635,7 +10635,7 @@
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>steel gear</t>
+          <t>steel bearing seats</t>
         </is>
       </c>
       <c r="F187" t="inlineStr">
@@ -10677,12 +10677,12 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>S1_SWEEP_GEAR_DRUM_S</t>
+          <t>S1_SWEEP_GEAR_DRUM_N</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>12T gear on the south east belt idler</t>
+          <t>12T gear on the north east belt idler</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
@@ -10734,12 +10734,12 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>S1_SWEEP_GEAR_N</t>
+          <t>S1_SWEEP_GEAR_DRUM_S</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>12T gear on the north sweep shaft</t>
+          <t>12T gear on the south east belt idler</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
@@ -10791,12 +10791,12 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>S1_SWEEP_GEAR_S</t>
+          <t>S1_SWEEP_GEAR_N</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>12T gear on the south sweep shaft</t>
+          <t>12T gear on the north sweep shaft</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
@@ -10848,12 +10848,12 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>S1_SWEEP_NORTH</t>
+          <t>S1_SWEEP_GEAR_S</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>north transverse screw x224 y235.5..359 radius 7.2 flight feeding central lane</t>
+          <t>12T gear on the south sweep shaft</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
@@ -10863,7 +10863,7 @@
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>steel shaft and flight</t>
+          <t>steel gear</t>
         </is>
       </c>
       <c r="F191" t="inlineStr">
@@ -10878,7 +10878,7 @@
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>VP1-REFERENCE-FEED</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
@@ -10893,7 +10893,7 @@
       </c>
       <c r="K191" t="inlineStr">
         <is>
-          <t>Swept flight reaches previously stranded Ø3 mm envelope near x223/z336.5; actual same-particle pickup untested; UNQUOTED</t>
+          <t>UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10905,12 +10905,12 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>S1_SWEEP_SOUTH</t>
+          <t>S1_SWEEP_NORTH</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>south transverse screw x224 y127..228.5 radius 7.2 flight feeding central lane</t>
+          <t>north transverse screw x224 y235.5..359 radius 7.2 flight feeding central lane</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
@@ -10950,7 +10950,7 @@
       </c>
       <c r="K192" t="inlineStr">
         <is>
-          <t>Floor relief provides swept clearance; flake capture and torque not proven; UNQUOTED</t>
+          <t>Swept flight reaches previously stranded Ø3 mm envelope near x223/z336.5; actual same-particle pickup untested; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10962,12 +10962,12 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>S1_TRANSFER_BEARINGS</t>
+          <t>S1_SWEEP_SOUTH</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>two central idler support rings</t>
+          <t>south transverse screw x224 y127..228.5 radius 7.2 flight feeding central lane</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
@@ -10977,7 +10977,7 @@
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>steel bearing seats</t>
+          <t>steel shaft and flight</t>
         </is>
       </c>
       <c r="F193" t="inlineStr">
@@ -10992,7 +10992,7 @@
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>VP1-REFERENCE-FEED</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
@@ -11007,7 +11007,7 @@
       </c>
       <c r="K193" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>Floor relief provides swept clearance; flake capture and torque not proven; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -11019,12 +11019,12 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>S1_TRANSFER_BELT</t>
+          <t>S1_TRANSFER_BEARINGS</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>central 17 mm tread from x80 to x270 inside two side loops</t>
+          <t>two central idler support rings</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
@@ -11034,7 +11034,7 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>polymer belt</t>
+          <t>steel bearing seats</t>
         </is>
       </c>
       <c r="F194" t="inlineStr">
@@ -11049,7 +11049,7 @@
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>VP1-REFERENCE-FEED</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
@@ -11064,7 +11064,7 @@
       </c>
       <c r="K194" t="inlineStr">
         <is>
-          <t>Extended drum and ramp towards auger inlet; traction and throughflow unproven; UNQUOTED</t>
+          <t>UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -11076,12 +11076,12 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>S1_TRANSFER_IDLER</t>
+          <t>S1_TRANSFER_BELT</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>central east r2.05/2.45 idler at x270</t>
+          <t>central 17 mm tread from x80 to x270 inside two side loops</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
@@ -11091,7 +11091,7 @@
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>steel drum</t>
+          <t>polymer belt</t>
         </is>
       </c>
       <c r="F195" t="inlineStr">
@@ -11121,7 +11121,7 @@
       </c>
       <c r="K195" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>Extended drum and ramp towards auger inlet; traction and throughflow unproven; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -11133,12 +11133,12 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>SERVICE-HOPPER</t>
+          <t>S1_TRANSFER_IDLER</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>SWAP hollow side-inlet for reference material on FEED-BUF saddle; not in production assembly</t>
+          <t>central east r2.05/2.45 idler at x270</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
@@ -11148,22 +11148,22 @@
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>steel sheet 3 mm</t>
+          <t>steel drum</t>
         </is>
       </c>
       <c r="F196" t="inlineStr">
         <is>
-          <t>SWAP_PART_NO_INTERLOCK</t>
+          <t>TRANSFER_UNRATED</t>
         </is>
       </c>
       <c r="G196" t="inlineStr">
         <is>
-          <t>VP1-STAGE6</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>VP1-STAGE6</t>
+          <t>VP1-REFERENCE-FEED</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
@@ -11178,7 +11178,7 @@
       </c>
       <c r="K196" t="inlineStr">
         <is>
-          <t>S2 off; saddle seal/fasteners and flow remain HOLD; no interlock credit; UNQUOTED</t>
+          <t>UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -11190,12 +11190,12 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>WIND_CLUTCH_REF</t>
+          <t>SERVICE-HOPPER</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>keyed collar + spring envelope + friction washer between driven shaft and loose spool flange</t>
+          <t>SWAP hollow side-inlet for reference material on FEED-BUF saddle; not in production assembly</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
@@ -11205,22 +11205,22 @@
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>steel collar + friction pad + spring reference</t>
+          <t>steel sheet 3 mm</t>
         </is>
       </c>
       <c r="F197" t="inlineStr">
         <is>
-          <t>TORQUE_LIMIT_UNQUALIFIED</t>
+          <t>SWAP_PART_NO_INTERLOCK</t>
         </is>
       </c>
       <c r="G197" t="inlineStr">
         <is>
-          <t>VP1-REFERENCE-FEED</t>
+          <t>VP1-STAGE6</t>
         </is>
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>VP1-REFERENCE-FEED</t>
+          <t>VP1-STAGE6</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
@@ -11235,7 +11235,7 @@
       </c>
       <c r="K197" t="inlineStr">
         <is>
-          <t>Axial preload/retention and 70 Nmm sensitivity value not physically designed or rated; torque transmission and costs HOLD; UNQUOTED</t>
+          <t>S2 off; saddle seal/fasteners and flow remain HOLD; no interlock credit; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -11247,12 +11247,12 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>WIND_FLANGE_L</t>
+          <t>WIND_CLUTCH_REF</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>spool flange dia 200 x 3 mm</t>
+          <t>keyed collar + spring envelope + friction washer between driven shaft and loose spool flange</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
@@ -11262,22 +11262,22 @@
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>steel plate 3 mm screening candidate</t>
+          <t>steel collar + friction pad + spring reference</t>
         </is>
       </c>
       <c r="F198" t="inlineStr">
         <is>
-          <t>WINDER_STIFFNESS_SCREEN_PASS_HUB_HOLD</t>
+          <t>TORQUE_LIMIT_UNQUALIFIED</t>
         </is>
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-REFERENCE-FEED</t>
         </is>
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-REFERENCE-FEED</t>
         </is>
       </c>
       <c r="I198" t="inlineStr">
@@ -11292,7 +11292,7 @@
       </c>
       <c r="K198" t="inlineStr">
         <is>
-          <t>20 N assumed rim load; 43.33 MPa/0.194 mm beam screen only; hub bolt balance guard unqualified; unquoted</t>
+          <t>Axial preload/retention and 70 Nmm sensitivity value not physically designed or rated; torque transmission and costs HOLD; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -11304,7 +11304,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>WIND_FLANGE_R</t>
+          <t>WIND_FLANGE_L</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
@@ -11361,12 +11361,12 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>WIND_MOTOR_REF</t>
+          <t>WIND_FLANGE_R</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>spool gearmotor reference (not selected)</t>
+          <t>spool flange dia 200 x 3 mm</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
@@ -11376,12 +11376,12 @@
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>24 V gearmotor MPN unselected</t>
+          <t>steel plate 3 mm screening candidate</t>
         </is>
       </c>
       <c r="F200" t="inlineStr">
         <is>
-          <t>MOTOR_UNSELECTED</t>
+          <t>WINDER_STIFFNESS_SCREEN_PASS_HUB_HOLD</t>
         </is>
       </c>
       <c r="G200" t="inlineStr">
@@ -11406,7 +11406,7 @@
       </c>
       <c r="K200" t="inlineStr">
         <is>
-          <t>UNQUOTED; known motor floors exceed the 100000 KRW soft limit - not 0</t>
+          <t>20 N assumed rim load; 43.33 MPa/0.194 mm beam screen only; hub bolt balance guard unqualified; unquoted</t>
         </is>
       </c>
     </row>
@@ -11418,12 +11418,12 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>WIND_SPOOL_BEARINGS</t>
+          <t>WIND_MOTOR_REF</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>spool shaft bearing blocks at BOTH shaft ends</t>
+          <t>spool gearmotor reference (not selected)</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
@@ -11433,22 +11433,22 @@
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>steel plate 5 mm + bearing seats</t>
+          <t>24 V gearmotor MPN unselected</t>
         </is>
       </c>
       <c r="F201" t="inlineStr">
         <is>
-          <t>WINDER_UNRATED</t>
+          <t>MOTOR_UNSELECTED</t>
         </is>
       </c>
       <c r="G201" t="inlineStr">
         <is>
-          <t>VP1-STAGE4</t>
+          <t>VP1-STAGE2</t>
         </is>
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>VP1-STAGE4</t>
+          <t>VP1-STAGE3</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
@@ -11463,7 +11463,7 @@
       </c>
       <c r="K201" t="inlineStr">
         <is>
-          <t>VP1 Stage 4 grip redesign: shaft supported at both ends - UNQUOTED</t>
+          <t>UNQUOTED; known motor floors exceed the 100000 KRW soft limit - not 0</t>
         </is>
       </c>
     </row>
@@ -11475,12 +11475,12 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>WIND_SPOOL_DRUM</t>
+          <t>WIND_MOUNT</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>spool steel drum dia 70 x 58 with loose shaft bore; weld to steel flanges before winding</t>
+          <t>steel cantilever with front-profile face plate, two bearing rails and motor bed</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
@@ -11490,12 +11490,12 @@
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>steel tube candidate</t>
+          <t>steel plate/bar 4-8 mm + M5 candidate clearances</t>
         </is>
       </c>
       <c r="F202" t="inlineStr">
         <is>
-          <t>WINDER_UNRATED</t>
+          <t>WINDER_JOINT_HOLD</t>
         </is>
       </c>
       <c r="G202" t="inlineStr">
@@ -11520,7 +11520,7 @@
       </c>
       <c r="K202" t="inlineStr">
         <is>
-          <t>Flange seam and balance unqualified; printed drum would require separate fastener design; friction clutch drives flange rather than loose bore; UNQUOTED</t>
+          <t>BRep face contact to FR-2020-400_001 and bearing/motor seats; profile slot, fastener/weld sizes, cantilever stiffness, vibration and guard HOLD; no quote - NOT 0</t>
         </is>
       </c>
     </row>
@@ -11532,12 +11532,12 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>WIND_SPOOL_SHAFT</t>
+          <t>WIND_SPOOL_BEARINGS</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>spool shaft dia 16 x 98 with keyed clutch collar seat</t>
+          <t>spool shaft bearing blocks at BOTH shaft ends</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
@@ -11547,7 +11547,7 @@
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>C45 candidate</t>
+          <t>steel plate 5 mm + bearing seats</t>
         </is>
       </c>
       <c r="F203" t="inlineStr">
@@ -11557,12 +11557,12 @@
       </c>
       <c r="G203" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-STAGE4</t>
         </is>
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-STAGE4</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
@@ -11577,7 +11577,7 @@
       </c>
       <c r="K203" t="inlineStr">
         <is>
-          <t>Shaft bearing and key torque rating HOLD; UNQUOTED</t>
+          <t>VP1 Stage 4 grip redesign: shaft supported at both ends - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -11589,12 +11589,12 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>WIND_TENSIONER</t>
+          <t>WIND_SPOOL_DRUM</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>filament path-buffer post + wrap arm</t>
+          <t>spool dia 70 x 58 steel tube with 2 mm wall and two 3 mm internal annular webs; weld to steel flanges before winding</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
@@ -11604,22 +11604,22 @@
       </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t>steel</t>
+          <t>steel tube + steel webs candidate</t>
         </is>
       </c>
       <c r="F204" t="inlineStr">
         <is>
-          <t>TENSION_UNRATED</t>
+          <t>WINDER_UNRATED</t>
         </is>
       </c>
       <c r="G204" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-REFERENCE-FEED</t>
         </is>
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-REFERENCE-FEED</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
@@ -11634,7 +11634,7 @@
       </c>
       <c r="K204" t="inlineStr">
         <is>
-          <t>Not a calibrated torque limiter; UNQUOTED</t>
+          <t>Web-to-tube and flange seams and balance unqualified; loose Ø17 web bores clear Ø16 shaft; friction clutch drives flange; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -11646,12 +11646,12 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>WIND_TRAVERSE_RIDER</t>
+          <t>WIND_SPOOL_SHAFT</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>traverse rider block + guide eyelet</t>
+          <t>spool shaft dia 16 x 98 with keyed clutch collar seat</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
@@ -11661,7 +11661,7 @@
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t>steel + printed guide</t>
+          <t>C45 candidate</t>
         </is>
       </c>
       <c r="F205" t="inlineStr">
@@ -11691,7 +11691,7 @@
       </c>
       <c r="K205" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>Shaft bearing and key torque rating HOLD; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -11703,50 +11703,164 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
+          <t>WIND_TENSIONER</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>filament path-buffer post + wrap arm</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>steel</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>TENSION_UNRATED</t>
+        </is>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>VP1-STAGE2</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>VP1-STAGE3</t>
+        </is>
+      </c>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J206" t="inlineStr">
+        <is>
+          <t>UNQUOTED_NOT_ZERO</t>
+        </is>
+      </c>
+      <c r="K206" t="inlineStr">
+        <is>
+          <t>Not a calibrated torque limiter; UNQUOTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>vp1_stage1_3</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>WIND_TRAVERSE_RIDER</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>traverse rider block + guide eyelet</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>steel + printed guide</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>WINDER_UNRATED</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>VP1-STAGE2</t>
+        </is>
+      </c>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>VP1-STAGE3</t>
+        </is>
+      </c>
+      <c r="I207" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J207" t="inlineStr">
+        <is>
+          <t>UNQUOTED_NOT_ZERO</t>
+        </is>
+      </c>
+      <c r="K207" t="inlineStr">
+        <is>
+          <t>UNQUOTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>vp1_stage1_3</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
           <t>WIND_TRAVERSE_SCREW</t>
         </is>
       </c>
-      <c r="C206" t="inlineStr">
+      <c r="C208" t="inlineStr">
         <is>
           <t>traverse lead screw dia 8 x 80</t>
         </is>
       </c>
-      <c r="D206" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E206" t="inlineStr">
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
         <is>
           <t>steel rod</t>
         </is>
       </c>
-      <c r="F206" t="inlineStr">
+      <c r="F208" t="inlineStr">
         <is>
           <t>WINDER_UNRATED</t>
         </is>
       </c>
-      <c r="G206" t="inlineStr">
+      <c r="G208" t="inlineStr">
         <is>
           <t>VP1-STAGE2</t>
         </is>
       </c>
-      <c r="H206" t="inlineStr">
+      <c r="H208" t="inlineStr">
         <is>
           <t>VP1-STAGE3</t>
         </is>
       </c>
-      <c r="I206" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J206" t="inlineStr">
+      <c r="I208" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J208" t="inlineStr">
         <is>
           <t>UNQUOTED_NOT_ZERO</t>
         </is>
       </c>
-      <c r="K206" t="inlineStr">
+      <c r="K208" t="inlineStr">
         <is>
           <t>UNQUOTED</t>
         </is>

</xml_diff>

<commit_message>
VP1: retain winding spool axially in candidate CAD
</commit_message>
<xml_diff>
--- a/c2.1/bom/system_bom.xlsx
+++ b/c2.1/bom/system_bom.xlsx
@@ -11292,7 +11292,7 @@
       </c>
       <c r="K198" t="inlineStr">
         <is>
-          <t>Axial preload/retention and 70 Nmm sensitivity value not physically designed or rated; torque transmission and costs HOLD; UNQUOTED</t>
+          <t>Separate groove-backed retention closes candidate axial path; actual spring compression/preload and 70 Nmm sensitivity value not rated; torque transmission and costs HOLD; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -11646,12 +11646,12 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>WIND_SPOOL_SHAFT</t>
+          <t>WIND_SPOOL_RETENTION</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>spool shaft dia 16 x 98 with keyed clutch collar seat</t>
+          <t>two split external rings in shaft grooves plus right loose-flange thrust washer</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
@@ -11661,22 +11661,22 @@
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t>C45 candidate</t>
+          <t>steel ring + washer candidate</t>
         </is>
       </c>
       <c r="F205" t="inlineStr">
         <is>
-          <t>WINDER_UNRATED</t>
+          <t>AXIAL_PATH_GEOMETRY_ONLY</t>
         </is>
       </c>
       <c r="G205" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-REFERENCE-FEED</t>
         </is>
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-REFERENCE-FEED</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
@@ -11691,7 +11691,7 @@
       </c>
       <c r="K205" t="inlineStr">
         <is>
-          <t>Shaft bearing and key torque rating HOLD; UNQUOTED</t>
+          <t>Rings y96..97 and y168..169; washer y167..168; collar/spring/flanges contact nominally with no rated preload. Ring size/tolerance/fatigue/axial capacity and quote HOLD; unquoted NOT zero</t>
         </is>
       </c>
     </row>
@@ -11703,12 +11703,12 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>WIND_TENSIONER</t>
+          <t>WIND_SPOOL_SHAFT</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>filament path-buffer post + wrap arm</t>
+          <t>spool shaft dia 16 x 98 with keyed clutch collar seat and two 1 mm candidate external-ring grooves</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
@@ -11718,12 +11718,12 @@
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t>steel</t>
+          <t>C45 candidate</t>
         </is>
       </c>
       <c r="F206" t="inlineStr">
         <is>
-          <t>TENSION_UNRATED</t>
+          <t>WINDER_UNRATED</t>
         </is>
       </c>
       <c r="G206" t="inlineStr">
@@ -11748,7 +11748,7 @@
       </c>
       <c r="K206" t="inlineStr">
         <is>
-          <t>Not a calibrated torque limiter; UNQUOTED</t>
+          <t>Groove root radius 7.2 mm at y96..97 and y168..169; fatigue and ring groove standard HOLD; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -11760,12 +11760,12 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>WIND_TRAVERSE_RIDER</t>
+          <t>WIND_TENSIONER</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>traverse rider block + guide eyelet</t>
+          <t>filament path-buffer post + wrap arm</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
@@ -11775,12 +11775,12 @@
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t>steel + printed guide</t>
+          <t>steel</t>
         </is>
       </c>
       <c r="F207" t="inlineStr">
         <is>
-          <t>WINDER_UNRATED</t>
+          <t>TENSION_UNRATED</t>
         </is>
       </c>
       <c r="G207" t="inlineStr">
@@ -11805,7 +11805,7 @@
       </c>
       <c r="K207" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>Not a calibrated torque limiter; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -11817,50 +11817,107 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
+          <t>WIND_TRAVERSE_RIDER</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>traverse rider block + guide eyelet</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>steel + printed guide</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>WINDER_UNRATED</t>
+        </is>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>VP1-STAGE2</t>
+        </is>
+      </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>VP1-STAGE3</t>
+        </is>
+      </c>
+      <c r="I208" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J208" t="inlineStr">
+        <is>
+          <t>UNQUOTED_NOT_ZERO</t>
+        </is>
+      </c>
+      <c r="K208" t="inlineStr">
+        <is>
+          <t>UNQUOTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>vp1_stage1_3</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
           <t>WIND_TRAVERSE_SCREW</t>
         </is>
       </c>
-      <c r="C208" t="inlineStr">
+      <c r="C209" t="inlineStr">
         <is>
           <t>traverse lead screw dia 8 x 80</t>
         </is>
       </c>
-      <c r="D208" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E208" t="inlineStr">
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
         <is>
           <t>steel rod</t>
         </is>
       </c>
-      <c r="F208" t="inlineStr">
+      <c r="F209" t="inlineStr">
         <is>
           <t>WINDER_UNRATED</t>
         </is>
       </c>
-      <c r="G208" t="inlineStr">
+      <c r="G209" t="inlineStr">
         <is>
           <t>VP1-STAGE2</t>
         </is>
       </c>
-      <c r="H208" t="inlineStr">
+      <c r="H209" t="inlineStr">
         <is>
           <t>VP1-STAGE3</t>
         </is>
       </c>
-      <c r="I208" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J208" t="inlineStr">
+      <c r="I209" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J209" t="inlineStr">
         <is>
           <t>UNQUOTED_NOT_ZERO</t>
         </is>
       </c>
-      <c r="K208" t="inlineStr">
+      <c r="K209" t="inlineStr">
         <is>
           <t>UNQUOTED</t>
         </is>

</xml_diff>

<commit_message>
VP1: size spool retention to catalog ring envelope
</commit_message>
<xml_diff>
--- a/c2.1/bom/system_bom.xlsx
+++ b/c2.1/bom/system_bom.xlsx
@@ -11252,7 +11252,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>keyed collar + spring envelope + friction washer between driven shaft and loose spool flange</t>
+          <t>keyed collar + unselected 1 mm spring envelope + friction washer between driven shaft and loose spool flange</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
@@ -11262,7 +11262,7 @@
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>steel collar + friction pad + spring reference</t>
+          <t>steel collar + friction pad + spring unselected</t>
         </is>
       </c>
       <c r="F198" t="inlineStr">
@@ -11292,7 +11292,7 @@
       </c>
       <c r="K198" t="inlineStr">
         <is>
-          <t>Separate groove-backed retention closes candidate axial path; actual spring compression/preload and 70 Nmm sensitivity value not rated; torque transmission and costs HOLD; UNQUOTED</t>
+          <t>Smalley SSB-0087 clears dia16 shaft but its published 1.57 mm work height exceeds current 1 mm seat by 0.57 mm; solid height/force there unknown. Cannot assign the 62.3 N vendor work-point load or 70 Nmm model torque to assembly; no selected spring or quote</t>
         </is>
       </c>
     </row>
@@ -11651,7 +11651,7 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>two split external rings in shaft grooves plus right loose-flange thrust washer</t>
+          <t>two ES-16 nominal external-ring envelopes plus loose-flange OD30/ID16.2 thrust washer</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
@@ -11661,12 +11661,12 @@
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t>steel ring + washer candidate</t>
+          <t>ring spring steel candidate + steel washer</t>
         </is>
       </c>
       <c r="F205" t="inlineStr">
         <is>
-          <t>AXIAL_PATH_GEOMETRY_ONLY</t>
+          <t>AXIAL_FLOAT_PRELOAD_HOLD</t>
         </is>
       </c>
       <c r="G205" t="inlineStr">
@@ -11691,7 +11691,7 @@
       </c>
       <c r="K205" t="inlineStr">
         <is>
-          <t>Rings y96..97 and y168..169; washer y167..168; collar/spring/flanges contact nominally with no rated preload. Ring size/tolerance/fatigue/axial capacity and quote HOLD; unquoted NOT zero</t>
+          <t>Smalley ES-16 two-turn supplier detail unmodeled; 15.02 mm groove dia and 1.00 +0.08 mm width; nominal 0.89 +/-0.05 mm ring thickness and 1.40 +0.08/-0.13 radial wall. Groove clearance 0.06..0.24 mm per ring (two up to 0.48 mm) excludes rated clamp; maker groove yield 3820 N assumes 45000 psi shaft yield/SF2 and is NOT a PPR rating. MPN dimension reference only; installed fit/thrust/fatigue/landed price HOLD; unquoted NOT zero</t>
         </is>
       </c>
     </row>
@@ -11708,7 +11708,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>spool shaft dia 16 x 98 with keyed clutch collar seat and two 1 mm candidate external-ring grooves</t>
+          <t>spool shaft dia 16 x 98 with keyed clutch collar seat and two ES-16 dimensional-candidate 1 mm grooves</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
@@ -11728,12 +11728,12 @@
       </c>
       <c r="G206" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-REFERENCE-FEED</t>
         </is>
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-REFERENCE-FEED</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">
@@ -11748,7 +11748,7 @@
       </c>
       <c r="K206" t="inlineStr">
         <is>
-          <t>Groove root radius 7.2 mm at y96..97 and y168..169; fatigue and ring groove standard HOLD; UNQUOTED</t>
+          <t>Groove nominal diameter 15.02 mm at y96..97 and y168..169; supplier Dg tolerance +/-0.075 mm; shaft fatigue/actual ring procurement HOLD; UNQUOTED</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Separate puller idler motion and qualify digital nip geometry
</commit_message>
<xml_diff>
--- a/c2.1/bom/system_bom.xlsx
+++ b/c2.1/bom/system_bom.xlsx
@@ -9998,7 +9998,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>puller base and side plates with bored Ø8.4 axle seats and east bearing web</t>
+          <t>puller base and two Ø8.4 drive seats with slotted idler-axle plates, vertical Ø5 guides and spring caps</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -10008,7 +10008,7 @@
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>steel plate 5 mm + 3 mm</t>
+          <t>steel plate + guide rod candidates</t>
         </is>
       </c>
       <c r="F176" t="inlineStr">
@@ -10038,7 +10038,7 @@
       </c>
       <c r="K176" t="inlineStr">
         <is>
-          <t>Ø20 rollers center the filament 11 mm inboard of both roller ends; bearing selection and carriage linear guide still HOLD; UNQUOTED</t>
+          <t>1.5 mm idler translation has geometric clearance; bearing inserts and side-plate/cap/guide joints not selected; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10050,12 +10050,12 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>PULL_MOTOR_REF</t>
+          <t>PULL_IDLER_CARRIAGE</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>puller gearmotor reference (not selected)</t>
+          <t>two translating axle bearing seats joined behind roller</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
@@ -10065,22 +10065,22 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>24 V gearmotor MPN unselected</t>
+          <t>steel plate candidate</t>
         </is>
       </c>
       <c r="F177" t="inlineStr">
         <is>
-          <t>MOTOR_UNSELECTED</t>
+          <t>NIP_RATING_HOLD</t>
         </is>
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-REFERENCE-FEED</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-REFERENCE-FEED</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
@@ -10095,7 +10095,7 @@
       </c>
       <c r="K177" t="inlineStr">
         <is>
-          <t>UNQUOTED; known motor floors exceed the 100000 KRW soft limit - not 0</t>
+          <t>0..1.5 mm vertical stroke on two Ø5 guides with Ø5.2 sliding bores; tolerances/racking and fatigue unqualified; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10107,22 +10107,22 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>PULL_NIP_STOP</t>
+          <t>PULL_IDLER_SPRINGS</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>underside seat at 1.5 mm roller nip; touches frame/carriage without penetration</t>
+          <t>two vertical compression spring space envelopes</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>steel</t>
+          <t>springs unselected</t>
         </is>
       </c>
       <c r="F178" t="inlineStr">
@@ -10152,7 +10152,7 @@
       </c>
       <c r="K178" t="inlineStr">
         <is>
-          <t>Stop attachment and open setting hardware unqualified; UNQUOTED</t>
+          <t>Installed height 8.5..7.0 mm over stroke; no free height/solid height/rate/preload or working traction assigned; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10164,12 +10164,12 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>PULL_ROLLER_ADJ</t>
+          <t>PULL_MOTOR_REF</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>puller adjustable roller dia 20 + spring-loaded carriage and guide-post envelopes</t>
+          <t>puller gearmotor reference (not selected)</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
@@ -10179,22 +10179,22 @@
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>steel + springs unselected</t>
+          <t>24 V gearmotor MPN unselected</t>
         </is>
       </c>
       <c r="F179" t="inlineStr">
         <is>
-          <t>NIP_RATING_HOLD</t>
+          <t>MOTOR_UNSELECTED</t>
         </is>
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>VP1-REFERENCE-FEED</t>
+          <t>VP1-STAGE2</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>VP1-REFERENCE-FEED</t>
+          <t>VP1-STAGE3</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
@@ -10209,7 +10209,7 @@
       </c>
       <c r="K179" t="inlineStr">
         <is>
-          <t>At modeled minimum gap 1.5 mm the 1.75 mm strand intersects both compliant roller envelopes; actual spring force and guide travel not rated; UNQUOTED</t>
+          <t>UNQUOTED; known motor floors exceed the 100000 KRW soft limit - not 0</t>
         </is>
       </c>
     </row>
@@ -10221,12 +10221,12 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>PULL_ROLLER_FIXED</t>
+          <t>PULL_NIP_STOP</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>puller drive roller dia 20 x 22</t>
+          <t>two lower and two upper positive seats limiting gap 1.5..3.0 mm</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
@@ -10236,7 +10236,7 @@
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>steel; knurl or rubber per TPU grip</t>
+          <t>steel</t>
         </is>
       </c>
       <c r="F180" t="inlineStr">
@@ -10246,12 +10246,12 @@
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-REFERENCE-FEED</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-REFERENCE-FEED</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
@@ -10266,7 +10266,7 @@
       </c>
       <c r="K180" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>Stops contact carrier only at end positions; attachment and shock loads unqualified; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10278,37 +10278,37 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>S1_BELT</t>
+          <t>PULL_ROLLER_ADJ</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>two side-loop treads over x80..219; y163.5..223.2 and 240.8..323.5</t>
+          <t>independently rotating idler dia 20 x 22 with Ø6 axle</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>polymer belt with steel-supported drums</t>
+          <t>steel</t>
         </is>
       </c>
       <c r="F181" t="inlineStr">
         <is>
-          <t>TRANSFER_UNRATED</t>
+          <t>NIP_RATING_HOLD</t>
         </is>
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>VP1-REFERENCE-FEED</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>VP1-REFERENCE-FEED</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
@@ -10323,7 +10323,7 @@
       </c>
       <c r="K181" t="inlineStr">
         <is>
-          <t>Friction and tension unrated; UNQUOTED</t>
+          <t>Idler axle clears carrier nominal Ø6.04 bearing-envelope bore; bushing and axle retention unselected; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10335,12 +10335,12 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>S1_BELT_BEARINGS</t>
+          <t>PULL_ROLLER_FIXED</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>four belt shaft support rings in the side rails</t>
+          <t>puller driven roller dia 20 x 22 with Ø8 axle</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
@@ -10350,22 +10350,22 @@
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>steel bearing seats</t>
+          <t>steel; knurl or rubber per TPU grip</t>
         </is>
       </c>
       <c r="F182" t="inlineStr">
         <is>
-          <t>TRANSFER_UNRATED</t>
+          <t>NIP_RATING_HOLD</t>
         </is>
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>VP1-STAGE2</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>VP1-STAGE3</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
@@ -10380,7 +10380,7 @@
       </c>
       <c r="K182" t="inlineStr">
         <is>
-          <t>Bearing selection and loads unqualified; UNQUOTED</t>
+          <t>Drive bearings and grip unselected; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10392,22 +10392,22 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>S1_BELT_CHAIN</t>
+          <t>S1_BELT</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>#35 chain from S1B 24T to west belt 12T</t>
+          <t>two side-loop treads over x80..219; y163.5..223.2 and 240.8..323.5</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>ANSI35 steel chain</t>
+          <t>polymer belt with steel-supported drums</t>
         </is>
       </c>
       <c r="F183" t="inlineStr">
@@ -10437,7 +10437,7 @@
       </c>
       <c r="K183" t="inlineStr">
         <is>
-          <t>Tension and strength unrated; UNQUOTED</t>
+          <t>Friction and tension unrated; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10449,12 +10449,12 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>S1_BELT_DRIVE</t>
+          <t>S1_BELT_BEARINGS</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>common waisted drive drum at x80; separate r3.8 side and r2.3 central tread seats</t>
+          <t>four belt shaft support rings in the side rails</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
@@ -10464,7 +10464,7 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>steel shaft and drums</t>
+          <t>steel bearing seats</t>
         </is>
       </c>
       <c r="F184" t="inlineStr">
@@ -10494,7 +10494,7 @@
       </c>
       <c r="K184" t="inlineStr">
         <is>
-          <t>S1B chain-driven; torque and bearing load unrated; UNQUOTED</t>
+          <t>Bearing selection and loads unqualified; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10506,12 +10506,12 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>S1_BELT_FOLLOWER</t>
+          <t>S1_BELT_CHAIN</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>12T sprocket on the west belt driver</t>
+          <t>#35 chain from S1B 24T to west belt 12T</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
@@ -10521,7 +10521,7 @@
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>ANSI35 steel sprocket</t>
+          <t>ANSI35 steel chain</t>
         </is>
       </c>
       <c r="F185" t="inlineStr">
@@ -10551,7 +10551,7 @@
       </c>
       <c r="K185" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>Tension and strength unrated; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10563,12 +10563,12 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>S1_BELT_IDLER</t>
+          <t>S1_BELT_DRIVE</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>two split side idler drums at x219 leaving the central transfer corridor open</t>
+          <t>common waisted drive drum at x80; separate r3.8 side and r2.3 central tread seats</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
@@ -10578,7 +10578,7 @@
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>steel journals and drums</t>
+          <t>steel shaft and drums</t>
         </is>
       </c>
       <c r="F186" t="inlineStr">
@@ -10608,7 +10608,7 @@
       </c>
       <c r="K186" t="inlineStr">
         <is>
-          <t>Two independent journal halves; UNQUOTED</t>
+          <t>S1B chain-driven; torque and bearing load unrated; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10620,12 +10620,12 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>S1_SWEEP_BEARINGS</t>
+          <t>S1_BELT_FOLLOWER</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>two separated sweep bearing rings in the pan rails</t>
+          <t>12T sprocket on the west belt driver</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
@@ -10635,7 +10635,7 @@
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>steel bearing seats</t>
+          <t>ANSI35 steel sprocket</t>
         </is>
       </c>
       <c r="F187" t="inlineStr">
@@ -10677,12 +10677,12 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>S1_SWEEP_GEAR_DRUM_N</t>
+          <t>S1_BELT_IDLER</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>12T gear on the north east belt idler</t>
+          <t>two split side idler drums at x219 leaving the central transfer corridor open</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
@@ -10692,7 +10692,7 @@
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>steel gear</t>
+          <t>steel journals and drums</t>
         </is>
       </c>
       <c r="F188" t="inlineStr">
@@ -10722,7 +10722,7 @@
       </c>
       <c r="K188" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>Two independent journal halves; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10734,12 +10734,12 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>S1_SWEEP_GEAR_DRUM_S</t>
+          <t>S1_SWEEP_BEARINGS</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>12T gear on the south east belt idler</t>
+          <t>two separated sweep bearing rings in the pan rails</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
@@ -10749,7 +10749,7 @@
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>steel gear</t>
+          <t>steel bearing seats</t>
         </is>
       </c>
       <c r="F189" t="inlineStr">
@@ -10791,12 +10791,12 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>S1_SWEEP_GEAR_N</t>
+          <t>S1_SWEEP_GEAR_DRUM_N</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>12T gear on the north sweep shaft</t>
+          <t>12T gear on the north east belt idler</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
@@ -10848,12 +10848,12 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>S1_SWEEP_GEAR_S</t>
+          <t>S1_SWEEP_GEAR_DRUM_S</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>12T gear on the south sweep shaft</t>
+          <t>12T gear on the south east belt idler</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
@@ -10905,12 +10905,12 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>S1_SWEEP_NORTH</t>
+          <t>S1_SWEEP_GEAR_N</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>north transverse screw x224 y235.5..359 radius 7.2 flight feeding central lane</t>
+          <t>12T gear on the north sweep shaft</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
@@ -10920,7 +10920,7 @@
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>steel shaft and flight</t>
+          <t>steel gear</t>
         </is>
       </c>
       <c r="F192" t="inlineStr">
@@ -10935,7 +10935,7 @@
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>VP1-REFERENCE-FEED</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
@@ -10950,7 +10950,7 @@
       </c>
       <c r="K192" t="inlineStr">
         <is>
-          <t>Swept flight reaches previously stranded Ø3 mm envelope near x223/z336.5; actual same-particle pickup untested; UNQUOTED</t>
+          <t>UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -10962,12 +10962,12 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>S1_SWEEP_SOUTH</t>
+          <t>S1_SWEEP_GEAR_S</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>south transverse screw x224 y127..228.5 radius 7.2 flight feeding central lane</t>
+          <t>12T gear on the south sweep shaft</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
@@ -10977,7 +10977,7 @@
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>steel shaft and flight</t>
+          <t>steel gear</t>
         </is>
       </c>
       <c r="F193" t="inlineStr">
@@ -10992,7 +10992,7 @@
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>VP1-REFERENCE-FEED</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
@@ -11007,7 +11007,7 @@
       </c>
       <c r="K193" t="inlineStr">
         <is>
-          <t>Floor relief provides swept clearance; flake capture and torque not proven; UNQUOTED</t>
+          <t>UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -11019,12 +11019,12 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>S1_TRANSFER_BEARINGS</t>
+          <t>S1_SWEEP_NORTH</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>two central idler support rings</t>
+          <t>north transverse screw x224 y235.5..359 radius 7.2 flight feeding central lane</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
@@ -11034,7 +11034,7 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>steel bearing seats</t>
+          <t>steel shaft and flight</t>
         </is>
       </c>
       <c r="F194" t="inlineStr">
@@ -11049,7 +11049,7 @@
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>VP1-STAGE5</t>
+          <t>VP1-REFERENCE-FEED</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
@@ -11064,7 +11064,7 @@
       </c>
       <c r="K194" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>Swept flight reaches previously stranded Ø3 mm envelope near x223/z336.5; actual same-particle pickup untested; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -11076,12 +11076,12 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>S1_TRANSFER_BELT</t>
+          <t>S1_SWEEP_SOUTH</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>central 17 mm tread from x80 to x270 inside two side loops</t>
+          <t>south transverse screw x224 y127..228.5 radius 7.2 flight feeding central lane</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
@@ -11091,7 +11091,7 @@
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>polymer belt</t>
+          <t>steel shaft and flight</t>
         </is>
       </c>
       <c r="F195" t="inlineStr">
@@ -11121,7 +11121,7 @@
       </c>
       <c r="K195" t="inlineStr">
         <is>
-          <t>Extended drum and ramp towards auger inlet; traction and throughflow unproven; UNQUOTED</t>
+          <t>Floor relief provides swept clearance; flake capture and torque not proven; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -11133,12 +11133,12 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>S1_TRANSFER_IDLER</t>
+          <t>S1_TRANSFER_BEARINGS</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>central east r2.05/2.45 idler at x270</t>
+          <t>two central idler support rings</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
@@ -11148,7 +11148,7 @@
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>steel drum</t>
+          <t>steel bearing seats</t>
         </is>
       </c>
       <c r="F196" t="inlineStr">
@@ -11163,7 +11163,7 @@
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>VP1-REFERENCE-FEED</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
@@ -11190,12 +11190,12 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>SERVICE-HOPPER</t>
+          <t>S1_TRANSFER_BELT</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>SWAP hollow side-inlet for reference material on FEED-BUF saddle; not in production assembly</t>
+          <t>central 17 mm tread from x80 to x270 inside two side loops</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
@@ -11205,22 +11205,22 @@
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>steel sheet 3 mm</t>
+          <t>polymer belt</t>
         </is>
       </c>
       <c r="F197" t="inlineStr">
         <is>
-          <t>SWAP_PART_NO_INTERLOCK</t>
+          <t>TRANSFER_UNRATED</t>
         </is>
       </c>
       <c r="G197" t="inlineStr">
         <is>
-          <t>VP1-STAGE6</t>
+          <t>VP1-STAGE5</t>
         </is>
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>VP1-STAGE6</t>
+          <t>VP1-REFERENCE-FEED</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
@@ -11235,7 +11235,7 @@
       </c>
       <c r="K197" t="inlineStr">
         <is>
-          <t>S2 off; saddle seal/fasteners and flow remain HOLD; no interlock credit; UNQUOTED</t>
+          <t>Extended drum and ramp towards auger inlet; traction and throughflow unproven; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -11247,12 +11247,12 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>WIND_CLUTCH_REF</t>
+          <t>S1_TRANSFER_IDLER</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>keyed collar + unselected 1 mm spring envelope + friction washer between driven shaft and loose spool flange</t>
+          <t>central east r2.05/2.45 idler at x270</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
@@ -11262,24 +11262,24 @@
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>steel collar + friction pad + spring unselected</t>
+          <t>steel drum</t>
         </is>
       </c>
       <c r="F198" t="inlineStr">
         <is>
-          <t>TORQUE_LIMIT_UNQUALIFIED</t>
+          <t>TRANSFER_UNRATED</t>
         </is>
       </c>
       <c r="G198" t="inlineStr">
         <is>
+          <t>VP1-STAGE5</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
           <t>VP1-REFERENCE-FEED</t>
         </is>
       </c>
-      <c r="H198" t="inlineStr">
-        <is>
-          <t>VP1-REFERENCE-FEED</t>
-        </is>
-      </c>
       <c r="I198" t="inlineStr">
         <is>
           <t/>
@@ -11292,7 +11292,7 @@
       </c>
       <c r="K198" t="inlineStr">
         <is>
-          <t>Smalley SSB-0087 clears dia16 shaft but its published 1.57 mm work height exceeds current 1 mm seat by 0.57 mm; solid height/force there unknown. Cannot assign the 62.3 N vendor work-point load or 70 Nmm model torque to assembly; no selected spring or quote</t>
+          <t>UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -11304,12 +11304,12 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>WIND_FLANGE_L</t>
+          <t>SERVICE-HOPPER</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>spool flange dia 200 x 3 mm</t>
+          <t>SWAP hollow side-inlet for reference material on FEED-BUF saddle; not in production assembly</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
@@ -11319,22 +11319,22 @@
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>steel plate 3 mm screening candidate</t>
+          <t>steel sheet 3 mm</t>
         </is>
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t>WINDER_STIFFNESS_SCREEN_PASS_HUB_HOLD</t>
+          <t>SWAP_PART_NO_INTERLOCK</t>
         </is>
       </c>
       <c r="G199" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-STAGE6</t>
         </is>
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-STAGE6</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
@@ -11349,7 +11349,7 @@
       </c>
       <c r="K199" t="inlineStr">
         <is>
-          <t>20 N assumed rim load; 43.33 MPa/0.194 mm beam screen only; hub bolt balance guard unqualified; unquoted</t>
+          <t>S2 off; saddle seal/fasteners and flow remain HOLD; no interlock credit; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -11361,12 +11361,12 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>WIND_FLANGE_R</t>
+          <t>WIND_CLUTCH_REF</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>spool flange dia 200 x 3 mm</t>
+          <t>keyed collar + unselected 1 mm spring envelope + friction washer between driven shaft and loose spool flange</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
@@ -11376,22 +11376,22 @@
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>steel plate 3 mm screening candidate</t>
+          <t>steel collar + friction pad + spring unselected</t>
         </is>
       </c>
       <c r="F200" t="inlineStr">
         <is>
-          <t>WINDER_STIFFNESS_SCREEN_PASS_HUB_HOLD</t>
+          <t>TORQUE_LIMIT_UNQUALIFIED</t>
         </is>
       </c>
       <c r="G200" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-REFERENCE-FEED</t>
         </is>
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-REFERENCE-FEED</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
@@ -11406,7 +11406,7 @@
       </c>
       <c r="K200" t="inlineStr">
         <is>
-          <t>20 N assumed rim load; 43.33 MPa/0.194 mm beam screen only; hub bolt balance guard unqualified; unquoted</t>
+          <t>Smalley SSB-0087 clears dia16 shaft but its published 1.57 mm work height exceeds current 1 mm seat by 0.57 mm; solid height/force there unknown. Cannot assign the 62.3 N vendor work-point load or 70 Nmm model torque to assembly; no selected spring or quote</t>
         </is>
       </c>
     </row>
@@ -11418,12 +11418,12 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>WIND_MOTOR_REF</t>
+          <t>WIND_FLANGE_L</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>spool gearmotor reference (not selected)</t>
+          <t>spool flange dia 200 x 3 mm</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
@@ -11433,12 +11433,12 @@
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>24 V gearmotor MPN unselected</t>
+          <t>steel plate 3 mm screening candidate</t>
         </is>
       </c>
       <c r="F201" t="inlineStr">
         <is>
-          <t>MOTOR_UNSELECTED</t>
+          <t>WINDER_STIFFNESS_SCREEN_PASS_HUB_HOLD</t>
         </is>
       </c>
       <c r="G201" t="inlineStr">
@@ -11463,7 +11463,7 @@
       </c>
       <c r="K201" t="inlineStr">
         <is>
-          <t>UNQUOTED; known motor floors exceed the 100000 KRW soft limit - not 0</t>
+          <t>20 N assumed rim load; 43.33 MPa/0.194 mm beam screen only; hub bolt balance guard unqualified; unquoted</t>
         </is>
       </c>
     </row>
@@ -11475,12 +11475,12 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>WIND_MOUNT</t>
+          <t>WIND_FLANGE_R</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>steel cantilever with front-profile face plate, two bearing rails and motor bed</t>
+          <t>spool flange dia 200 x 3 mm</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
@@ -11490,22 +11490,22 @@
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>steel plate/bar 4-8 mm + M5 candidate clearances</t>
+          <t>steel plate 3 mm screening candidate</t>
         </is>
       </c>
       <c r="F202" t="inlineStr">
         <is>
-          <t>WINDER_JOINT_HOLD</t>
+          <t>WINDER_STIFFNESS_SCREEN_PASS_HUB_HOLD</t>
         </is>
       </c>
       <c r="G202" t="inlineStr">
         <is>
-          <t>VP1-REFERENCE-FEED</t>
+          <t>VP1-STAGE2</t>
         </is>
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>VP1-REFERENCE-FEED</t>
+          <t>VP1-STAGE3</t>
         </is>
       </c>
       <c r="I202" t="inlineStr">
@@ -11520,7 +11520,7 @@
       </c>
       <c r="K202" t="inlineStr">
         <is>
-          <t>BRep face contact to FR-2020-400_001 and bearing/motor seats; profile slot, fastener/weld sizes, cantilever stiffness, vibration and guard HOLD; no quote - NOT 0</t>
+          <t>20 N assumed rim load; 43.33 MPa/0.194 mm beam screen only; hub bolt balance guard unqualified; unquoted</t>
         </is>
       </c>
     </row>
@@ -11532,12 +11532,12 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>WIND_SPOOL_BEARINGS</t>
+          <t>WIND_MOTOR_REF</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>spool shaft bearing blocks at BOTH shaft ends</t>
+          <t>spool gearmotor reference (not selected)</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
@@ -11547,22 +11547,22 @@
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>steel plate 5 mm + bearing seats</t>
+          <t>24 V gearmotor MPN unselected</t>
         </is>
       </c>
       <c r="F203" t="inlineStr">
         <is>
-          <t>WINDER_UNRATED</t>
+          <t>MOTOR_UNSELECTED</t>
         </is>
       </c>
       <c r="G203" t="inlineStr">
         <is>
-          <t>VP1-STAGE4</t>
+          <t>VP1-STAGE2</t>
         </is>
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>VP1-STAGE4</t>
+          <t>VP1-STAGE3</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
@@ -11577,7 +11577,7 @@
       </c>
       <c r="K203" t="inlineStr">
         <is>
-          <t>VP1 Stage 4 grip redesign: shaft supported at both ends - UNQUOTED</t>
+          <t>UNQUOTED; known motor floors exceed the 100000 KRW soft limit - not 0</t>
         </is>
       </c>
     </row>
@@ -11589,12 +11589,12 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>WIND_SPOOL_DRUM</t>
+          <t>WIND_MOUNT</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>spool dia 70 x 58 steel tube with 2 mm wall and two 3 mm internal annular webs; weld to steel flanges before winding</t>
+          <t>steel cantilever with front-profile face plate, two bearing rails and motor bed</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
@@ -11604,12 +11604,12 @@
       </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t>steel tube + steel webs candidate</t>
+          <t>steel plate/bar 4-8 mm + M5 candidate clearances</t>
         </is>
       </c>
       <c r="F204" t="inlineStr">
         <is>
-          <t>WINDER_UNRATED</t>
+          <t>WINDER_JOINT_HOLD</t>
         </is>
       </c>
       <c r="G204" t="inlineStr">
@@ -11634,7 +11634,7 @@
       </c>
       <c r="K204" t="inlineStr">
         <is>
-          <t>Web-to-tube and flange seams and balance unqualified; loose Ø17 web bores clear Ø16 shaft; friction clutch drives flange; UNQUOTED</t>
+          <t>BRep face contact to FR-2020-400_001 and bearing/motor seats; profile slot, fastener/weld sizes, cantilever stiffness, vibration and guard HOLD; no quote - NOT 0</t>
         </is>
       </c>
     </row>
@@ -11646,12 +11646,12 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>WIND_SPOOL_RETENTION</t>
+          <t>WIND_SPOOL_BEARINGS</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>two ES-16 nominal external-ring envelopes plus loose-flange OD30/ID16.2 thrust washer</t>
+          <t>spool shaft bearing blocks at BOTH shaft ends</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
@@ -11661,22 +11661,22 @@
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t>ring spring steel candidate + steel washer</t>
+          <t>steel plate 5 mm + bearing seats</t>
         </is>
       </c>
       <c r="F205" t="inlineStr">
         <is>
-          <t>AXIAL_FLOAT_PRELOAD_HOLD</t>
+          <t>WINDER_UNRATED</t>
         </is>
       </c>
       <c r="G205" t="inlineStr">
         <is>
-          <t>VP1-REFERENCE-FEED</t>
+          <t>VP1-STAGE4</t>
         </is>
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>VP1-REFERENCE-FEED</t>
+          <t>VP1-STAGE4</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
@@ -11691,7 +11691,7 @@
       </c>
       <c r="K205" t="inlineStr">
         <is>
-          <t>Smalley ES-16 two-turn supplier detail unmodeled; 15.02 mm groove dia and 1.00 +0.08 mm width; nominal 0.89 +/-0.05 mm ring thickness and 1.40 +0.08/-0.13 radial wall. Groove clearance 0.06..0.24 mm per ring (two up to 0.48 mm) excludes rated clamp; maker groove yield 3820 N assumes 45000 psi shaft yield/SF2 and is NOT a PPR rating. MPN dimension reference only; installed fit/thrust/fatigue/landed price HOLD; unquoted NOT zero</t>
+          <t>VP1 Stage 4 grip redesign: shaft supported at both ends - UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -11703,12 +11703,12 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>WIND_SPOOL_SHAFT</t>
+          <t>WIND_SPOOL_DRUM</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>spool shaft dia 16 x 98 with keyed clutch collar seat and two ES-16 dimensional-candidate 1 mm grooves</t>
+          <t>spool dia 70 x 58 steel tube with 2 mm wall and two 3 mm internal annular webs; weld to steel flanges before winding</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
@@ -11718,7 +11718,7 @@
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t>C45 candidate</t>
+          <t>steel tube + steel webs candidate</t>
         </is>
       </c>
       <c r="F206" t="inlineStr">
@@ -11748,7 +11748,7 @@
       </c>
       <c r="K206" t="inlineStr">
         <is>
-          <t>Groove nominal diameter 15.02 mm at y96..97 and y168..169; supplier Dg tolerance +/-0.075 mm; shaft fatigue/actual ring procurement HOLD; UNQUOTED</t>
+          <t>Web-to-tube and flange seams and balance unqualified; loose Ø17 web bores clear Ø16 shaft; friction clutch drives flange; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -11760,12 +11760,12 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>WIND_TENSIONER</t>
+          <t>WIND_SPOOL_RETENTION</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>filament path-buffer post + wrap arm</t>
+          <t>two ES-16 nominal external-ring envelopes plus loose-flange OD30/ID16.2 thrust washer</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
@@ -11775,22 +11775,22 @@
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t>steel</t>
+          <t>ring spring steel candidate + steel washer</t>
         </is>
       </c>
       <c r="F207" t="inlineStr">
         <is>
-          <t>TENSION_UNRATED</t>
+          <t>AXIAL_FLOAT_PRELOAD_HOLD</t>
         </is>
       </c>
       <c r="G207" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-REFERENCE-FEED</t>
         </is>
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-REFERENCE-FEED</t>
         </is>
       </c>
       <c r="I207" t="inlineStr">
@@ -11805,7 +11805,7 @@
       </c>
       <c r="K207" t="inlineStr">
         <is>
-          <t>Not a calibrated torque limiter; UNQUOTED</t>
+          <t>Smalley ES-16 two-turn supplier detail unmodeled; 15.02 mm groove dia and 1.00 +0.08 mm width; nominal 0.89 +/-0.05 mm ring thickness and 1.40 +0.08/-0.13 radial wall. Groove clearance 0.06..0.24 mm per ring (two up to 0.48 mm) excludes rated clamp; maker groove yield 3820 N assumes 45000 psi shaft yield/SF2 and is NOT a PPR rating. MPN dimension reference only; installed fit/thrust/fatigue/landed price HOLD; unquoted NOT zero</t>
         </is>
       </c>
     </row>
@@ -11817,12 +11817,12 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>WIND_TRAVERSE_RIDER</t>
+          <t>WIND_SPOOL_SHAFT</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>traverse rider block + guide eyelet</t>
+          <t>spool shaft dia 16 x 98 with keyed clutch collar seat and two ES-16 dimensional-candidate 1 mm grooves</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
@@ -11832,7 +11832,7 @@
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t>steel + printed guide</t>
+          <t>C45 candidate</t>
         </is>
       </c>
       <c r="F208" t="inlineStr">
@@ -11842,12 +11842,12 @@
       </c>
       <c r="G208" t="inlineStr">
         <is>
-          <t>VP1-STAGE2</t>
+          <t>VP1-REFERENCE-FEED</t>
         </is>
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>VP1-STAGE3</t>
+          <t>VP1-REFERENCE-FEED</t>
         </is>
       </c>
       <c r="I208" t="inlineStr">
@@ -11862,7 +11862,7 @@
       </c>
       <c r="K208" t="inlineStr">
         <is>
-          <t>UNQUOTED</t>
+          <t>Groove nominal diameter 15.02 mm at y96..97 and y168..169; supplier Dg tolerance +/-0.075 mm; shaft fatigue/actual ring procurement HOLD; UNQUOTED</t>
         </is>
       </c>
     </row>
@@ -11874,50 +11874,164 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
+          <t>WIND_TENSIONER</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>filament path-buffer post + wrap arm</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>steel</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>TENSION_UNRATED</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>VP1-STAGE2</t>
+        </is>
+      </c>
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>VP1-STAGE3</t>
+        </is>
+      </c>
+      <c r="I209" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J209" t="inlineStr">
+        <is>
+          <t>UNQUOTED_NOT_ZERO</t>
+        </is>
+      </c>
+      <c r="K209" t="inlineStr">
+        <is>
+          <t>Not a calibrated torque limiter; UNQUOTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>vp1_stage1_3</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>WIND_TRAVERSE_RIDER</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>traverse rider block + guide eyelet</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>steel + printed guide</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>WINDER_UNRATED</t>
+        </is>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>VP1-STAGE2</t>
+        </is>
+      </c>
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>VP1-STAGE3</t>
+        </is>
+      </c>
+      <c r="I210" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J210" t="inlineStr">
+        <is>
+          <t>UNQUOTED_NOT_ZERO</t>
+        </is>
+      </c>
+      <c r="K210" t="inlineStr">
+        <is>
+          <t>UNQUOTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>vp1_stage1_3</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
           <t>WIND_TRAVERSE_SCREW</t>
         </is>
       </c>
-      <c r="C209" t="inlineStr">
+      <c r="C211" t="inlineStr">
         <is>
           <t>traverse lead screw dia 8 x 80</t>
         </is>
       </c>
-      <c r="D209" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E209" t="inlineStr">
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
         <is>
           <t>steel rod</t>
         </is>
       </c>
-      <c r="F209" t="inlineStr">
+      <c r="F211" t="inlineStr">
         <is>
           <t>WINDER_UNRATED</t>
         </is>
       </c>
-      <c r="G209" t="inlineStr">
+      <c r="G211" t="inlineStr">
         <is>
           <t>VP1-STAGE2</t>
         </is>
       </c>
-      <c r="H209" t="inlineStr">
+      <c r="H211" t="inlineStr">
         <is>
           <t>VP1-STAGE3</t>
         </is>
       </c>
-      <c r="I209" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J209" t="inlineStr">
+      <c r="I211" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J211" t="inlineStr">
         <is>
           <t>UNQUOTED_NOT_ZERO</t>
         </is>
       </c>
-      <c r="K209" t="inlineStr">
+      <c r="K211" t="inlineStr">
         <is>
           <t>UNQUOTED</t>
         </is>

</xml_diff>

<commit_message>
Correct active BOM for no owned inventory and unpriced procurement
</commit_message>
<xml_diff>
--- a/c2.1/bom/system_bom.xlsx
+++ b/c2.1/bom/system_bom.xlsx
@@ -4640,7 +4640,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Owned 24V 800W PSU</t>
+          <t>24V 800W PSU</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -4655,7 +4655,7 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>OWNED_MOUNTING_PATTERN_UNMEASURED</t>
+          <t>PROCUREMENT_HOLD</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -4665,22 +4665,22 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>C1_INTERFACE_BASELINE</t>
+          <t>C1_GEOMETRY_REFERENCE_USER_REPORTS_NO_STOCK</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>0</t>
+          <t/>
         </is>
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>OWNED_NO_NEW_PURCHASE</t>
+          <t>UNQUOTED_NOT_ZERO</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
         <is>
-          <t>No guessed mounting holes. 120x240x65 user measurement; model contains true body only.</t>
+          <t>No guessed mounting holes. 120x240x65 historical reference envelope; model contains true body only. Historical handover assumed stock; current user reports none. Obtain landed quote; not zero.</t>
         </is>
       </c>
     </row>
@@ -5562,12 +5562,12 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Al extrusion - existing</t>
+          <t>Al extrusion candidate</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>OWNED_SLOT_PATTERN_TO_MEASURE</t>
+          <t>PROCUREMENT_HOLD</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
@@ -5577,22 +5577,22 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>C1_INTERFACE_BASELINE</t>
+          <t>C1_GEOMETRY_REFERENCE_USER_REPORTS_NO_STOCK</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>0</t>
+          <t/>
         </is>
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>OWNED_NO_NEW_PURCHASE</t>
+          <t>UNQUOTED_NOT_ZERO</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
         <is>
-          <t>Nominal section only. Confirm slot series before buying brackets; 3 mm saw kerf.</t>
+          <t>Nominal section only. Confirm slot series before buying brackets; 3 mm saw kerf. Historical handover assumed stock; current user reports none. Obtain landed quote; not zero.</t>
         </is>
       </c>
     </row>
@@ -5619,12 +5619,12 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Al extrusion - existing</t>
+          <t>Al extrusion candidate</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>OWNED_SLOT_PATTERN_TO_MEASURE</t>
+          <t>PROCUREMENT_HOLD</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
@@ -5634,22 +5634,22 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>C1_INTERFACE_BASELINE</t>
+          <t>C1_GEOMETRY_REFERENCE_USER_REPORTS_NO_STOCK</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>0</t>
+          <t/>
         </is>
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>OWNED_NO_NEW_PURCHASE</t>
+          <t>UNQUOTED_NOT_ZERO</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
         <is>
-          <t>Nominal section only. Confirm slot series before buying brackets; 3 mm saw kerf.</t>
+          <t>Nominal section only. Confirm slot series before buying brackets; 3 mm saw kerf. Historical handover assumed stock; current user reports none. Obtain landed quote; not zero.</t>
         </is>
       </c>
     </row>
@@ -5676,12 +5676,12 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Al extrusion - existing</t>
+          <t>Al extrusion candidate</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>OWNED_SLOT_PATTERN_TO_MEASURE</t>
+          <t>PROCUREMENT_HOLD</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
@@ -5691,22 +5691,22 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>C1_INTERFACE_BASELINE</t>
+          <t>C1_GEOMETRY_REFERENCE_USER_REPORTS_NO_STOCK</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>0</t>
+          <t/>
         </is>
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>OWNED_NO_NEW_PURCHASE</t>
+          <t>UNQUOTED_NOT_ZERO</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
         <is>
-          <t>Nominal section only. Confirm slot series before buying brackets; 3 mm saw kerf.</t>
+          <t>Nominal section only. Confirm slot series before buying brackets; 3 mm saw kerf. Historical handover assumed stock; current user reports none. Obtain landed quote; not zero.</t>
         </is>
       </c>
     </row>
@@ -5733,12 +5733,12 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Al extrusion - existing</t>
+          <t>Al extrusion candidate</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>OWNED_SLOT_PATTERN_TO_MEASURE</t>
+          <t>PROCUREMENT_HOLD</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
@@ -5748,22 +5748,22 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>C1_INTERFACE_BASELINE</t>
+          <t>C1_GEOMETRY_REFERENCE_USER_REPORTS_NO_STOCK</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>0</t>
+          <t/>
         </is>
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>OWNED_NO_NEW_PURCHASE</t>
+          <t>UNQUOTED_NOT_ZERO</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
         <is>
-          <t>Nominal section only. Confirm slot series before buying brackets; 3 mm saw kerf.</t>
+          <t>Nominal section only. Confirm slot series before buying brackets; 3 mm saw kerf. Historical handover assumed stock; current user reports none. Obtain landed quote; not zero.</t>
         </is>
       </c>
     </row>
@@ -5790,12 +5790,12 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Al extrusion - existing</t>
+          <t>Al extrusion candidate</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>OWNED_SLOT_PATTERN_TO_MEASURE</t>
+          <t>PROCUREMENT_HOLD</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
@@ -5805,22 +5805,22 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>C1_INTERFACE_BASELINE</t>
+          <t>C1_GEOMETRY_REFERENCE_USER_REPORTS_NO_STOCK</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>0</t>
+          <t/>
         </is>
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>OWNED_NO_NEW_PURCHASE</t>
+          <t>UNQUOTED_NOT_ZERO</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
         <is>
-          <t>Nominal section only. Confirm slot series before buying brackets; 3 mm saw kerf.</t>
+          <t>Nominal section only. Confirm slot series before buying brackets; 3 mm saw kerf. Historical handover assumed stock; current user reports none. Obtain landed quote; not zero.</t>
         </is>
       </c>
     </row>
@@ -5847,12 +5847,12 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Al extrusion - existing</t>
+          <t>Al extrusion candidate</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>OWNED_SLOT_PATTERN_TO_MEASURE</t>
+          <t>PROCUREMENT_HOLD</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
@@ -5862,22 +5862,22 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>C1_INTERFACE_BASELINE</t>
+          <t>C1_GEOMETRY_REFERENCE_USER_REPORTS_NO_STOCK</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>0</t>
+          <t/>
         </is>
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>OWNED_NO_NEW_PURCHASE</t>
+          <t>UNQUOTED_NOT_ZERO</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
         <is>
-          <t>Nominal section only. Confirm slot series before buying brackets; 3 mm saw kerf.</t>
+          <t>Nominal section only. Confirm slot series before buying brackets; 3 mm saw kerf. Historical handover assumed stock; current user reports none. Obtain landed quote; not zero.</t>
         </is>
       </c>
     </row>
@@ -5904,12 +5904,12 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Al extrusion - existing</t>
+          <t>Al extrusion candidate</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>OWNED_SLOT_PATTERN_TO_MEASURE</t>
+          <t>PROCUREMENT_HOLD</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
@@ -5919,22 +5919,22 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>C1_INTERFACE_BASELINE</t>
+          <t>C1_GEOMETRY_REFERENCE_USER_REPORTS_NO_STOCK</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>0</t>
+          <t/>
         </is>
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>OWNED_NO_NEW_PURCHASE</t>
+          <t>UNQUOTED_NOT_ZERO</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
         <is>
-          <t>Nominal section only. Confirm slot series before buying brackets; 3 mm saw kerf.</t>
+          <t>Nominal section only. Confirm slot series before buying brackets; 3 mm saw kerf. Historical handover assumed stock; current user reports none. Obtain landed quote; not zero.</t>
         </is>
       </c>
     </row>
@@ -6707,7 +6707,7 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>OWNED</t>
+          <t>PROCUREMENT_HOLD</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
@@ -6717,22 +6717,22 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>C1_INTERFACE_BASELINE</t>
+          <t>C1_GEOMETRY_REFERENCE_USER_REPORTS_NO_STOCK</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>0</t>
+          <t/>
         </is>
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>OWNED_NO_NEW_PURCHASE</t>
+          <t>UNQUOTED_NOT_ZERO</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
         <is>
-          <t>Reference power allocator is NOT deployable heater firmware.</t>
+          <t>Reference power allocator is NOT deployable heater firmware. Historical handover assumed stock; current user reports none. Obtain landed quote; not zero.</t>
         </is>
       </c>
     </row>
@@ -6806,7 +6806,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Existing BTS7960 modules</t>
+          <t>BTS7960 modules</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -6821,7 +6821,7 @@
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>OWNED_UNQUALIFIED</t>
+          <t>PROCUREMENT_HOLD</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
@@ -6831,22 +6831,22 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>C1_INTERFACE_BASELINE</t>
+          <t>C1_GEOMETRY_REFERENCE_USER_REPORTS_NO_STOCK</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>0</t>
+          <t/>
         </is>
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>OWNED_NO_NEW_PURCHASE</t>
+          <t>UNQUOTED_NOT_ZERO</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>Do not assume advertised43A continuous.</t>
+          <t>Do not assume advertised43A continuous. Historical handover assumed stock; current user reports none. Obtain landed quote; not zero.</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Existing E-stop</t>
+          <t>E-stop</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -7391,7 +7391,7 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>OWNED_RATING_VERIFY</t>
+          <t>PROCUREMENT_HOLD</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
@@ -7401,22 +7401,22 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>C1_INTERFACE_BASELINE</t>
+          <t>C1_GEOMETRY_REFERENCE_USER_REPORTS_NO_STOCK</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>0</t>
+          <t/>
         </is>
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>OWNED_NO_NEW_PURCHASE</t>
+          <t>UNQUOTED_NOT_ZERO</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>Independent hard cut with contactor; contact configuration verify.</t>
+          <t>Independent hard cut with contactor; contact configuration verify. Historical handover assumed stock; current user reports none. Obtain landed quote; not zero.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Account for Chiron donor PSU and stop-button stock
Treat the reported PSU and 2NC button as unqualified owned assets, not required purchases. Screen Chiron profile reuse against the current cut plan without inventing stock lengths or electrical ratings, and preserve unquoted whole-system cost and physical HOLD.
</commit_message>
<xml_diff>
--- a/c2.1/bom/system_bom.xlsx
+++ b/c2.1/bom/system_bom.xlsx
@@ -4640,7 +4640,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>24V 800W PSU</t>
+          <t>User-reported Anycubic Chiron donor PSU, 24V 800W (label unverified)</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -4650,12 +4650,12 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Purchased</t>
+          <t>Donor PSU (unverified)</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>PROCUREMENT_HOLD</t>
+          <t>OWNED_REPORTED_RATING_HOLD</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -4665,7 +4665,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>C1_GEOMETRY_REFERENCE_USER_REPORTS_NO_STOCK</t>
+          <t>USER_REPORTED_CHIRON_PSU_LABEL_UNVERIFIED</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -4675,12 +4675,12 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>UNQUOTED_NOT_ZERO</t>
+          <t>OWNED_DONOR_PSU_NO_NEW_PURCHASE_UNQUALIFIED</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
         <is>
-          <t>No guessed mounting holes. 120x240x65 historical reference envelope; model contains true body only. Historical handover assumed stock; current user reports none. Obtain landed quote; not zero.</t>
+          <t>No guessed mounting holes. 120x240x65 historical modeled envelope; model contains true body only. Chiron donor PSU reported owned; 24V 800W is historical user report and 240x120x65 mm is a modeled envelope, not a measured nameplate or fit. Check label, dimensions, condition, protection and 500W staged duty; no replacement PSU purchase assumed.</t>
         </is>
       </c>
     </row>
@@ -5567,7 +5567,7 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>PROCUREMENT_HOLD</t>
+          <t>DONOR_CUT_FIT_OR_PROCUREMENT_HOLD</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
@@ -5577,7 +5577,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>C1_GEOMETRY_REFERENCE_USER_REPORTS_NO_STOCK</t>
+          <t>C1_GEOMETRY_REFERENCE_CURRENT_STOCK_UNCONFIRMED</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -5592,7 +5592,7 @@
       </c>
       <c r="K98" t="inlineStr">
         <is>
-          <t>Nominal section only. Confirm slot series before buying brackets; 3 mm saw kerf. Historical handover assumed stock; current user reports none. Obtain landed quote; not zero.</t>
+          <t>Nominal section only. Confirm slot series before buying brackets; 3 mm saw kerf. Historical handover is not current qualified stock; confirm donor part identity/interface or obtain landed quote.</t>
         </is>
       </c>
     </row>
@@ -5624,7 +5624,7 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>PROCUREMENT_HOLD</t>
+          <t>DONOR_CUT_FIT_OR_PROCUREMENT_HOLD</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
@@ -5634,7 +5634,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>C1_GEOMETRY_REFERENCE_USER_REPORTS_NO_STOCK</t>
+          <t>C1_GEOMETRY_REFERENCE_CURRENT_STOCK_UNCONFIRMED</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -5649,7 +5649,7 @@
       </c>
       <c r="K99" t="inlineStr">
         <is>
-          <t>Nominal section only. Confirm slot series before buying brackets; 3 mm saw kerf. Historical handover assumed stock; current user reports none. Obtain landed quote; not zero.</t>
+          <t>Nominal section only. Confirm slot series before buying brackets; 3 mm saw kerf. Historical handover is not current qualified stock; confirm donor part identity/interface or obtain landed quote.</t>
         </is>
       </c>
     </row>
@@ -5681,7 +5681,7 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>PROCUREMENT_HOLD</t>
+          <t>DONOR_CUT_FIT_OR_PROCUREMENT_HOLD</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
@@ -5691,7 +5691,7 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>C1_GEOMETRY_REFERENCE_USER_REPORTS_NO_STOCK</t>
+          <t>C1_GEOMETRY_REFERENCE_CURRENT_STOCK_UNCONFIRMED</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -5706,7 +5706,7 @@
       </c>
       <c r="K100" t="inlineStr">
         <is>
-          <t>Nominal section only. Confirm slot series before buying brackets; 3 mm saw kerf. Historical handover assumed stock; current user reports none. Obtain landed quote; not zero.</t>
+          <t>Nominal section only. Confirm slot series before buying brackets; 3 mm saw kerf. Historical handover is not current qualified stock; confirm donor part identity/interface or obtain landed quote.</t>
         </is>
       </c>
     </row>
@@ -5738,7 +5738,7 @@
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>PROCUREMENT_HOLD</t>
+          <t>DONOR_CUT_FIT_OR_PROCUREMENT_HOLD</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
@@ -5748,7 +5748,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>C1_GEOMETRY_REFERENCE_USER_REPORTS_NO_STOCK</t>
+          <t>C1_GEOMETRY_REFERENCE_CURRENT_STOCK_UNCONFIRMED</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -5763,7 +5763,7 @@
       </c>
       <c r="K101" t="inlineStr">
         <is>
-          <t>Nominal section only. Confirm slot series before buying brackets; 3 mm saw kerf. Historical handover assumed stock; current user reports none. Obtain landed quote; not zero.</t>
+          <t>Nominal section only. Confirm slot series before buying brackets; 3 mm saw kerf. Historical handover is not current qualified stock; confirm donor part identity/interface or obtain landed quote.</t>
         </is>
       </c>
     </row>
@@ -5795,7 +5795,7 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>PROCUREMENT_HOLD</t>
+          <t>DONOR_CUT_FIT_OR_PROCUREMENT_HOLD</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
@@ -5805,7 +5805,7 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>C1_GEOMETRY_REFERENCE_USER_REPORTS_NO_STOCK</t>
+          <t>C1_GEOMETRY_REFERENCE_CURRENT_STOCK_UNCONFIRMED</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -5820,7 +5820,7 @@
       </c>
       <c r="K102" t="inlineStr">
         <is>
-          <t>Nominal section only. Confirm slot series before buying brackets; 3 mm saw kerf. Historical handover assumed stock; current user reports none. Obtain landed quote; not zero.</t>
+          <t>Nominal section only. Confirm slot series before buying brackets; 3 mm saw kerf. Historical handover is not current qualified stock; confirm donor part identity/interface or obtain landed quote.</t>
         </is>
       </c>
     </row>
@@ -5852,7 +5852,7 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>PROCUREMENT_HOLD</t>
+          <t>DONOR_CUT_FIT_OR_PROCUREMENT_HOLD</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
@@ -5862,7 +5862,7 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>C1_GEOMETRY_REFERENCE_USER_REPORTS_NO_STOCK</t>
+          <t>C1_GEOMETRY_REFERENCE_CURRENT_STOCK_UNCONFIRMED</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -5877,7 +5877,7 @@
       </c>
       <c r="K103" t="inlineStr">
         <is>
-          <t>Nominal section only. Confirm slot series before buying brackets; 3 mm saw kerf. Historical handover assumed stock; current user reports none. Obtain landed quote; not zero.</t>
+          <t>Nominal section only. Confirm slot series before buying brackets; 3 mm saw kerf. Historical handover is not current qualified stock; confirm donor part identity/interface or obtain landed quote.</t>
         </is>
       </c>
     </row>
@@ -5909,7 +5909,7 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>PROCUREMENT_HOLD</t>
+          <t>DONOR_CUT_FIT_OR_PROCUREMENT_HOLD</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
@@ -5919,7 +5919,7 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>C1_GEOMETRY_REFERENCE_USER_REPORTS_NO_STOCK</t>
+          <t>C1_GEOMETRY_REFERENCE_CURRENT_STOCK_UNCONFIRMED</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -5934,7 +5934,7 @@
       </c>
       <c r="K104" t="inlineStr">
         <is>
-          <t>Nominal section only. Confirm slot series before buying brackets; 3 mm saw kerf. Historical handover assumed stock; current user reports none. Obtain landed quote; not zero.</t>
+          <t>Nominal section only. Confirm slot series before buying brackets; 3 mm saw kerf. Historical handover is not current qualified stock; confirm donor part identity/interface or obtain landed quote.</t>
         </is>
       </c>
     </row>
@@ -6717,7 +6717,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>C1_GEOMETRY_REFERENCE_USER_REPORTS_NO_STOCK</t>
+          <t>C1_GEOMETRY_REFERENCE_CURRENT_STOCK_UNCONFIRMED</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -6732,7 +6732,7 @@
       </c>
       <c r="K118" t="inlineStr">
         <is>
-          <t>Reference power allocator is NOT deployable heater firmware. Historical handover assumed stock; current user reports none. Obtain landed quote; not zero.</t>
+          <t>Reference power allocator is NOT deployable heater firmware. Historical handover is not current qualified stock; confirm donor part identity/interface or obtain landed quote.</t>
         </is>
       </c>
     </row>
@@ -6831,7 +6831,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>C1_GEOMETRY_REFERENCE_USER_REPORTS_NO_STOCK</t>
+          <t>C1_GEOMETRY_REFERENCE_CURRENT_STOCK_UNCONFIRMED</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -6846,7 +6846,7 @@
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>Do not assume advertised43A continuous. Historical handover assumed stock; current user reports none. Obtain landed quote; not zero.</t>
+          <t>Do not assume advertised43A continuous. Historical handover is not current qualified stock; confirm donor part identity/interface or obtain landed quote.</t>
         </is>
       </c>
     </row>
@@ -6903,7 +6903,7 @@
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>Configurable current limit; board21A is not terminal43A. Existing BTS7960 requires qualification.</t>
+          <t>Configurable current limit; board21A is not terminal43A. BTS7960 candidate requires qualification.</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>E-stop</t>
+          <t>User-reported 2NC emergency stop button</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -7391,7 +7391,7 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>PROCUREMENT_HOLD</t>
+          <t>OWNED_REPORTED_RATING_HOLD</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
@@ -7401,7 +7401,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>C1_GEOMETRY_REFERENCE_USER_REPORTS_NO_STOCK</t>
+          <t>USER_REPORTED_2NC_BUTTON_MODEL_UNVERIFIED</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -7411,12 +7411,12 @@
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>UNQUOTED_NOT_ZERO</t>
+          <t>OWNED_BUTTON_NO_NEW_PURCHASE_UNQUALIFIED</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>Independent hard cut with contactor; contact configuration verify. Historical handover assumed stock; current user reports none. Obtain landed quote; not zero.</t>
+          <t>Independent hard cut with contactor; contact configuration verify. One 2NC button reported owned; model, contact rating, positive opening, wiring and hard-cut contactor unverified. No additional button purchase assumed; full safety circuit still unquoted.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record reported donor dimensions and quote reference pellets
Keep reported PSU and stop-button dimensions distinct from verified mounts and safety ratings. Compare reference PLA pellet public quotes without ordering or assigning a system landed cost.
</commit_message>
<xml_diff>
--- a/c2.1/bom/system_bom.xlsx
+++ b/c2.1/bom/system_bom.xlsx
@@ -4680,7 +4680,7 @@
       </c>
       <c r="K82" t="inlineStr">
         <is>
-          <t>No guessed mounting holes. 120x240x65 historical modeled envelope; model contains true body only. Chiron donor PSU reported owned; 24V 800W is historical user report and 240x120x65 mm is a modeled envelope, not a measured nameplate or fit. Check label, dimensions, condition, protection and 500W staged duty; no replacement PSU purchase assumed.</t>
+          <t>No guessed mounting holes. 240x120x65 mm user-reported exterior; CAD box is an exterior envelope only. Chiron donor PSU reported owned; 24V 800W is user-reported. Label, mounting pattern, condition, protection and 500W staged duty remain unverified; no replacement PSU purchase assumed.</t>
         </is>
       </c>
     </row>
@@ -7416,7 +7416,7 @@
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>Independent hard cut with contactor; contact configuration verify. One 2NC button reported owned; model, contact rating, positive opening, wiring and hard-cut contactor unverified. No additional button purchase assumed; full safety circuit still unquoted.</t>
+          <t>Independent hard cut with contactor; contact configuration verify. One 2NC button reported owned, with a reported 35x35 mm size (which face, body depth and panel cutout unidentified); model, contact rating, positive opening, wiring and hard-cut contactor unverified. No additional button purchase assumed; full safety circuit unquoted.</t>
         </is>
       </c>
     </row>

</xml_diff>